<commit_message>
[FIX] Keep target in model name
</commit_message>
<xml_diff>
--- a/results/metrics_modelling3.xlsx
+++ b/results/metrics_modelling3.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Logit_test</t>
+          <t>Logit_splashing_test</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -613,12 +613,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>0.006796121597290039, 0.005709648132324219, 0.009855985641479492, 0.0030870437622070312, 0.008744001388549805</t>
+          <t>0.0074918270111083984, 0.0032570362091064453, 0.003041982650756836, 0.0076830387115478516, 0.004441261291503906</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>0.0317230224609375, 0.004549264907836914, 0.010825872421264648, 0.0075531005859375, 0.007467031478881836</t>
+          <t>0.01373600959777832, 0.004681110382080078, 0.006099224090576172, 0.009279966354370117, 0.004483699798583984</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">

</xml_diff>

<commit_message>
[ADD] Test of XGB, CatBoost, KNN, SVC
</commit_message>
<xml_diff>
--- a/results/metrics_modelling3.xlsx
+++ b/results/metrics_modelling3.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z2"/>
+  <dimension ref="A1:Z9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -669,6 +669,800 @@
       <c r="Z2" t="inlineStr">
         <is>
           <t>0.8862599206349207, 0.8992807539682539, 0.8969388757861635, 0.8968406053459119, 0.9042354559748428</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>LogisticRegression_splashing_test</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>{'estimator': LogisticRegression(), 'source_features': ['init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'], 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': None, 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Re', 'sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>0.8133333333333334</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.8035714285714286</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.9375</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.8653846153846154</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.8912037037037037</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.8148148148148148</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.8407960199004975</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.8802083333333334</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.8600508905852416</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0.9132688492063492</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>0.018549442291259766, 0.0, 0.01028299331665039, 0.007892370223999023, 0.0</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>0.004538774490356445, 0.013784646987915039, 0.008110523223876953, 0.008096694946289062, 0.02117133140563965</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>0.84, 0.8133333333333334, 0.7837837837837838, 0.7972972972972973, 0.7702702702702703</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>0.8080808080808081, 0.8181818181818182, 0.8154362416107382, 0.8389261744966443, 0.8221476510067114</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>0.8461538461538461, 0.8269230769230769, 0.8636363636363636, 0.8235294117647058, 0.7818181818181819</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>0.8292682926829268, 0.8415841584158416, 0.8309178743961353, 0.86, 0.8390243902439024</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>0.9166666666666666, 0.8958333333333334, 0.7916666666666666, 0.875, 0.8958333333333334</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>0.8854166666666666, 0.8854166666666666, 0.8958333333333334, 0.8958333333333334, 0.8958333333333334</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>0.8799999999999999, 0.86, 0.8260869565217391, 0.8484848484848485, 0.8349514563106797</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>0.8564231738035264, 0.8629441624365483, 0.862155388471178, 0.8775510204081632, 0.8664987405541561</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>0.9436728395061728, 0.8935185185185186, 0.889423076923077, 0.9046474358974359, 0.8509615384615384</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>0.8981150793650794, 0.9085565476190476, 0.9093700864779874, 0.9061271619496855, 0.9170106132075472</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>KNeighborsClassifier_splashing_test</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>{'estimator': KNeighborsClassifier(), 'source_features': ['init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'], 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': None, 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Re', 'sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>0.8133333333333334</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.8269230769230769</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.8958333333333334</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.880787037037037</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.9158249158249159</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.9282051282051282</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.9427083333333334</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.9354005167958657</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0.9661954365079365</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>0.013483047485351562, 0.008872747421264648, 0.0, 0.00803828239440918, 0.015599966049194336</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>0.0032334327697753906, 0.008018970489501953, 0.02013373374938965, 0.00797891616821289, 0.0</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>0.9333333333333333, 0.7733333333333333, 0.8108108108108109, 0.8648648648648649, 0.7297297297297297</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>0.898989898989899, 0.8888888888888888, 0.889261744966443, 0.8993288590604027, 0.8859060402684564</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>0.9387755102040817, 0.8444444444444444, 0.8541666666666666, 0.9318181818181818, 0.7916666666666666</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>0.9263157894736842, 0.9206349206349206, 0.9035532994923858, 0.9263157894736842, 0.9157894736842105</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>0.9583333333333334, 0.7916666666666666, 0.8541666666666666, 0.8541666666666666, 0.7916666666666666</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>0.9166666666666666, 0.90625, 0.9270833333333334, 0.9166666666666666, 0.90625</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>0.9484536082474228, 0.8172043010752689, 0.8541666666666666, 0.8913043478260869, 0.7916666666666666</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>0.9214659685863874, 0.9133858267716536, 0.9151670951156814, 0.9214659685863874, 0.9109947643979057</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>0.970679012345679, 0.8873456790123456, 0.923477564102564, 0.938301282051282, 0.8257211538461537</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>0.9578869047619047, 0.9656250000000001, 0.9632468553459119, 0.9583824685534591, 0.9681603773584906</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>SVC_splashing_test</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>{'estimator': SVC(probability=True), 'source_features': ['init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'], 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': None, 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Re', 'sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.8214285714285714</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.9583333333333334</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.8846153846153847</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.8958333333333334</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.8855218855218855</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.9030612244897959</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.921875</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.9123711340206186</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.9497271825396826</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>0.02239513397216797, 0.014011144638061523, 0.011605024337768555, 0.008462667465209961, 0.015657901763916016</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>0.014072656631469727, 0.008000850677490234, 0.012187957763671875, 0.013071537017822266, 0.0</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>0.88, 0.7733333333333333, 0.8513513513513513, 0.8648648648648649, 0.8378378378378378</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>0.8754208754208754, 0.8821548821548821, 0.8791946308724832, 0.8590604026845637, 0.8993288590604027</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>0.8545454545454545, 0.8297872340425532, 0.9302325581395349, 0.9523809523809523, 0.875</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>0.8743961352657005, 0.943502824858757, 0.9333333333333333, 0.9261363636363636, 0.9175257731958762</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>0.9791666666666666, 0.8125, 0.8333333333333334, 0.8333333333333334, 0.875</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>0.9427083333333334, 0.8697916666666666, 0.875, 0.8489583333333334, 0.9270833333333334</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>0.912621359223301, 0.8210526315789474, 0.8791208791208791, 0.888888888888889, 0.875</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>0.9072681704260651, 0.9051490514905148, 0.9032258064516129, 0.8858695652173912, 0.9222797927461139</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>0.9606481481481481, 0.8966049382716049, 0.9350961538461539, 0.9663461538461539, 0.8669871794871795</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>0.9385416666666667, 0.9472966269841271, 0.946221501572327, 0.9348221305031447, 0.9523142688679246</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CatBoostClassifier_splashing_test</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>{'estimator': &lt;catboost.core.CatBoostClassifier object at 0x000001FA077EBB20&gt;, 'source_features': ['init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'], 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': None, 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Re', 'sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.8679245283018868</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.9583333333333334</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.910891089108911</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.9483024691358024</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.9966329966329966</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.9948186528497409</v>
+      </c>
+      <c r="L6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.9974025974025974</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.9988343253968255</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>1.8345623016357422, 1.5924808979034424, 1.5990405082702637, 1.5497426986694336, 1.6355464458465576</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>0.0, 0.011824607849121094, 0.011261940002441406, 0.015034914016723633, 0.013416528701782227</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>0.9333333333333333, 0.8933333333333333, 0.8648648648648649, 0.9459459459459459, 0.8648648648648649</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>0.98989898989899, 0.98989898989899, 0.9932885906040269, 0.9865771812080537, 0.9966442953020134</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>0.9387755102040817, 0.8846153846153846, 0.9318181818181818, 0.9583333333333334, 0.8958333333333334</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>0.9896373056994818, 0.9896373056994818, 0.9947916666666666, 0.9845360824742269, 0.9948186528497409</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>0.9583333333333334, 0.9583333333333334, 0.8541666666666666, 0.9583333333333334, 0.8958333333333334</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>0.9947916666666666, 0.9947916666666666, 0.9947916666666666, 0.9947916666666666, 1.0</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>0.9484536082474228, 0.9199999999999999, 0.8913043478260869, 0.9583333333333334, 0.8958333333333334</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>0.9922077922077923, 0.9922077922077923, 0.9947916666666666, 0.9896373056994819, 0.9974025974025974</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>0.9814814814814814, 0.9722222222222222, 0.9455128205128205, 0.969551282051282, 0.905448717948718</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>0.9982638888888888, 0.9980406746031746, 0.9985996462264151, 0.9984522405660378, 1.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CatBoostClassifier_splashing_test</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>{'estimator': &lt;catboost.core.CatBoostClassifier object at 0x000001FA077E87F0&gt;, 'source_features': ['init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'], 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': None, 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Re', 'sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.8679245283018868</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.9583333333333334</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.910891089108911</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.9483024691358024</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.9966329966329966</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.9948186528497409</v>
+      </c>
+      <c r="L7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.9974025974025974</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0.9988343253968255</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>1.5326519012451172, 1.561889886856079, 1.562685251235962, 1.514699935913086, 1.5161700248718262</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>0.010239601135253906, 0.009035110473632812, 0.00038623809814453125, 0.008512496948242188, 0.01370692253112793</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>0.9333333333333333, 0.8933333333333333, 0.8648648648648649, 0.9459459459459459, 0.8648648648648649</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>0.98989898989899, 0.98989898989899, 0.9932885906040269, 0.9865771812080537, 0.9966442953020134</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>0.9387755102040817, 0.8846153846153846, 0.9318181818181818, 0.9583333333333334, 0.8958333333333334</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>0.9896373056994818, 0.9896373056994818, 0.9947916666666666, 0.9845360824742269, 0.9948186528497409</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>0.9583333333333334, 0.9583333333333334, 0.8541666666666666, 0.9583333333333334, 0.8958333333333334</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>0.9947916666666666, 0.9947916666666666, 0.9947916666666666, 0.9947916666666666, 1.0</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>0.9484536082474228, 0.9199999999999999, 0.8913043478260869, 0.9583333333333334, 0.8958333333333334</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>0.9922077922077923, 0.9922077922077923, 0.9947916666666666, 0.9896373056994819, 0.9974025974025974</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>0.9814814814814814, 0.9722222222222222, 0.9455128205128205, 0.969551282051282, 0.905448717948718</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>0.9982638888888888, 0.9980406746031746, 0.9985996462264151, 0.9984522405660378, 1.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CatBoostClassifier_splashing_test</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>{'estimator': &lt;catboost.core.CatBoostClassifier object at 0x000001FA05B67970&gt;, 'source_features': ['init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'], 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': None, 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Re', 'sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.8679245283018868</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.9583333333333334</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.910891089108911</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.9483024691358024</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.9966329966329966</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.9948186528497409</v>
+      </c>
+      <c r="L8" t="n">
+        <v>1</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.9974025974025974</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0.9988343253968255</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>1.5839686393737793, 1.4876301288604736, 1.5380446910858154, 1.614840030670166, 1.587310791015625</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>0.01909041404724121, 0.01392221450805664, 0.016156911849975586, 0.014037370681762695, 0.008305072784423828</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>0.9333333333333333, 0.8933333333333333, 0.8648648648648649, 0.9459459459459459, 0.8648648648648649</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>0.98989898989899, 0.98989898989899, 0.9932885906040269, 0.9865771812080537, 0.9966442953020134</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>0.9387755102040817, 0.8846153846153846, 0.9318181818181818, 0.9583333333333334, 0.8958333333333334</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>0.9896373056994818, 0.9896373056994818, 0.9947916666666666, 0.9845360824742269, 0.9948186528497409</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>0.9583333333333334, 0.9583333333333334, 0.8541666666666666, 0.9583333333333334, 0.8958333333333334</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>0.9947916666666666, 0.9947916666666666, 0.9947916666666666, 0.9947916666666666, 1.0</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>0.9484536082474228, 0.9199999999999999, 0.8913043478260869, 0.9583333333333334, 0.8958333333333334</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>0.9922077922077923, 0.9922077922077923, 0.9947916666666666, 0.9896373056994819, 0.9974025974025974</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>0.9814814814814814, 0.9722222222222222, 0.9455128205128205, 0.969551282051282, 0.905448717948718</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>0.9982638888888888, 0.9980406746031746, 0.9985996462264151, 0.9984522405660378, 1.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>XGBClassifier_splashing_test</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>{'estimator': XGBClassifier(base_score=None, booster=None, callbacks=None,
+              colsample_bylevel=None, colsample_bynode=None,
+              colsample_bytree=None, early_stopping_rounds=None,
+              enable_categorical=False, eval_metric=None, feature_types=None,
+              gamma=None, gpu_id=None, grow_policy=None, importance_type=None,
+              interaction_constraints=None, learning_rate=None, max_bin=None,
+              max_cat_threshold=None, max_cat_to_onehot=None,
+              max_delta_step=None, max_depth=None, max_leaves=None,
+              min_child_weight=None, missing=nan, monotone_constraints=None,
+              n_estimators=100, n_jobs=None, num_parallel_tree=None,
+              predictor=None, random_state=None, ...), 'source_features': ['init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'], 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': None, 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Re', 'sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.8679245283018868</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.9583333333333334</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.910891089108911</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.9513888888888888</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.9966329966329966</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.9948186528497409</v>
+      </c>
+      <c r="L9" t="n">
+        <v>1</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0.9974025974025974</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0.9999751984126984</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>0.09089159965515137, 0.059160709381103516, 0.08683967590332031, 0.10107588768005371, 0.06659388542175293</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>0.016202449798583984, 0.007999658584594727, 0.01626896858215332, 0.01671314239501953, 0.014142274856567383</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>0.9466666666666667, 0.8933333333333333, 0.8378378378378378, 0.9324324324324325, 0.8108108108108109</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>1.0, 0.9966329966329966, 0.9966442953020134, 0.9966442953020134, 1.0</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>0.94, 0.9, 0.9090909090909091, 0.9574468085106383, 0.84</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>1.0, 0.9948186528497409, 0.9948186528497409, 0.9948186528497409, 1.0</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>0.9791666666666666, 0.9375, 0.8333333333333334, 0.9375, 0.875</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>0.9591836734693877, 0.9183673469387755, 0.8695652173913043, 0.9473684210526315, 0.8571428571428572</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>1.0, 0.9974025974025974, 0.9974025974025974, 0.9974025974025974, 1.0</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>0.9822530864197532, 0.9737654320987654, 0.9174679487179487, 0.9599358974358974, 0.8870192307692307</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>1.0, 0.9999751984126984, 0.9999754323899371, 0.9999754323899371, 1.0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[ADD] SHAP v0, CV metrics stats
</commit_message>
<xml_diff>
--- a/results/metrics_modelling3.xlsx
+++ b/results/metrics_modelling3.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z7"/>
+  <dimension ref="A1:Z8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1242,6 +1242,118 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>no_fragmentation</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CatBoostClassifier_no_fragmentation_base</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>{'estimator': &lt;catboost.core.CatBoostClassifier object at 0x0000029003465F50&gt;, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Re', 'sedimentation_Stk'), 'log_features': ('relative_roughness',), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sign_sedimentation_Re', 'particle_liquid_density_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>0.9066666666666666</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.8095238095238095</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.8292682926829269</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.9781818181818182</v>
+      </c>
+      <c r="J8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L8" t="n">
+        <v>1</v>
+      </c>
+      <c r="M8" t="n">
+        <v>1</v>
+      </c>
+      <c r="N8" t="n">
+        <v>1</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>1.3808012008666992, 1.0942845344543457, 1.1142067909240723, 1.0898537635803223, 1.101231575012207, 1.0872023105621338, 1.101468563079834</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>0.008841991424560547, 0.008999824523925781, 0.008000373840332031, 0.007999897003173828, 0.00800180435180664, 0.007001399993896484, 0.008001089096069336</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>0.9074074074074074, 0.8301886792452831, 0.9622641509433962, 0.8867924528301887, 0.9056603773584906, 0.9433962264150944, 0.8867924528301887</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>0.9937106918238994, 1.0, 0.9968652037617555, 0.9968652037617555, 0.9937304075235109, 0.9968652037617555, 0.9905956112852664</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>0.9166666666666666, 0.6470588235294118, 0.9285714285714286, 0.75, 1.0, 0.9230769230769231, 0.7857142857142857</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>0.9880952380952381, 1.0, 0.9883720930232558, 1.0, 0.9882352941176471, 0.9883720930232558, 0.9880952380952381</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>0.7333333333333333, 0.7857142857142857, 0.9285714285714286, 0.8571428571428571, 0.6428571428571429, 0.8571428571428571, 0.7857142857142857</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>0.9880952380952381, 1.0, 1.0, 0.9882352941176471, 0.9882352941176471, 1.0, 0.9764705882352941</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>0.8148148148148148, 0.7096774193548386, 0.9285714285714286, 0.7999999999999999, 0.782608695652174, 0.888888888888889, 0.7857142857142857</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>0.9880952380952381, 1.0, 0.9941520467836257, 0.9940828402366864, 0.9882352941176471, 0.9941520467836257, 0.9822485207100591</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>0.9641025641025642, 0.9084249084249085, 0.9908424908424909, 0.9084249084249084, 0.989010989010989, 0.9688644688644689, 0.9761904761904763</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>0.999949124949125, 1.0, 0.9998994469582705, 1.0, 0.9998491704374057, 0.9998994469582704, 0.9998994469582705</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
[ADD] No fragmentation base models
</commit_message>
<xml_diff>
--- a/results/metrics_modelling3.xlsx
+++ b/results/metrics_modelling3.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BJ8"/>
+  <dimension ref="A1:BJ12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2290,6 +2290,896 @@
         <v>1.988619454760789e-05</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>no_fragmentation</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>LogisticRegression_no_fragmentation_base</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>{'estimator': LogisticRegression(), 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Re', 'sedimentation_Stk'), 'log_features': ('relative_roughness',), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sign_sedimentation_Re', 'particle_liquid_density_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>0.8533333333333334</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.7368421052631579</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.717948717948718</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.9254545454545455</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.8754208754208754</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.8181818181818182</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.6835443037974683</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0.7448275862068965</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0.9316571826733249</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>0.00896906852722168, 0.013093233108520508, 0.0, 0.008106708526611328, 0.010124683380126953, 0.0, 0.0</t>
+        </is>
+      </c>
+      <c r="P9" t="n">
+        <v>0.005756241934640067</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0.008106708526611328</v>
+      </c>
+      <c r="R9" t="n">
+        <v>0.005184656369554661</v>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>0.007524251937866211, 0.005464315414428711, 0.010611295700073242, 0.0, 0.0, 0.0, 0.010504722595214844</t>
+        </is>
+      </c>
+      <c r="T9" t="n">
+        <v>0.00487208366394043</v>
+      </c>
+      <c r="U9" t="n">
+        <v>0.005464315414428711</v>
+      </c>
+      <c r="V9" t="n">
+        <v>0.004523928583663451</v>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>0.8148148148148148, 0.7924528301886793, 0.9245283018867925, 0.8490566037735849, 0.8490566037735849, 0.8490566037735849, 0.8867924528301887</t>
+        </is>
+      </c>
+      <c r="X9" t="n">
+        <v>0.85225117300589</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>0.8490566037735849</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>0.04039982656823135</v>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>0.5833333333333334, 0.6206896551724138, 0.8571428571428571, 0.7333333333333334, 0.6363636363636364, 0.6666666666666666, 0.7999999999999999</t>
+        </is>
+      </c>
+      <c r="AB9" t="n">
+        <v>0.6996470688588915</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>0.09324779318350135</v>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>0.7777777777777778, 0.6, 0.8571428571428571, 0.6875, 0.875, 0.8, 0.75</t>
+        </is>
+      </c>
+      <c r="AF9" t="n">
+        <v>0.7639172335600907</v>
+      </c>
+      <c r="AG9" t="n">
+        <v>0.7777777777777778</v>
+      </c>
+      <c r="AH9" t="n">
+        <v>0.08898364299549143</v>
+      </c>
+      <c r="AI9" t="inlineStr">
+        <is>
+          <t>0.4666666666666667, 0.6428571428571429, 0.8571428571428571, 0.7857142857142857, 0.5, 0.5714285714285714, 0.8571428571428571</t>
+        </is>
+      </c>
+      <c r="AJ9" t="n">
+        <v>0.6687074829931972</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>0.6428571428571429</v>
+      </c>
+      <c r="AL9" t="n">
+        <v>0.1531201700556019</v>
+      </c>
+      <c r="AM9" t="inlineStr">
+        <is>
+          <t>0.9418803418803419, 0.8498168498168499, 0.9578754578754578, 0.8864468864468865, 0.9560439560439561, 0.9212454212454212, 0.9633699633699634</t>
+        </is>
+      </c>
+      <c r="AN9" t="n">
+        <v>0.9252398395255538</v>
+      </c>
+      <c r="AO9" t="n">
+        <v>0.9418803418803419</v>
+      </c>
+      <c r="AP9" t="n">
+        <v>0.03955875522584676</v>
+      </c>
+      <c r="AQ9" t="inlineStr">
+        <is>
+          <t>0.8773584905660378, 0.877742946708464, 0.8589341692789969, 0.877742946708464, 0.8746081504702194, 0.8714733542319749, 0.8526645768025078</t>
+        </is>
+      </c>
+      <c r="AR9" t="n">
+        <v>0.8700749478238093</v>
+      </c>
+      <c r="AS9" t="n">
+        <v>0.8746081504702194</v>
+      </c>
+      <c r="AT9" t="n">
+        <v>0.009414197796548299</v>
+      </c>
+      <c r="AU9" t="inlineStr">
+        <is>
+          <t>0.7547169811320756, 0.7577639751552795, 0.7133757961783439, 0.751592356687898, 0.7468354430379747, 0.7453416149068324, 0.69281045751634</t>
+        </is>
+      </c>
+      <c r="AV9" t="n">
+        <v>0.737490946373535</v>
+      </c>
+      <c r="AW9" t="n">
+        <v>0.7468354430379747</v>
+      </c>
+      <c r="AX9" t="n">
+        <v>0.02278289116899502</v>
+      </c>
+      <c r="AY9" t="inlineStr">
+        <is>
+          <t>0.8, 0.8026315789473685, 0.7777777777777778, 0.8194444444444444, 0.8082191780821918, 0.7894736842105263, 0.7794117647058824</t>
+        </is>
+      </c>
+      <c r="AZ9" t="n">
+        <v>0.7967083468811701</v>
+      </c>
+      <c r="BA9" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="BB9" t="n">
+        <v>0.014168514244079</v>
+      </c>
+      <c r="BC9" t="inlineStr">
+        <is>
+          <t>0.7142857142857143, 0.7176470588235294, 0.6588235294117647, 0.6941176470588235, 0.6941176470588235, 0.7058823529411765, 0.6235294117647059</t>
+        </is>
+      </c>
+      <c r="BD9" t="n">
+        <v>0.6869147659063627</v>
+      </c>
+      <c r="BE9" t="n">
+        <v>0.6941176470588235</v>
+      </c>
+      <c r="BF9" t="n">
+        <v>0.03154134629409137</v>
+      </c>
+      <c r="BG9" t="inlineStr">
+        <is>
+          <t>0.9281135531135531, 0.9407742584213172, 0.9262443438914028, 0.9370035193564605, 0.9277526395173454, 0.9327300150829563, 0.9243841126194067</t>
+        </is>
+      </c>
+      <c r="BH9" t="n">
+        <v>0.9310003488574919</v>
+      </c>
+      <c r="BI9" t="n">
+        <v>0.9281135531135531</v>
+      </c>
+      <c r="BJ9" t="n">
+        <v>0.005604009792409489</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>no_fragmentation</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>KNeighborsClassifier_no_fragmentation_base</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>{'estimator': KNeighborsClassifier(), 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Re', 'sedimentation_Stk'), 'log_features': ('relative_roughness',), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sign_sedimentation_Re', 'particle_liquid_density_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.7894736842105263</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.7692307692307692</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.9495454545454545</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.8922558922558923</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.8309859154929577</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.7468354430379747</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.7866666666666666</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0.9578155847172223</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>0.007361412048339844, 0.0034761428833007812, 0.0, 0.004326820373535156, 0.0, 0.01344752311706543, 0.00612187385559082</t>
+        </is>
+      </c>
+      <c r="P10" t="n">
+        <v>0.004961967468261719</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>0.004326820373535156</v>
+      </c>
+      <c r="R10" t="n">
+        <v>0.00432535218434897</v>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>0.010094881057739258, 0.002934694290161133, 0.013010263442993164, 0.004120349884033203, 0.0160982608795166, 0.0, 0.008006095886230469</t>
+        </is>
+      </c>
+      <c r="T10" t="n">
+        <v>0.007752077920096261</v>
+      </c>
+      <c r="U10" t="n">
+        <v>0.008006095886230469</v>
+      </c>
+      <c r="V10" t="n">
+        <v>0.005336556973224901</v>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>0.8888888888888888, 0.7735849056603774, 0.8679245283018868, 0.8301886792452831, 0.8490566037735849, 0.8490566037735849, 0.8867924528301887</t>
+        </is>
+      </c>
+      <c r="X10" t="n">
+        <v>0.8493560946391135</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>0.8490566037735849</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>0.03667999015847824</v>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>0.8000000000000002, 0.5714285714285714, 0.7200000000000001, 0.6666666666666666, 0.6923076923076924, 0.6666666666666666, 0.8125000000000001</t>
+        </is>
+      </c>
+      <c r="AB10" t="n">
+        <v>0.7042242281527996</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>0.6923076923076924</v>
+      </c>
+      <c r="AD10" t="n">
+        <v>0.07722263485750151</v>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>0.8, 0.5714285714285714, 0.8181818181818182, 0.6923076923076923, 0.75, 0.8, 0.7222222222222222</t>
+        </is>
+      </c>
+      <c r="AF10" t="n">
+        <v>0.7363057577343292</v>
+      </c>
+      <c r="AG10" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AH10" t="n">
+        <v>0.07957368269107451</v>
+      </c>
+      <c r="AI10" t="inlineStr">
+        <is>
+          <t>0.8, 0.5714285714285714, 0.6428571428571429, 0.6428571428571429, 0.6428571428571429, 0.5714285714285714, 0.9285714285714286</t>
+        </is>
+      </c>
+      <c r="AJ10" t="n">
+        <v>0.6857142857142857</v>
+      </c>
+      <c r="AK10" t="n">
+        <v>0.6428571428571429</v>
+      </c>
+      <c r="AL10" t="n">
+        <v>0.1216983797214333</v>
+      </c>
+      <c r="AM10" t="inlineStr">
+        <is>
+          <t>0.9444444444444444, 0.8772893772893773, 0.9487179487179488, 0.8946886446886448, 0.9010989010989011, 0.903846153846154, 0.9468864468864469</t>
+        </is>
+      </c>
+      <c r="AN10" t="n">
+        <v>0.9167102738531312</v>
+      </c>
+      <c r="AO10" t="n">
+        <v>0.903846153846154</v>
+      </c>
+      <c r="AP10" t="n">
+        <v>0.02713046960614661</v>
+      </c>
+      <c r="AQ10" t="inlineStr">
+        <is>
+          <t>0.89937106918239, 0.9059561128526645, 0.9122257053291536, 0.9028213166144201, 0.9059561128526645, 0.9028213166144201, 0.9028213166144201</t>
+        </is>
+      </c>
+      <c r="AR10" t="n">
+        <v>0.9045675642943048</v>
+      </c>
+      <c r="AS10" t="n">
+        <v>0.9028213166144201</v>
+      </c>
+      <c r="AT10" t="n">
+        <v>0.003754139860286498</v>
+      </c>
+      <c r="AU10" t="inlineStr">
+        <is>
+          <t>0.8117647058823529, 0.8255813953488372, 0.829268292682927, 0.8165680473372781, 0.8255813953488372, 0.822857142857143, 0.8143712574850299</t>
+        </is>
+      </c>
+      <c r="AV10" t="n">
+        <v>0.820856033848915</v>
+      </c>
+      <c r="AW10" t="n">
+        <v>0.822857142857143</v>
+      </c>
+      <c r="AX10" t="n">
+        <v>0.00612395781888402</v>
+      </c>
+      <c r="AY10" t="inlineStr">
+        <is>
+          <t>0.8023255813953488, 0.8160919540229885, 0.8607594936708861, 0.8214285714285714, 0.8160919540229885, 0.8, 0.8292682926829268</t>
+        </is>
+      </c>
+      <c r="AZ10" t="n">
+        <v>0.8208522638891014</v>
+      </c>
+      <c r="BA10" t="n">
+        <v>0.8160919540229885</v>
+      </c>
+      <c r="BB10" t="n">
+        <v>0.01884949652022786</v>
+      </c>
+      <c r="BC10" t="inlineStr">
+        <is>
+          <t>0.8214285714285714, 0.8352941176470589, 0.8, 0.8117647058823529, 0.8352941176470589, 0.8470588235294118, 0.8</t>
+        </is>
+      </c>
+      <c r="BD10" t="n">
+        <v>0.821548619447779</v>
+      </c>
+      <c r="BE10" t="n">
+        <v>0.8214285714285714</v>
+      </c>
+      <c r="BF10" t="n">
+        <v>0.01712589238622703</v>
+      </c>
+      <c r="BG10" t="inlineStr">
+        <is>
+          <t>0.9602920227920229, 0.9680744092508797, 0.9614379084967319, 0.9640020110608346, 0.9654600301659125, 0.9612116641528407, 0.9623428858722977</t>
+        </is>
+      </c>
+      <c r="BH10" t="n">
+        <v>0.9632601331130743</v>
+      </c>
+      <c r="BI10" t="n">
+        <v>0.9623428858722977</v>
+      </c>
+      <c r="BJ10" t="n">
+        <v>0.002556083322909469</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>no_fragmentation</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>SVC_no_fragmentation_base</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>{'estimator': SVC(probability=True), 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Re', 'sedimentation_Stk'), 'log_features': ('relative_roughness',), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sign_sedimentation_Re', 'particle_liquid_density_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.7222222222222222</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.6842105263157895</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.9281818181818182</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.8888888888888888</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0.8194444444444444</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.7468354430379747</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0.781456953642384</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0.9624898385785624</v>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>0.008918046951293945, 0.015131235122680664, 0.00925302505493164, 0.005823373794555664, 0.015625, 0.015604257583618164, 0.026727914810180664</t>
+        </is>
+      </c>
+      <c r="P11" t="n">
+        <v>0.01386897904532296</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>0.01513123512268066</v>
+      </c>
+      <c r="R11" t="n">
+        <v>0.006364980577914103</v>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>0.029338359832763672, 0.008470535278320312, 0.011104106903076172, 0.010102987289428711, 0.0, 0.0, 0.0024471282958984375</t>
+        </is>
+      </c>
+      <c r="T11" t="n">
+        <v>0.00878044537135533</v>
+      </c>
+      <c r="U11" t="n">
+        <v>0.008470535278320312</v>
+      </c>
+      <c r="V11" t="n">
+        <v>0.009442879088229031</v>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>0.8333333333333334, 0.7358490566037735, 0.8679245283018868, 0.8867924528301887, 0.8867924528301887, 0.8679245283018868, 0.8301886792452831</t>
+        </is>
+      </c>
+      <c r="X11" t="n">
+        <v>0.844115004492363</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>0.8679245283018868</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>0.04900177617977858</v>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>0.6666666666666665, 0.5, 0.6956521739130435, 0.7857142857142857, 0.75, 0.7200000000000001, 0.689655172413793</t>
+        </is>
+      </c>
+      <c r="AB11" t="n">
+        <v>0.6868126141011126</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>0.6956521739130435</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>0.08474045998405863</v>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>0.75, 0.5, 0.8888888888888888, 0.7857142857142857, 0.9, 0.8181818181818182, 0.6666666666666666</t>
+        </is>
+      </c>
+      <c r="AF11" t="n">
+        <v>0.75849309420738</v>
+      </c>
+      <c r="AG11" t="n">
+        <v>0.7857142857142857</v>
+      </c>
+      <c r="AH11" t="n">
+        <v>0.1290923865694569</v>
+      </c>
+      <c r="AI11" t="inlineStr">
+        <is>
+          <t>0.6, 0.5, 0.5714285714285714, 0.7857142857142857, 0.6428571428571429, 0.6428571428571429, 0.7142857142857143</t>
+        </is>
+      </c>
+      <c r="AJ11" t="n">
+        <v>0.636734693877551</v>
+      </c>
+      <c r="AK11" t="n">
+        <v>0.6428571428571429</v>
+      </c>
+      <c r="AL11" t="n">
+        <v>0.08668065543508287</v>
+      </c>
+      <c r="AM11" t="inlineStr">
+        <is>
+          <t>0.9384615384615385, 0.8626373626373627, 0.9725274725274725, 0.9267399267399268, 0.9523809523809523, 0.9432234432234433, 0.9413919413919414</t>
+        </is>
+      </c>
+      <c r="AN11" t="n">
+        <v>0.9339089481946626</v>
+      </c>
+      <c r="AO11" t="n">
+        <v>0.9413919413919414</v>
+      </c>
+      <c r="AP11" t="n">
+        <v>0.03190862001703766</v>
+      </c>
+      <c r="AQ11" t="inlineStr">
+        <is>
+          <t>0.8805031446540881, 0.9028213166144201, 0.8683385579937304, 0.8840125391849529, 0.8808777429467085, 0.8840125391849529, 0.8746081504702194</t>
+        </is>
+      </c>
+      <c r="AR11" t="n">
+        <v>0.8821677130070105</v>
+      </c>
+      <c r="AS11" t="n">
+        <v>0.8808777429467085</v>
+      </c>
+      <c r="AT11" t="n">
+        <v>0.009900977108437748</v>
+      </c>
+      <c r="AU11" t="inlineStr">
+        <is>
+          <t>0.7532467532467533, 0.8248587570621468, 0.7272727272727274, 0.7836257309941521, 0.7790697674418604, 0.7784431137724551, 0.7368421052631579</t>
+        </is>
+      </c>
+      <c r="AV11" t="n">
+        <v>0.7690512792933218</v>
+      </c>
+      <c r="AW11" t="n">
+        <v>0.7784431137724551</v>
+      </c>
+      <c r="AX11" t="n">
+        <v>0.03058507390673511</v>
+      </c>
+      <c r="AY11" t="inlineStr">
+        <is>
+          <t>0.8285714285714286, 0.7934782608695652, 0.8115942028985508, 0.7790697674418605, 0.7701149425287356, 0.7926829268292683, 0.835820895522388</t>
+        </is>
+      </c>
+      <c r="AZ11" t="n">
+        <v>0.8016189178088281</v>
+      </c>
+      <c r="BA11" t="n">
+        <v>0.7934782608695652</v>
+      </c>
+      <c r="BB11" t="n">
+        <v>0.02281229712069013</v>
+      </c>
+      <c r="BC11" t="inlineStr">
+        <is>
+          <t>0.6904761904761905, 0.8588235294117647, 0.6588235294117647, 0.788235294117647, 0.788235294117647, 0.7647058823529411, 0.6588235294117647</t>
+        </is>
+      </c>
+      <c r="BD11" t="n">
+        <v>0.7440176070428172</v>
+      </c>
+      <c r="BE11" t="n">
+        <v>0.7647058823529411</v>
+      </c>
+      <c r="BF11" t="n">
+        <v>0.07061116591341229</v>
+      </c>
+      <c r="BG11" t="inlineStr">
+        <is>
+          <t>0.9595543345543346, 0.9641025641025641, 0.9572146807440925, 0.9567621920563096, 0.9577677224736049, 0.956913021618904, 0.9638511814982402</t>
+        </is>
+      </c>
+      <c r="BH11" t="n">
+        <v>0.9594522424354358</v>
+      </c>
+      <c r="BI11" t="n">
+        <v>0.9577677224736049</v>
+      </c>
+      <c r="BJ11" t="n">
+        <v>0.002988427262158618</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>no_fragmentation</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>XGBClassifier_no_fragmentation_base</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>{'estimator': XGBClassifier(base_score=None, booster=None, callbacks=None,
+              colsample_bylevel=None, colsample_bynode=None,
+              colsample_bytree=None, early_stopping_rounds=None,
+              enable_categorical=False, eval_metric=None, feature_types=None,
+              gamma=None, gpu_id=None, grow_policy=None, importance_type=None,
+              interaction_constraints=None, learning_rate=None, max_bin=None,
+              max_cat_threshold=None, max_cat_to_onehot=None,
+              max_delta_step=None, max_depth=None, max_leaves=None,
+              min_child_weight=None, missing=nan, monotone_constraints=None,
+              n_estimators=100, n_jobs=None, num_parallel_tree=None,
+              predictor=None, random_state=None, ...), 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Re', 'sedimentation_Stk'), 'log_features': ('relative_roughness',), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sign_sedimentation_Re', 'particle_liquid_density_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.7619047619047619</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.7804878048780488</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.9654545454545455</v>
+      </c>
+      <c r="J12" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" t="n">
+        <v>1</v>
+      </c>
+      <c r="L12" t="n">
+        <v>1</v>
+      </c>
+      <c r="M12" t="n">
+        <v>1</v>
+      </c>
+      <c r="N12" t="n">
+        <v>1</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>0.07788205146789551, 0.05489039421081543, 0.06288433074951172, 0.057038068771362305, 0.04688525199890137, 0.07667183876037598, 0.0814962387084961</t>
+        </is>
+      </c>
+      <c r="P12" t="n">
+        <v>0.0653925963810512</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>0.06288433074951172</v>
+      </c>
+      <c r="R12" t="n">
+        <v>0.01237187286775673</v>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>0.019135475158691406, 0.01563429832458496, 0.016017913818359375, 0.01617717742919922, 0.015770435333251953, 0.015863656997680664, 0.013914346694946289</t>
+        </is>
+      </c>
+      <c r="T12" t="n">
+        <v>0.01607332910810198</v>
+      </c>
+      <c r="U12" t="n">
+        <v>0.01586365699768066</v>
+      </c>
+      <c r="V12" t="n">
+        <v>0.001433290613797244</v>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>0.9074074074074074, 0.8113207547169812, 0.9433962264150944, 0.8867924528301887, 0.9245283018867925, 0.8867924528301887, 0.9056603773584906</t>
+        </is>
+      </c>
+      <c r="X12" t="n">
+        <v>0.8951282819207348</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>0.9056603773584906</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>0.03894782463392368</v>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>0.8, 0.6428571428571429, 0.88, 0.7999999999999999, 0.8571428571428571, 0.7857142857142857, 0.8275862068965518</t>
+        </is>
+      </c>
+      <c r="AB12" t="n">
+        <v>0.7990429275158339</v>
+      </c>
+      <c r="AC12" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AD12" t="n">
+        <v>0.07103103165205046</v>
+      </c>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t>1.0, 0.6428571428571429, 1.0, 0.75, 0.8571428571428571, 0.7857142857142857, 0.8</t>
+        </is>
+      </c>
+      <c r="AF12" t="n">
+        <v>0.8336734693877551</v>
+      </c>
+      <c r="AG12" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AH12" t="n">
+        <v>0.1211409730861799</v>
+      </c>
+      <c r="AI12" t="inlineStr">
+        <is>
+          <t>0.6666666666666666, 0.6428571428571429, 0.7857142857142857, 0.8571428571428571, 0.8571428571428571, 0.7857142857142857, 0.8571428571428571</t>
+        </is>
+      </c>
+      <c r="AJ12" t="n">
+        <v>0.7789115646258503</v>
+      </c>
+      <c r="AK12" t="n">
+        <v>0.7857142857142857</v>
+      </c>
+      <c r="AL12" t="n">
+        <v>0.08414501276770733</v>
+      </c>
+      <c r="AM12" t="inlineStr">
+        <is>
+          <t>0.9709401709401709, 0.8736263736263736, 0.9798534798534799, 0.9267399267399268, 0.9780219780219781, 0.967032967032967, 0.9780219780219781</t>
+        </is>
+      </c>
+      <c r="AN12" t="n">
+        <v>0.9534624106052678</v>
+      </c>
+      <c r="AO12" t="n">
+        <v>0.9709401709401709</v>
+      </c>
+      <c r="AP12" t="n">
+        <v>0.03680129906862034</v>
+      </c>
+      <c r="AQ12" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="AR12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU12" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="AV12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY12" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="AZ12" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA12" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC12" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="BD12" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE12" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG12" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 0.9999999999999999, 1.0, 0.9999999999999999, 1.0</t>
+        </is>
+      </c>
+      <c r="BH12" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI12" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ12" t="n">
+        <v>5.934391687221749e-17</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
[ADD] Best features in logit research
</commit_message>
<xml_diff>
--- a/results/metrics_modelling3.xlsx
+++ b/results/metrics_modelling3.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BJ12"/>
+  <dimension ref="A1:BJ13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -793,31 +793,31 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>0.005259990692138672, 0.00709986686706543, 0.008516073226928711, 0.0029969215393066406, 0.0077550411224365234, 0.0030901432037353516, 0.007534027099609375</t>
+          <t>0.02117919921875, 0.0032470226287841797, 0.003450155258178711, 0.0030150413513183594, 0.0029571056365966797, 0.003010988235473633, 0.0067059993743896484</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>0.006036009107317243</v>
+        <v>0.006223644529070173</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.00709986686706543</v>
+        <v>0.00324702262878418</v>
       </c>
       <c r="R2" t="n">
-        <v>0.002104350055521584</v>
+        <v>0.006230574086080055</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>0.014683961868286133, 0.007281303405761719, 0.007439851760864258, 0.004224061965942383, 0.004151821136474609, 0.0070989131927490234, 0.00782012939453125</t>
+          <t>0.011981725692749023, 0.006932973861694336, 0.008883953094482422, 0.006124019622802734, 0.004461050033569336, 0.004125833511352539, 0.01243901252746582</t>
         </is>
       </c>
       <c r="T2" t="n">
-        <v>0.007528577532087054</v>
+        <v>0.007849795477730888</v>
       </c>
       <c r="U2" t="n">
-        <v>0.007281303405761719</v>
+        <v>0.006932973861694336</v>
       </c>
       <c r="V2" t="n">
-        <v>0.003248306428409989</v>
+        <v>0.003125325011603613</v>
       </c>
       <c r="W2" t="inlineStr">
         <is>
@@ -968,216 +968,216 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>splashing</t>
+          <t>no_fragmentation</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>LogisticRegression_splashing_base</t>
+          <t>Logit_no_fragmentation_base</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>{'estimator': LogisticRegression(), 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Re', 'sedimentation_Stk'), 'log_features': ('relative_roughness',), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sign_sedimentation_Re', 'particle_liquid_density_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
+          <t>{'estimator': StatsModelsEstimator(model_class=&lt;class 'statsmodels.discrete.discrete_model.Logit'&gt;), 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Re', 'sedimentation_Stk'), 'log_features': ('relative_roughness',), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sign_sedimentation_Re', 'particle_liquid_density_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.8133333333333334</v>
+        <v>0.84</v>
       </c>
       <c r="F3" t="n">
-        <v>0.8035714285714286</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="G3" t="n">
-        <v>0.9375</v>
+        <v>0.8</v>
       </c>
       <c r="H3" t="n">
-        <v>0.8653846153846154</v>
+        <v>0.7272727272727272</v>
       </c>
       <c r="I3" t="n">
-        <v>0.8912037037037037</v>
+        <v>0.9081818181818181</v>
       </c>
       <c r="J3" t="n">
-        <v>0.8148148148148148</v>
+        <v>0.8282828282828283</v>
       </c>
       <c r="K3" t="n">
-        <v>0.8407960199004975</v>
+        <v>0.6555555555555556</v>
       </c>
       <c r="L3" t="n">
-        <v>0.8802083333333334</v>
+        <v>0.7468354430379747</v>
       </c>
       <c r="M3" t="n">
-        <v>0.8600508905852416</v>
+        <v>0.698224852071006</v>
       </c>
       <c r="N3" t="n">
-        <v>0.9132688492063492</v>
+        <v>0.9099988386946928</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>0.00602412223815918, 0.0033731460571289062, 0.0034301280975341797, 0.003506898880004883, 0.003591775894165039, 0.004220008850097656, 0.0030460357666015625</t>
+          <t>0.0072820186614990234, 0.0034618377685546875, 0.005471229553222656, 0.0029850006103515625, 0.009046792984008789, 0.002930879592895508, 0.0034608840942382812</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>0.003884587969098772</v>
+        <v>0.00494837760925293</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.003506898880004883</v>
+        <v>0.003461837768554688</v>
       </c>
       <c r="R3" t="n">
-        <v>0.0009327209363421094</v>
+        <v>0.002231714537591837</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>0.00506901741027832, 0.004395723342895508, 0.00477290153503418, 0.004426002502441406, 0.004522085189819336, 0.004422187805175781, 0.004745006561279297</t>
+          <t>0.009822845458984375, 0.004209995269775391, 0.00435185432434082, 0.010168075561523438, 0.006246089935302734, 0.004252195358276367, 0.004079103469848633</t>
         </is>
       </c>
       <c r="T3" t="n">
-        <v>0.004621846335274833</v>
+        <v>0.00616145133972168</v>
       </c>
       <c r="U3" t="n">
-        <v>0.004522085189819336</v>
+        <v>0.00435185432434082</v>
       </c>
       <c r="V3" t="n">
-        <v>0.0002321484482853146</v>
+        <v>0.0025221946636105</v>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>0.8703703703703703, 0.7924528301886793, 0.8490566037735849, 0.7735849056603774, 0.8301886792452831, 0.7547169811320755, 0.7735849056603774</t>
+          <t>0.8518518518518519, 0.8113207547169812, 0.8867924528301887, 0.7547169811320755, 0.8301886792452831, 0.8490566037735849, 0.8679245283018868</t>
         </is>
       </c>
       <c r="X3" t="n">
-        <v>0.8062793251472496</v>
+        <v>0.835978835978836</v>
       </c>
       <c r="Y3" t="n">
-        <v>0.7924528301886793</v>
+        <v>0.8490566037735849</v>
       </c>
       <c r="Z3" t="n">
-        <v>0.04052673239832488</v>
+        <v>0.0401258155209778</v>
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>0.9090909090909091, 0.8405797101449276, 0.8857142857142858, 0.8235294117647058, 0.8695652173913043, 0.8115942028985507, 0.8333333333333333</t>
+          <t>0.7142857142857142, 0.6428571428571429, 0.7999999999999999, 0.6285714285714286, 0.6666666666666666, 0.6923076923076924, 0.7878787878787878</t>
         </is>
       </c>
       <c r="AB3" t="n">
-        <v>0.8533438671911453</v>
+        <v>0.704652490366776</v>
       </c>
       <c r="AC3" t="n">
-        <v>0.8405797101449276</v>
+        <v>0.6923076923076924</v>
       </c>
       <c r="AD3" t="n">
-        <v>0.03298049265322964</v>
+        <v>0.06246470200147004</v>
       </c>
       <c r="AE3" t="inlineStr">
         <is>
-          <t>0.8333333333333334, 0.8529411764705882, 0.8611111111111112, 0.8235294117647058, 0.8571428571428571, 0.8, 0.7894736842105263</t>
+          <t>0.7692307692307693, 0.6428571428571429, 0.75, 0.5238095238095238, 0.6923076923076923, 0.75, 0.6842105263157895</t>
         </is>
       </c>
       <c r="AF3" t="n">
-        <v>0.8310759391475887</v>
+        <v>0.6874879506458454</v>
       </c>
       <c r="AG3" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.6923076923076923</v>
       </c>
       <c r="AH3" t="n">
-        <v>0.02623572233655289</v>
+        <v>0.07866194292625306</v>
       </c>
       <c r="AI3" t="inlineStr">
         <is>
-          <t>1.0, 0.8285714285714286, 0.9117647058823529, 0.8235294117647058, 0.8823529411764706, 0.8235294117647058, 0.8823529411764706</t>
+          <t>0.6666666666666666, 0.6428571428571429, 0.8571428571428571, 0.7857142857142857, 0.6428571428571429, 0.6428571428571429, 0.9285714285714286</t>
         </is>
       </c>
       <c r="AJ3" t="n">
-        <v>0.8788715486194477</v>
+        <v>0.7380952380952381</v>
       </c>
       <c r="AK3" t="n">
-        <v>0.8823529411764706</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="AL3" t="n">
-        <v>0.05908094691303778</v>
+        <v>0.1102166785443514</v>
       </c>
       <c r="AM3" t="inlineStr">
         <is>
-          <t>0.9578947368421054, 0.8571428571428572, 0.9504643962848297, 0.8869969040247677, 0.9411764705882353, 0.8126934984520124, 0.8606811145510836</t>
+          <t>0.9316239316239316, 0.8644688644688645, 0.9340659340659341, 0.86996336996337, 0.9102564102564102, 0.9065934065934067, 0.9578754578754578</t>
         </is>
       </c>
       <c r="AN3" t="n">
-        <v>0.8952928539836987</v>
+        <v>0.9106924821210536</v>
       </c>
       <c r="AO3" t="n">
-        <v>0.8869969040247677</v>
+        <v>0.9102564102564102</v>
       </c>
       <c r="AP3" t="n">
-        <v>0.05156559231488393</v>
+        <v>0.03167503077011312</v>
       </c>
       <c r="AQ3" t="inlineStr">
         <is>
-          <t>0.8113207547169812, 0.8119122257053292, 0.8119122257053292, 0.8150470219435737, 0.8119122257053292, 0.8463949843260188, 0.8181818181818182</t>
+          <t>0.8333333333333334, 0.8338557993730408, 0.8338557993730408, 0.8495297805642633, 0.8275862068965517, 0.8463949843260188, 0.8369905956112853</t>
         </is>
       </c>
       <c r="AR3" t="n">
-        <v>0.8180973223263399</v>
+        <v>0.8373637856396476</v>
       </c>
       <c r="AS3" t="n">
-        <v>0.8119122257053292</v>
+        <v>0.8338557993730408</v>
       </c>
       <c r="AT3" t="n">
-        <v>0.01177623075655056</v>
+        <v>0.007232572948425511</v>
       </c>
       <c r="AU3" t="inlineStr">
         <is>
-          <t>0.8578199052132701, 0.8584905660377359, 0.8584905660377358, 0.8618266978922716, 0.8591549295774649, 0.883054892601432, 0.8632075471698114</t>
+          <t>0.6971428571428572, 0.707182320441989, 0.6971428571428572, 0.7303370786516853, 0.6892655367231638, 0.7134502923976608, 0.7078651685393259</t>
         </is>
       </c>
       <c r="AV3" t="n">
-        <v>0.8631493006471033</v>
+        <v>0.7060551587199342</v>
       </c>
       <c r="AW3" t="n">
-        <v>0.8591549295774649</v>
+        <v>0.707182320441989</v>
       </c>
       <c r="AX3" t="n">
-        <v>0.008330240384199985</v>
+        <v>0.01247623977448649</v>
       </c>
       <c r="AY3" t="inlineStr">
         <is>
-          <t>0.8341013824884793, 0.8310502283105022, 0.8348623853211009, 0.832579185520362, 0.8318181818181818, 0.8685446009389671, 0.8394495412844036</t>
+          <t>0.6703296703296703, 0.6666666666666666, 0.6777777777777778, 0.6989247311827957, 0.6630434782608695, 0.7093023255813954, 0.6774193548387096</t>
         </is>
       </c>
       <c r="AZ3" t="n">
-        <v>0.8389150722402852</v>
+        <v>0.6804948578054122</v>
       </c>
       <c r="BA3" t="n">
-        <v>0.8341013824884793</v>
+        <v>0.6774193548387096</v>
       </c>
       <c r="BB3" t="n">
-        <v>0.01236443975154782</v>
+        <v>0.01597083157929664</v>
       </c>
       <c r="BC3" t="inlineStr">
         <is>
-          <t>0.8829268292682927, 0.8878048780487805, 0.883495145631068, 0.8932038834951457, 0.8883495145631068, 0.8980582524271845, 0.8883495145631068</t>
+          <t>0.7261904761904762, 0.7529411764705882, 0.7176470588235294, 0.7647058823529411, 0.7176470588235294, 0.7176470588235294, 0.7411764705882353</t>
         </is>
       </c>
       <c r="BD3" t="n">
-        <v>0.888884002570955</v>
+        <v>0.7339935974389756</v>
       </c>
       <c r="BE3" t="n">
-        <v>0.8883495145631068</v>
+        <v>0.7261904761904762</v>
       </c>
       <c r="BF3" t="n">
-        <v>0.00491487231480214</v>
+        <v>0.01779392166608651</v>
       </c>
       <c r="BG3" t="inlineStr">
         <is>
-          <t>0.8975825598963955, 0.9145485665382971, 0.9012586992009622, 0.9084328550562764, 0.8984234040725149, 0.9190652117879542, 0.9092061173640348</t>
+          <t>0.907967032967033, 0.9191050779286074, 0.9073906485671193, 0.9190548014077425, 0.9080945198592257, 0.9143790849673202, 0.9038712921065862</t>
         </is>
       </c>
       <c r="BH3" t="n">
-        <v>0.9069310591309193</v>
+        <v>0.9114089225433765</v>
       </c>
       <c r="BI3" t="n">
-        <v>0.9084328550562764</v>
+        <v>0.9080945198592257</v>
       </c>
       <c r="BJ3" t="n">
-        <v>0.007603060102699606</v>
+        <v>0.005635428789683134</v>
       </c>
     </row>
     <row r="4">
@@ -1193,211 +1193,211 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>KNeighborsClassifier_splashing_base</t>
+          <t>LogisticRegression_splashing_base</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>{'estimator': KNeighborsClassifier(), 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Re', 'sedimentation_Stk'), 'log_features': ('relative_roughness',), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sign_sedimentation_Re', 'particle_liquid_density_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
+          <t>{'estimator': LogisticRegression(), 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Re', 'sedimentation_Stk'), 'log_features': ('relative_roughness',), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sign_sedimentation_Re', 'particle_liquid_density_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
         </is>
       </c>
       <c r="E4" t="n">
         <v>0.8133333333333334</v>
       </c>
       <c r="F4" t="n">
-        <v>0.8269230769230769</v>
+        <v>0.8035714285714286</v>
       </c>
       <c r="G4" t="n">
-        <v>0.8958333333333334</v>
+        <v>0.9375</v>
       </c>
       <c r="H4" t="n">
-        <v>0.86</v>
+        <v>0.8653846153846154</v>
       </c>
       <c r="I4" t="n">
-        <v>0.880787037037037</v>
+        <v>0.8912037037037037</v>
       </c>
       <c r="J4" t="n">
-        <v>0.9158249158249159</v>
+        <v>0.8148148148148148</v>
       </c>
       <c r="K4" t="n">
-        <v>0.9282051282051282</v>
+        <v>0.8407960199004975</v>
       </c>
       <c r="L4" t="n">
-        <v>0.9427083333333334</v>
+        <v>0.8802083333333334</v>
       </c>
       <c r="M4" t="n">
-        <v>0.9354005167958657</v>
+        <v>0.8600508905852416</v>
       </c>
       <c r="N4" t="n">
-        <v>0.9661954365079365</v>
+        <v>0.9132688492063492</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>0.0033121109008789062, 0.002633333206176758, 0.002763032913208008, 0.0028138160705566406, 0.0028731822967529297, 0.002604961395263672, 0.002413034439086914</t>
+          <t>0.0065839290618896484, 0.003679990768432617, 0.00339508056640625, 0.003592967987060547, 0.0034291744232177734, 0.004132270812988281, 0.003287076950073242</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>0.002773353031703404</v>
+        <v>0.004014355795724052</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.002763032913208008</v>
+        <v>0.003592967987060547</v>
       </c>
       <c r="R4" t="n">
-        <v>0.0002617961227112058</v>
+        <v>0.001079738853742046</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>0.009039878845214844, 0.006004810333251953, 0.006154060363769531, 0.005715131759643555, 0.005308866500854492, 0.005414009094238281, 0.00579380989074707</t>
+          <t>0.004926919937133789, 0.004796266555786133, 0.00476384162902832, 0.004468202590942383, 0.0047719478607177734, 0.004295825958251953, 0.004725933074951172</t>
         </is>
       </c>
       <c r="T4" t="n">
-        <v>0.006204366683959961</v>
+        <v>0.004678419658115932</v>
       </c>
       <c r="U4" t="n">
-        <v>0.00579380989074707</v>
+        <v>0.00476384162902832</v>
       </c>
       <c r="V4" t="n">
-        <v>0.001190256639119724</v>
+        <v>0.0002016047749735491</v>
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>0.8888888888888888, 0.8301886792452831, 0.8679245283018868, 0.8113207547169812, 0.8490566037735849, 0.8113207547169812, 0.7735849056603774</t>
+          <t>0.8703703703703703, 0.7924528301886793, 0.8490566037735849, 0.7735849056603774, 0.8301886792452831, 0.7547169811320755, 0.7735849056603774</t>
         </is>
       </c>
       <c r="X4" t="n">
-        <v>0.833183587900569</v>
+        <v>0.8062793251472496</v>
       </c>
       <c r="Y4" t="n">
-        <v>0.8301886792452831</v>
+        <v>0.7924528301886793</v>
       </c>
       <c r="Z4" t="n">
-        <v>0.03601369874946368</v>
+        <v>0.04052673239832488</v>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>0.9166666666666667, 0.8695652173913043, 0.8955223880597014, 0.8484848484848485, 0.8857142857142858, 0.84375, 0.8333333333333333</t>
+          <t>0.9090909090909091, 0.8405797101449276, 0.8857142857142858, 0.8235294117647058, 0.8695652173913043, 0.8115942028985507, 0.8333333333333333</t>
         </is>
       </c>
       <c r="AB4" t="n">
-        <v>0.87043381995002</v>
+        <v>0.8533438671911453</v>
       </c>
       <c r="AC4" t="n">
-        <v>0.8695652173913043</v>
+        <v>0.8405797101449276</v>
       </c>
       <c r="AD4" t="n">
-        <v>0.02821192547334734</v>
+        <v>0.03298049265322964</v>
       </c>
       <c r="AE4" t="inlineStr">
         <is>
-          <t>0.8918918918918919, 0.8823529411764706, 0.9090909090909091, 0.875, 0.8611111111111112, 0.9, 0.7894736842105263</t>
+          <t>0.8333333333333334, 0.8529411764705882, 0.8611111111111112, 0.8235294117647058, 0.8571428571428571, 0.8, 0.7894736842105263</t>
         </is>
       </c>
       <c r="AF4" t="n">
-        <v>0.8727029339258443</v>
+        <v>0.8310759391475887</v>
       </c>
       <c r="AG4" t="n">
-        <v>0.8823529411764706</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="AH4" t="n">
-        <v>0.03702761166157346</v>
+        <v>0.02623572233655289</v>
       </c>
       <c r="AI4" t="inlineStr">
         <is>
-          <t>0.9428571428571428, 0.8571428571428571, 0.8823529411764706, 0.8235294117647058, 0.9117647058823529, 0.7941176470588235, 0.8823529411764706</t>
+          <t>1.0, 0.8285714285714286, 0.9117647058823529, 0.8235294117647058, 0.8823529411764706, 0.8235294117647058, 0.8823529411764706</t>
         </is>
       </c>
       <c r="AJ4" t="n">
-        <v>0.8705882352941176</v>
+        <v>0.8788715486194477</v>
       </c>
       <c r="AK4" t="n">
         <v>0.8823529411764706</v>
       </c>
       <c r="AL4" t="n">
-        <v>0.04696225729259014</v>
+        <v>0.05908094691303778</v>
       </c>
       <c r="AM4" t="inlineStr">
         <is>
-          <t>0.9624060150375939, 0.8849206349206349, 0.9272445820433436, 0.914860681114551, 0.8924148606811145, 0.923374613003096, 0.846749226006192</t>
+          <t>0.9578947368421054, 0.8571428571428572, 0.9504643962848297, 0.8869969040247677, 0.9411764705882353, 0.8126934984520124, 0.8606811145510836</t>
         </is>
       </c>
       <c r="AN4" t="n">
-        <v>0.9074243732580752</v>
+        <v>0.8952928539836987</v>
       </c>
       <c r="AO4" t="n">
-        <v>0.914860681114551</v>
+        <v>0.8869969040247677</v>
       </c>
       <c r="AP4" t="n">
-        <v>0.03409798408896362</v>
+        <v>0.05156559231488393</v>
       </c>
       <c r="AQ4" t="inlineStr">
         <is>
-          <t>0.8962264150943396, 0.896551724137931, 0.8808777429467085, 0.8934169278996865, 0.8934169278996865, 0.890282131661442, 0.8934169278996865</t>
+          <t>0.8113207547169812, 0.8119122257053292, 0.8119122257053292, 0.8150470219435737, 0.8119122257053292, 0.8463949843260188, 0.8181818181818182</t>
         </is>
       </c>
       <c r="AR4" t="n">
-        <v>0.8920269710770686</v>
+        <v>0.8180973223263399</v>
       </c>
       <c r="AS4" t="n">
-        <v>0.8934169278996865</v>
+        <v>0.8119122257053292</v>
       </c>
       <c r="AT4" t="n">
-        <v>0.004946202189722954</v>
+        <v>0.01177623075655056</v>
       </c>
       <c r="AU4" t="inlineStr">
         <is>
-          <t>0.9197080291970803, 0.9193154034229828, 0.9068627450980392, 0.9174757281553398, 0.9170731707317074, 0.9152542372881356, 0.9170731707317074</t>
+          <t>0.8578199052132701, 0.8584905660377359, 0.8584905660377358, 0.8618266978922716, 0.8591549295774649, 0.883054892601432, 0.8632075471698114</t>
         </is>
       </c>
       <c r="AV4" t="n">
-        <v>0.916108926374999</v>
+        <v>0.8631493006471033</v>
       </c>
       <c r="AW4" t="n">
-        <v>0.9170731707317074</v>
+        <v>0.8591549295774649</v>
       </c>
       <c r="AX4" t="n">
-        <v>0.004021106444933429</v>
+        <v>0.008330240384199985</v>
       </c>
       <c r="AY4" t="inlineStr">
         <is>
-          <t>0.9174757281553398, 0.9215686274509803, 0.9158415841584159, 0.9174757281553398, 0.9215686274509803, 0.9130434782608695, 0.9215686274509803</t>
+          <t>0.8341013824884793, 0.8310502283105022, 0.8348623853211009, 0.832579185520362, 0.8318181818181818, 0.8685446009389671, 0.8394495412844036</t>
         </is>
       </c>
       <c r="AZ4" t="n">
-        <v>0.918363200154701</v>
+        <v>0.8389150722402852</v>
       </c>
       <c r="BA4" t="n">
-        <v>0.9174757281553398</v>
+        <v>0.8341013824884793</v>
       </c>
       <c r="BB4" t="n">
-        <v>0.003095099671022134</v>
+        <v>0.01236443975154782</v>
       </c>
       <c r="BC4" t="inlineStr">
         <is>
-          <t>0.9219512195121952, 0.9170731707317074, 0.8980582524271845, 0.9174757281553398, 0.912621359223301, 0.9174757281553398, 0.912621359223301</t>
+          <t>0.8829268292682927, 0.8878048780487805, 0.883495145631068, 0.8932038834951457, 0.8883495145631068, 0.8980582524271845, 0.8883495145631068</t>
         </is>
       </c>
       <c r="BD4" t="n">
-        <v>0.9138966882040529</v>
+        <v>0.888884002570955</v>
       </c>
       <c r="BE4" t="n">
-        <v>0.9170731707317074</v>
+        <v>0.8883495145631068</v>
       </c>
       <c r="BF4" t="n">
-        <v>0.007118321889567089</v>
+        <v>0.00491487231480214</v>
       </c>
       <c r="BG4" t="inlineStr">
         <is>
-          <t>0.9620332398014245, 0.9660034231921266, 0.9626256551250107, 0.9647521264713463, 0.9616805567488615, 0.9633774379242204, 0.967694819142538</t>
+          <t>0.8975825598963955, 0.9145485665382971, 0.9012586992009622, 0.9084328550562764, 0.8984234040725149, 0.9190652117879542, 0.9092061173640348</t>
         </is>
       </c>
       <c r="BH4" t="n">
-        <v>0.9640238940579325</v>
+        <v>0.9069310591309193</v>
       </c>
       <c r="BI4" t="n">
-        <v>0.9633774379242204</v>
+        <v>0.9084328550562764</v>
       </c>
       <c r="BJ4" t="n">
-        <v>0.002061603425119283</v>
+        <v>0.007603060102699606</v>
       </c>
     </row>
     <row r="5">
@@ -1408,216 +1408,216 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>splashing</t>
+          <t>no_fragmentation</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>SVC_splashing_base</t>
+          <t>LogisticRegression_no_fragmentation_base</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>{'estimator': SVC(probability=True), 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Re', 'sedimentation_Stk'), 'log_features': ('relative_roughness',), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sign_sedimentation_Re', 'particle_liquid_density_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
+          <t>{'estimator': LogisticRegression(), 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Re', 'sedimentation_Stk'), 'log_features': ('relative_roughness',), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sign_sedimentation_Re', 'particle_liquid_density_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.84</v>
+        <v>0.8533333333333334</v>
       </c>
       <c r="F5" t="n">
-        <v>0.8214285714285714</v>
+        <v>0.7368421052631579</v>
       </c>
       <c r="G5" t="n">
-        <v>0.9583333333333334</v>
+        <v>0.7</v>
       </c>
       <c r="H5" t="n">
-        <v>0.8846153846153847</v>
+        <v>0.717948717948718</v>
       </c>
       <c r="I5" t="n">
-        <v>0.8958333333333334</v>
+        <v>0.9254545454545455</v>
       </c>
       <c r="J5" t="n">
-        <v>0.8855218855218855</v>
+        <v>0.8754208754208754</v>
       </c>
       <c r="K5" t="n">
-        <v>0.9030612244897959</v>
+        <v>0.8181818181818182</v>
       </c>
       <c r="L5" t="n">
-        <v>0.921875</v>
+        <v>0.6835443037974683</v>
       </c>
       <c r="M5" t="n">
-        <v>0.9123711340206186</v>
+        <v>0.7448275862068965</v>
       </c>
       <c r="N5" t="n">
-        <v>0.9497271825396826</v>
+        <v>0.9316571826733249</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>0.009903192520141602, 0.008059978485107422, 0.007985115051269531, 0.007807016372680664, 0.007658958435058594, 0.00767207145690918, 0.007129192352294922</t>
+          <t>0.0056149959564208984, 0.0036008358001708984, 0.003214120864868164, 0.0038242340087890625, 0.0033888816833496094, 0.0032241344451904297, 0.0030870437622070312</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>0.008030789239065987</v>
+        <v>0.003707749502999442</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.007807016372680664</v>
+        <v>0.003388881683349609</v>
       </c>
       <c r="R5" t="n">
-        <v>0.0008140480879537349</v>
+        <v>0.0008130272595688407</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>0.005318880081176758, 0.004998207092285156, 0.005772113800048828, 0.005053997039794922, 0.005886077880859375, 0.0056569576263427734, 0.005222797393798828</t>
+          <t>0.005347013473510742, 0.004559040069580078, 0.004645824432373047, 0.004475831985473633, 0.004625797271728516, 0.004248857498168945, 0.004568815231323242</t>
         </is>
       </c>
       <c r="T5" t="n">
-        <v>0.005415575844900948</v>
+        <v>0.004638739994594029</v>
       </c>
       <c r="U5" t="n">
-        <v>0.005318880081176758</v>
+        <v>0.004568815231323242</v>
       </c>
       <c r="V5" t="n">
-        <v>0.0003291126931631227</v>
+        <v>0.0003143378426585304</v>
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>0.9074074074074074, 0.7547169811320755, 0.8679245283018868, 0.8679245283018868, 0.8867924528301887, 0.8490566037735849, 0.8490566037735849</t>
+          <t>0.8148148148148148, 0.7924528301886793, 0.9245283018867925, 0.8490566037735849, 0.8490566037735849, 0.8490566037735849, 0.8867924528301887</t>
         </is>
       </c>
       <c r="X5" t="n">
-        <v>0.8546970150743736</v>
+        <v>0.85225117300589</v>
       </c>
       <c r="Y5" t="n">
-        <v>0.8679245283018868</v>
+        <v>0.8490566037735849</v>
       </c>
       <c r="Z5" t="n">
-        <v>0.0450683171313999</v>
+        <v>0.04039982656823135</v>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>0.9333333333333333, 0.8059701492537314, 0.8923076923076922, 0.8923076923076922, 0.90625, 0.8749999999999999, 0.8857142857142858</t>
+          <t>0.5833333333333334, 0.6206896551724138, 0.8571428571428571, 0.7333333333333334, 0.6363636363636364, 0.6666666666666666, 0.7999999999999999</t>
         </is>
       </c>
       <c r="AB5" t="n">
-        <v>0.8844118789881049</v>
+        <v>0.6996470688588915</v>
       </c>
       <c r="AC5" t="n">
-        <v>0.8923076923076922</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="AD5" t="n">
-        <v>0.03632843171013504</v>
+        <v>0.09324779318350135</v>
       </c>
       <c r="AE5" t="inlineStr">
         <is>
-          <t>0.875, 0.84375, 0.9354838709677419, 0.9354838709677419, 0.9666666666666667, 0.9333333333333333, 0.8611111111111112</t>
+          <t>0.7777777777777778, 0.6, 0.8571428571428571, 0.6875, 0.875, 0.8, 0.75</t>
         </is>
       </c>
       <c r="AF5" t="n">
-        <v>0.9072612647209422</v>
+        <v>0.7639172335600907</v>
       </c>
       <c r="AG5" t="n">
-        <v>0.9333333333333333</v>
+        <v>0.7777777777777778</v>
       </c>
       <c r="AH5" t="n">
-        <v>0.04310467686730826</v>
+        <v>0.08898364299549143</v>
       </c>
       <c r="AI5" t="inlineStr">
         <is>
-          <t>1.0, 0.7714285714285715, 0.8529411764705882, 0.8529411764705882, 0.8529411764705882, 0.8235294117647058, 0.9117647058823529</t>
+          <t>0.4666666666666667, 0.6428571428571429, 0.8571428571428571, 0.7857142857142857, 0.5, 0.5714285714285714, 0.8571428571428571</t>
         </is>
       </c>
       <c r="AJ5" t="n">
-        <v>0.8665066026410564</v>
+        <v>0.6687074829931972</v>
       </c>
       <c r="AK5" t="n">
-        <v>0.8529411764705882</v>
+        <v>0.6428571428571429</v>
       </c>
       <c r="AL5" t="n">
-        <v>0.06687698340327823</v>
+        <v>0.1531201700556019</v>
       </c>
       <c r="AM5" t="inlineStr">
         <is>
-          <t>0.9699248120300752, 0.8333333333333334, 0.9705882352941176, 0.9303405572755418, 0.9504643962848297, 0.9055727554179567, 0.8839009287925697</t>
+          <t>0.9418803418803419, 0.8498168498168499, 0.9578754578754578, 0.8864468864468865, 0.9560439560439561, 0.9212454212454212, 0.9633699633699634</t>
         </is>
       </c>
       <c r="AN5" t="n">
-        <v>0.9205892883469178</v>
+        <v>0.9252398395255538</v>
       </c>
       <c r="AO5" t="n">
-        <v>0.9303405572755418</v>
+        <v>0.9418803418803419</v>
       </c>
       <c r="AP5" t="n">
-        <v>0.04645524972067035</v>
+        <v>0.03955875522584676</v>
       </c>
       <c r="AQ5" t="inlineStr">
         <is>
-          <t>0.8710691823899371, 0.8746081504702194, 0.8683385579937304, 0.877742946708464, 0.8746081504702194, 0.877742946708464, 0.890282131661442</t>
+          <t>0.8773584905660378, 0.877742946708464, 0.8589341692789969, 0.877742946708464, 0.8746081504702194, 0.8714733542319749, 0.8526645768025078</t>
         </is>
       </c>
       <c r="AR5" t="n">
-        <v>0.8763417237717823</v>
+        <v>0.8700749478238093</v>
       </c>
       <c r="AS5" t="n">
         <v>0.8746081504702194</v>
       </c>
       <c r="AT5" t="n">
-        <v>0.006504094660230648</v>
+        <v>0.009414197796548299</v>
       </c>
       <c r="AU5" t="inlineStr">
         <is>
-          <t>0.9044289044289044, 0.898477157360406, 0.8934010152284263, 0.9041769041769042, 0.900497512437811, 0.9027431421446385, 0.913151364764268</t>
+          <t>0.7547169811320756, 0.7577639751552795, 0.7133757961783439, 0.751592356687898, 0.7468354430379747, 0.7453416149068324, 0.69281045751634</t>
         </is>
       </c>
       <c r="AV5" t="n">
-        <v>0.902410857220194</v>
+        <v>0.737490946373535</v>
       </c>
       <c r="AW5" t="n">
-        <v>0.9027431421446385</v>
+        <v>0.7468354430379747</v>
       </c>
       <c r="AX5" t="n">
-        <v>0.005643865032366699</v>
+        <v>0.02278289116899502</v>
       </c>
       <c r="AY5" t="inlineStr">
         <is>
-          <t>0.8660714285714286, 0.9365079365079365, 0.9361702127659575, 0.9154228855721394, 0.923469387755102, 0.9282051282051282, 0.934010152284264</t>
+          <t>0.8, 0.8026315789473685, 0.7777777777777778, 0.8194444444444444, 0.8082191780821918, 0.7894736842105263, 0.7794117647058824</t>
         </is>
       </c>
       <c r="AZ5" t="n">
-        <v>0.9199795902374223</v>
+        <v>0.7967083468811701</v>
       </c>
       <c r="BA5" t="n">
-        <v>0.9282051282051282</v>
+        <v>0.8</v>
       </c>
       <c r="BB5" t="n">
-        <v>0.02311113143313012</v>
+        <v>0.014168514244079</v>
       </c>
       <c r="BC5" t="inlineStr">
         <is>
-          <t>0.9463414634146341, 0.8634146341463415, 0.8543689320388349, 0.8932038834951457, 0.8786407766990292, 0.8786407766990292, 0.8932038834951457</t>
+          <t>0.7142857142857143, 0.7176470588235294, 0.6588235294117647, 0.6941176470588235, 0.6941176470588235, 0.7058823529411765, 0.6235294117647059</t>
         </is>
       </c>
       <c r="BD5" t="n">
-        <v>0.8868306214268801</v>
+        <v>0.6869147659063627</v>
       </c>
       <c r="BE5" t="n">
-        <v>0.8786407766990292</v>
+        <v>0.6941176470588235</v>
       </c>
       <c r="BF5" t="n">
-        <v>0.02766894624575639</v>
+        <v>0.03154134629409137</v>
       </c>
       <c r="BG5" t="inlineStr">
         <is>
-          <t>0.9373839844593136, 0.9515618314077879, 0.9390196752298307, 0.9434444539908927, 0.936485093221067, 0.9465589827304751, 0.9486854540768108</t>
+          <t>0.9281135531135531, 0.9407742584213172, 0.9262443438914028, 0.9370035193564605, 0.9277526395173454, 0.9327300150829563, 0.9243841126194067</t>
         </is>
       </c>
       <c r="BH5" t="n">
-        <v>0.9433056393023111</v>
+        <v>0.9310003488574919</v>
       </c>
       <c r="BI5" t="n">
-        <v>0.9434444539908927</v>
+        <v>0.9281135531135531</v>
       </c>
       <c r="BJ5" t="n">
-        <v>0.005446702292296702</v>
+        <v>0.005604009792409489</v>
       </c>
     </row>
     <row r="6">
@@ -1633,211 +1633,211 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>CatBoostClassifier_splashing_base</t>
+          <t>KNeighborsClassifier_splashing_base</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>{'estimator': &lt;catboost.core.CatBoostClassifier object at 0x16a90c850&gt;, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Re', 'sedimentation_Stk'), 'log_features': ('relative_roughness',), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sign_sedimentation_Re', 'particle_liquid_density_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
+          <t>{'estimator': KNeighborsClassifier(), 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Re', 'sedimentation_Stk'), 'log_features': ('relative_roughness',), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sign_sedimentation_Re', 'particle_liquid_density_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.88</v>
+        <v>0.8133333333333334</v>
       </c>
       <c r="F6" t="n">
-        <v>0.8679245283018868</v>
+        <v>0.8269230769230769</v>
       </c>
       <c r="G6" t="n">
-        <v>0.9583333333333334</v>
+        <v>0.8958333333333334</v>
       </c>
       <c r="H6" t="n">
-        <v>0.910891089108911</v>
+        <v>0.86</v>
       </c>
       <c r="I6" t="n">
-        <v>0.9467592592592593</v>
+        <v>0.880787037037037</v>
       </c>
       <c r="J6" t="n">
-        <v>0.9966329966329966</v>
+        <v>0.9158249158249159</v>
       </c>
       <c r="K6" t="n">
-        <v>0.9948186528497409</v>
+        <v>0.9282051282051282</v>
       </c>
       <c r="L6" t="n">
-        <v>1</v>
+        <v>0.9427083333333334</v>
       </c>
       <c r="M6" t="n">
-        <v>0.9974025974025974</v>
+        <v>0.9354005167958657</v>
       </c>
       <c r="N6" t="n">
-        <v>0.9988839285714286</v>
+        <v>0.9661954365079365</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>0.6268463134765625, 0.5556938648223877, 0.5717732906341553, 0.5568299293518066, 0.5568921566009521, 0.5782740116119385, 0.5516190528869629</t>
+          <t>0.0038111209869384766, 0.0026099681854248047, 0.002904653549194336, 0.0025260448455810547, 0.002437114715576172, 0.0027048587799072266, 0.0025479793548583984</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>0.5711326599121094</v>
+        <v>0.00279167720249721</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.5568921566009521</v>
+        <v>0.002609968185424805</v>
       </c>
       <c r="R6" t="n">
-        <v>0.02444211176962691</v>
+        <v>0.00043887008117464</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>0.005814075469970703, 0.0051081180572509766, 0.005595684051513672, 0.0057680606842041016, 0.00548100471496582, 0.005693197250366211, 0.00574803352355957</t>
+          <t>0.03403282165527344, 0.006546974182128906, 0.005788326263427734, 0.005702018737792969, 0.005563974380493164, 0.0058040618896484375, 0.005694150924682617</t>
         </is>
       </c>
       <c r="T6" t="n">
-        <v>0.005601167678833008</v>
+        <v>0.009876046861921037</v>
       </c>
       <c r="U6" t="n">
-        <v>0.005693197250366211</v>
+        <v>0.005788326263427734</v>
       </c>
       <c r="V6" t="n">
-        <v>0.0002270271093154386</v>
+        <v>0.009866449268142702</v>
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>0.9629629629629629, 0.8679245283018868, 0.9056603773584906, 0.8301886792452831, 0.8867924528301887, 0.8867924528301887, 0.8679245283018868</t>
+          <t>0.8888888888888888, 0.8301886792452831, 0.8679245283018868, 0.8113207547169812, 0.8490566037735849, 0.8113207547169812, 0.7735849056603774</t>
         </is>
       </c>
       <c r="X6" t="n">
-        <v>0.8868922831186982</v>
+        <v>0.833183587900569</v>
       </c>
       <c r="Y6" t="n">
-        <v>0.8867924528301887</v>
+        <v>0.8301886792452831</v>
       </c>
       <c r="Z6" t="n">
-        <v>0.03793577234399872</v>
+        <v>0.03601369874946368</v>
       </c>
       <c r="AA6" t="inlineStr">
         <is>
-          <t>0.9722222222222222, 0.8985507246376812, 0.9275362318840579, 0.8656716417910447, 0.9090909090909091, 0.9090909090909091, 0.8985507246376812</t>
+          <t>0.9166666666666667, 0.8695652173913043, 0.8955223880597014, 0.8484848484848485, 0.8857142857142858, 0.84375, 0.8333333333333333</t>
         </is>
       </c>
       <c r="AB6" t="n">
-        <v>0.9115304804792151</v>
+        <v>0.87043381995002</v>
       </c>
       <c r="AC6" t="n">
-        <v>0.9090909090909091</v>
+        <v>0.8695652173913043</v>
       </c>
       <c r="AD6" t="n">
-        <v>0.03021720375687164</v>
+        <v>0.02821192547334734</v>
       </c>
       <c r="AE6" t="inlineStr">
         <is>
-          <t>0.9459459459459459, 0.9117647058823529, 0.9142857142857143, 0.8787878787878788, 0.9375, 0.9375, 0.8857142857142857</t>
+          <t>0.8918918918918919, 0.8823529411764706, 0.9090909090909091, 0.875, 0.8611111111111112, 0.9, 0.7894736842105263</t>
         </is>
       </c>
       <c r="AF6" t="n">
-        <v>0.915928361516597</v>
+        <v>0.8727029339258443</v>
       </c>
       <c r="AG6" t="n">
-        <v>0.9142857142857143</v>
+        <v>0.8823529411764706</v>
       </c>
       <c r="AH6" t="n">
-        <v>0.02433124593359062</v>
+        <v>0.03702761166157346</v>
       </c>
       <c r="AI6" t="inlineStr">
         <is>
-          <t>1.0, 0.8857142857142857, 0.9411764705882353, 0.8529411764705882, 0.8823529411764706, 0.8823529411764706, 0.9117647058823529</t>
+          <t>0.9428571428571428, 0.8571428571428571, 0.8823529411764706, 0.8235294117647058, 0.9117647058823529, 0.7941176470588235, 0.8823529411764706</t>
         </is>
       </c>
       <c r="AJ6" t="n">
-        <v>0.9080432172869148</v>
+        <v>0.8705882352941176</v>
       </c>
       <c r="AK6" t="n">
-        <v>0.8857142857142857</v>
+        <v>0.8823529411764706</v>
       </c>
       <c r="AL6" t="n">
-        <v>0.04539117047431458</v>
+        <v>0.04696225729259014</v>
       </c>
       <c r="AM6" t="inlineStr">
         <is>
-          <t>1.0, 0.9396825396825397, 0.9736842105263158, 0.93343653250774, 0.9705882352941176, 0.9504643962848298, 0.9226006191950464</t>
+          <t>0.9624060150375939, 0.8849206349206349, 0.9272445820433436, 0.914860681114551, 0.8924148606811145, 0.923374613003096, 0.846749226006192</t>
         </is>
       </c>
       <c r="AN6" t="n">
-        <v>0.9557795047843699</v>
+        <v>0.9074243732580752</v>
       </c>
       <c r="AO6" t="n">
-        <v>0.9504643962848298</v>
+        <v>0.914860681114551</v>
       </c>
       <c r="AP6" t="n">
-        <v>0.02502210082274886</v>
+        <v>0.03409798408896362</v>
       </c>
       <c r="AQ6" t="inlineStr">
         <is>
-          <t>0.9874213836477987, 0.9937304075235109, 0.9905956112852664, 0.9905956112852664, 0.987460815047022, 0.9937304075235109, 0.9905956112852664</t>
+          <t>0.8962264150943396, 0.896551724137931, 0.8808777429467085, 0.8934169278996865, 0.8934169278996865, 0.890282131661442, 0.8934169278996865</t>
         </is>
       </c>
       <c r="AR6" t="n">
-        <v>0.9905899782282346</v>
+        <v>0.8920269710770686</v>
       </c>
       <c r="AS6" t="n">
-        <v>0.9905956112852664</v>
+        <v>0.8934169278996865</v>
       </c>
       <c r="AT6" t="n">
-        <v>0.002377163415894737</v>
+        <v>0.004946202189722954</v>
       </c>
       <c r="AU6" t="inlineStr">
         <is>
-          <t>0.9902912621359223, 0.9951456310679612, 0.9927360774818401, 0.9927007299270073, 0.9902912621359223, 0.9951456310679612, 0.9927360774818401</t>
+          <t>0.9197080291970803, 0.9193154034229828, 0.9068627450980392, 0.9174757281553398, 0.9170731707317074, 0.9152542372881356, 0.9170731707317074</t>
         </is>
       </c>
       <c r="AV6" t="n">
-        <v>0.9927209530426364</v>
+        <v>0.916108926374999</v>
       </c>
       <c r="AW6" t="n">
-        <v>0.9927360774818401</v>
+        <v>0.9170731707317074</v>
       </c>
       <c r="AX6" t="n">
-        <v>0.001834813705181454</v>
+        <v>0.004021106444933429</v>
       </c>
       <c r="AY6" t="inlineStr">
         <is>
-          <t>0.9855072463768116, 0.9903381642512077, 0.9903381642512077, 0.9951219512195122, 0.9902912621359223, 0.9951456310679612, 0.9903381642512077</t>
+          <t>0.9174757281553398, 0.9215686274509803, 0.9158415841584159, 0.9174757281553398, 0.9215686274509803, 0.9130434782608695, 0.9215686274509803</t>
         </is>
       </c>
       <c r="AZ6" t="n">
-        <v>0.9910115119362616</v>
+        <v>0.918363200154701</v>
       </c>
       <c r="BA6" t="n">
-        <v>0.9903381642512077</v>
+        <v>0.9174757281553398</v>
       </c>
       <c r="BB6" t="n">
-        <v>0.003074376650758704</v>
+        <v>0.003095099671022134</v>
       </c>
       <c r="BC6" t="inlineStr">
         <is>
-          <t>0.9951219512195122, 1.0, 0.9951456310679612, 0.9902912621359223, 0.9902912621359223, 0.9951456310679612, 0.9951456310679612</t>
+          <t>0.9219512195121952, 0.9170731707317074, 0.8980582524271845, 0.9174757281553398, 0.912621359223301, 0.9174757281553398, 0.912621359223301</t>
         </is>
       </c>
       <c r="BD6" t="n">
-        <v>0.994448766956463</v>
+        <v>0.9138966882040529</v>
       </c>
       <c r="BE6" t="n">
-        <v>0.9951456310679612</v>
+        <v>0.9170731707317074</v>
       </c>
       <c r="BF6" t="n">
-        <v>0.003100597103577546</v>
+        <v>0.007118321889567089</v>
       </c>
       <c r="BG6" t="inlineStr">
         <is>
-          <t>0.9979063241959854, 0.9986307231493367, 0.9984319958759343, 0.9985179139101297, 0.9984319958759343, 0.9999570409829023, 0.9984319958759343</t>
+          <t>0.9620332398014245, 0.9660034231921266, 0.9626256551250107, 0.9647521264713463, 0.9616805567488615, 0.9633774379242204, 0.967694819142538</t>
         </is>
       </c>
       <c r="BH6" t="n">
-        <v>0.9986154271237367</v>
+        <v>0.9640238940579325</v>
       </c>
       <c r="BI6" t="n">
-        <v>0.9984319958759343</v>
+        <v>0.9633774379242204</v>
       </c>
       <c r="BJ6" t="n">
-        <v>0.0005871770933261723</v>
+        <v>0.002061603425119283</v>
       </c>
     </row>
     <row r="7">
@@ -1853,211 +1853,211 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>CatBoostClassifier_no_fragmentation_base</t>
+          <t>KNeighborsClassifier_no_fragmentation_base</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>{'estimator': &lt;catboost.core.CatBoostClassifier object at 0x14932f850&gt;, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Re', 'sedimentation_Stk'), 'log_features': ('relative_roughness',), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sign_sedimentation_Re', 'particle_liquid_density_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
+          <t>{'estimator': KNeighborsClassifier(), 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Re', 'sedimentation_Stk'), 'log_features': ('relative_roughness',), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sign_sedimentation_Re', 'particle_liquid_density_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.9066666666666666</v>
+        <v>0.88</v>
       </c>
       <c r="F7" t="n">
-        <v>0.8095238095238095</v>
+        <v>0.7894736842105263</v>
       </c>
       <c r="G7" t="n">
-        <v>0.85</v>
+        <v>0.75</v>
       </c>
       <c r="H7" t="n">
-        <v>0.8292682926829269</v>
+        <v>0.7692307692307692</v>
       </c>
       <c r="I7" t="n">
-        <v>0.9781818181818182</v>
+        <v>0.9495454545454545</v>
       </c>
       <c r="J7" t="n">
-        <v>1</v>
+        <v>0.8922558922558923</v>
       </c>
       <c r="K7" t="n">
-        <v>1</v>
+        <v>0.8309859154929577</v>
       </c>
       <c r="L7" t="n">
-        <v>1</v>
+        <v>0.7468354430379747</v>
       </c>
       <c r="M7" t="n">
-        <v>1</v>
+        <v>0.7866666666666666</v>
       </c>
       <c r="N7" t="n">
-        <v>1</v>
+        <v>0.9578155847172223</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>0.5788400173187256, 0.5555107593536377, 0.5553131103515625, 0.5709900856018066, 0.5529239177703857, 0.547766923904419, 0.5719518661499023</t>
+          <t>0.013814210891723633, 0.0026061534881591797, 0.0027799606323242188, 0.0025517940521240234, 0.0026178359985351562, 0.0024237632751464844, 0.0025777816772460938</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>0.5618995257786342</v>
+        <v>0.004195928573608398</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.5555107593536377</v>
+        <v>0.00260615348815918</v>
       </c>
       <c r="R7" t="n">
-        <v>0.01092282837470189</v>
+        <v>0.003927853439721885</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>0.005773782730102539, 0.005828142166137695, 0.0057828426361083984, 0.0059468746185302734, 0.005060911178588867, 0.005029201507568359, 0.005877971649169922</t>
+          <t>0.03016972541809082, 0.00638580322265625, 0.006022214889526367, 0.005488157272338867, 0.005755186080932617, 0.00590205192565918, 0.005587339401245117</t>
         </is>
       </c>
       <c r="T7" t="n">
-        <v>0.005614246640886579</v>
+        <v>0.009330068315778459</v>
       </c>
       <c r="U7" t="n">
-        <v>0.005782842636108398</v>
+        <v>0.00590205192565918</v>
       </c>
       <c r="V7" t="n">
-        <v>0.0003641581019381846</v>
+        <v>0.008512186884758929</v>
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>0.9074074074074074, 0.8301886792452831, 0.9622641509433962, 0.8867924528301887, 0.8867924528301887, 0.9433962264150944, 0.8867924528301887</t>
+          <t>0.8888888888888888, 0.7735849056603774, 0.8679245283018868, 0.8301886792452831, 0.8490566037735849, 0.8490566037735849, 0.8867924528301887</t>
         </is>
       </c>
       <c r="X7" t="n">
-        <v>0.9005191175002497</v>
+        <v>0.8493560946391135</v>
       </c>
       <c r="Y7" t="n">
-        <v>0.8867924528301887</v>
+        <v>0.8490566037735849</v>
       </c>
       <c r="Z7" t="n">
-        <v>0.04001781509646558</v>
+        <v>0.03667999015847824</v>
       </c>
       <c r="AA7" t="inlineStr">
         <is>
-          <t>0.8148148148148148, 0.7096774193548386, 0.9285714285714286, 0.7999999999999999, 0.7272727272727273, 0.888888888888889, 0.7857142857142857</t>
+          <t>0.8000000000000002, 0.5714285714285714, 0.7200000000000001, 0.6666666666666666, 0.6923076923076924, 0.6666666666666666, 0.8125000000000001</t>
         </is>
       </c>
       <c r="AB7" t="n">
-        <v>0.8078485092309977</v>
+        <v>0.7042242281527996</v>
       </c>
       <c r="AC7" t="n">
-        <v>0.7999999999999999</v>
+        <v>0.6923076923076924</v>
       </c>
       <c r="AD7" t="n">
-        <v>0.07355429314085414</v>
+        <v>0.07722263485750151</v>
       </c>
       <c r="AE7" t="inlineStr">
         <is>
-          <t>0.9166666666666666, 0.6470588235294118, 0.9285714285714286, 0.75, 1.0, 0.9230769230769231, 0.7857142857142857</t>
+          <t>0.8, 0.5714285714285714, 0.8181818181818182, 0.6923076923076923, 0.75, 0.8, 0.7222222222222222</t>
         </is>
       </c>
       <c r="AF7" t="n">
-        <v>0.8501554467941023</v>
+        <v>0.7363057577343292</v>
       </c>
       <c r="AG7" t="n">
-        <v>0.9166666666666666</v>
+        <v>0.75</v>
       </c>
       <c r="AH7" t="n">
-        <v>0.1157434080450252</v>
+        <v>0.07957368269107451</v>
       </c>
       <c r="AI7" t="inlineStr">
         <is>
-          <t>0.7333333333333333, 0.7857142857142857, 0.9285714285714286, 0.8571428571428571, 0.5714285714285714, 0.8571428571428571, 0.7857142857142857</t>
+          <t>0.8, 0.5714285714285714, 0.6428571428571429, 0.6428571428571429, 0.6428571428571429, 0.5714285714285714, 0.9285714285714286</t>
         </is>
       </c>
       <c r="AJ7" t="n">
-        <v>0.7884353741496598</v>
+        <v>0.6857142857142857</v>
       </c>
       <c r="AK7" t="n">
-        <v>0.7857142857142857</v>
+        <v>0.6428571428571429</v>
       </c>
       <c r="AL7" t="n">
-        <v>0.106383770352787</v>
+        <v>0.1216983797214333</v>
       </c>
       <c r="AM7" t="inlineStr">
         <is>
-          <t>0.9641025641025642, 0.9084249084249085, 0.9908424908424909, 0.9084249084249084, 0.989010989010989, 0.9688644688644689, 0.9761904761904763</t>
+          <t>0.9444444444444444, 0.8772893772893773, 0.9487179487179488, 0.8946886446886448, 0.9010989010989011, 0.903846153846154, 0.9468864468864469</t>
         </is>
       </c>
       <c r="AN7" t="n">
-        <v>0.9579801151229724</v>
+        <v>0.9167102738531312</v>
       </c>
       <c r="AO7" t="n">
-        <v>0.9688644688644689</v>
+        <v>0.903846153846154</v>
       </c>
       <c r="AP7" t="n">
-        <v>0.03260556193142309</v>
+        <v>0.02713046960614661</v>
       </c>
       <c r="AQ7" t="inlineStr">
         <is>
-          <t>0.9937106918238994, 1.0, 0.9968652037617555, 0.9968652037617555, 0.9937304075235109, 0.9968652037617555, 0.9905956112852664</t>
+          <t>0.89937106918239, 0.9059561128526645, 0.9122257053291536, 0.9028213166144201, 0.9059561128526645, 0.9028213166144201, 0.9028213166144201</t>
         </is>
       </c>
       <c r="AR7" t="n">
-        <v>0.9955189031311348</v>
+        <v>0.9045675642943048</v>
       </c>
       <c r="AS7" t="n">
-        <v>0.9968652037617555</v>
+        <v>0.9028213166144201</v>
       </c>
       <c r="AT7" t="n">
-        <v>0.002834102341681714</v>
+        <v>0.003754139860286498</v>
       </c>
       <c r="AU7" t="inlineStr">
         <is>
-          <t>0.9880952380952381, 1.0, 0.9941520467836257, 0.9940828402366864, 0.9882352941176471, 0.9941520467836257, 0.9822485207100591</t>
+          <t>0.8117647058823529, 0.8255813953488372, 0.829268292682927, 0.8165680473372781, 0.8255813953488372, 0.822857142857143, 0.8143712574850299</t>
         </is>
       </c>
       <c r="AV7" t="n">
-        <v>0.9915665695324117</v>
+        <v>0.820856033848915</v>
       </c>
       <c r="AW7" t="n">
-        <v>0.9940828402366864</v>
+        <v>0.822857142857143</v>
       </c>
       <c r="AX7" t="n">
-        <v>0.005355868938882427</v>
+        <v>0.00612395781888402</v>
       </c>
       <c r="AY7" t="inlineStr">
         <is>
-          <t>0.9880952380952381, 1.0, 0.9883720930232558, 1.0, 0.9882352941176471, 0.9883720930232558, 0.9880952380952381</t>
+          <t>0.8023255813953488, 0.8160919540229885, 0.8607594936708861, 0.8214285714285714, 0.8160919540229885, 0.8, 0.8292682926829268</t>
         </is>
       </c>
       <c r="AZ7" t="n">
-        <v>0.9915957080506621</v>
+        <v>0.8208522638891014</v>
       </c>
       <c r="BA7" t="n">
-        <v>0.9883720930232558</v>
+        <v>0.8160919540229885</v>
       </c>
       <c r="BB7" t="n">
-        <v>0.005316370884193521</v>
+        <v>0.01884949652022786</v>
       </c>
       <c r="BC7" t="inlineStr">
         <is>
-          <t>0.9880952380952381, 1.0, 1.0, 0.9882352941176471, 0.9882352941176471, 1.0, 0.9764705882352941</t>
+          <t>0.8214285714285714, 0.8352941176470589, 0.8, 0.8117647058823529, 0.8352941176470589, 0.8470588235294118, 0.8</t>
         </is>
       </c>
       <c r="BD7" t="n">
-        <v>0.991576630652261</v>
+        <v>0.821548619447779</v>
       </c>
       <c r="BE7" t="n">
-        <v>0.9882352941176471</v>
+        <v>0.8214285714285714</v>
       </c>
       <c r="BF7" t="n">
-        <v>0.008241888868281137</v>
+        <v>0.01712589238622703</v>
       </c>
       <c r="BG7" t="inlineStr">
         <is>
-          <t>0.999949124949125, 1.0, 0.9998994469582705, 1.0, 0.9998491704374057, 0.9998994469582704, 0.9998994469582704</t>
+          <t>0.9602920227920229, 0.9680744092508797, 0.9614379084967319, 0.9640020110608346, 0.9654600301659125, 0.9612116641528407, 0.9623428858722977</t>
         </is>
       </c>
       <c r="BH7" t="n">
-        <v>0.9999280908944774</v>
+        <v>0.9632601331130743</v>
       </c>
       <c r="BI7" t="n">
-        <v>0.9998994469582705</v>
+        <v>0.9623428858722977</v>
       </c>
       <c r="BJ7" t="n">
-        <v>5.274484965747932e-05</v>
+        <v>0.002556083322909469</v>
       </c>
     </row>
     <row r="8">
@@ -2073,10 +2073,890 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
+          <t>SVC_splashing_base</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>{'estimator': SVC(probability=True), 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Re', 'sedimentation_Stk'), 'log_features': ('relative_roughness',), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sign_sedimentation_Re', 'particle_liquid_density_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.8214285714285714</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.9583333333333334</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.8846153846153847</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.8958333333333334</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.8855218855218855</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.9030612244897959</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.921875</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.9123711340206186</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0.9497271825396826</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>0.009201288223266602, 0.007555246353149414, 0.00789785385131836, 0.0074770450592041016, 0.007703065872192383, 0.007289886474609375, 0.007388114929199219</t>
+        </is>
+      </c>
+      <c r="P8" t="n">
+        <v>0.007787500108991351</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0.007555246353149414</v>
+      </c>
+      <c r="R8" t="n">
+        <v>0.0006065777440287308</v>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>0.0058438777923583984, 0.005338907241821289, 0.005315065383911133, 0.005349874496459961, 0.005384206771850586, 0.005096912384033203, 0.005342006683349609</t>
+        </is>
+      </c>
+      <c r="T8" t="n">
+        <v>0.005381550107683454</v>
+      </c>
+      <c r="U8" t="n">
+        <v>0.005342006683349609</v>
+      </c>
+      <c r="V8" t="n">
+        <v>0.0002082506178569593</v>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>0.9074074074074074, 0.7547169811320755, 0.8679245283018868, 0.8679245283018868, 0.8867924528301887, 0.8490566037735849, 0.8490566037735849</t>
+        </is>
+      </c>
+      <c r="X8" t="n">
+        <v>0.8546970150743736</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>0.8679245283018868</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>0.0450683171313999</v>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>0.9333333333333333, 0.8059701492537314, 0.8923076923076922, 0.8923076923076922, 0.90625, 0.8749999999999999, 0.8857142857142858</t>
+        </is>
+      </c>
+      <c r="AB8" t="n">
+        <v>0.8844118789881049</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>0.8923076923076922</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>0.03632843171013504</v>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>0.875, 0.84375, 0.9354838709677419, 0.9354838709677419, 0.9666666666666667, 0.9333333333333333, 0.8611111111111112</t>
+        </is>
+      </c>
+      <c r="AF8" t="n">
+        <v>0.9072612647209422</v>
+      </c>
+      <c r="AG8" t="n">
+        <v>0.9333333333333333</v>
+      </c>
+      <c r="AH8" t="n">
+        <v>0.04310467686730826</v>
+      </c>
+      <c r="AI8" t="inlineStr">
+        <is>
+          <t>1.0, 0.7714285714285715, 0.8529411764705882, 0.8529411764705882, 0.8529411764705882, 0.8235294117647058, 0.9117647058823529</t>
+        </is>
+      </c>
+      <c r="AJ8" t="n">
+        <v>0.8665066026410564</v>
+      </c>
+      <c r="AK8" t="n">
+        <v>0.8529411764705882</v>
+      </c>
+      <c r="AL8" t="n">
+        <v>0.06687698340327823</v>
+      </c>
+      <c r="AM8" t="inlineStr">
+        <is>
+          <t>0.9699248120300752, 0.8317460317460317, 0.9705882352941176, 0.9303405572755418, 0.9504643962848297, 0.9055727554179567, 0.8839009287925697</t>
+        </is>
+      </c>
+      <c r="AN8" t="n">
+        <v>0.9203625309773033</v>
+      </c>
+      <c r="AO8" t="n">
+        <v>0.9303405572755418</v>
+      </c>
+      <c r="AP8" t="n">
+        <v>0.04688251914863425</v>
+      </c>
+      <c r="AQ8" t="inlineStr">
+        <is>
+          <t>0.8710691823899371, 0.8746081504702194, 0.8683385579937304, 0.877742946708464, 0.8746081504702194, 0.877742946708464, 0.890282131661442</t>
+        </is>
+      </c>
+      <c r="AR8" t="n">
+        <v>0.8763417237717823</v>
+      </c>
+      <c r="AS8" t="n">
+        <v>0.8746081504702194</v>
+      </c>
+      <c r="AT8" t="n">
+        <v>0.006504094660230648</v>
+      </c>
+      <c r="AU8" t="inlineStr">
+        <is>
+          <t>0.9044289044289044, 0.898477157360406, 0.8934010152284263, 0.9041769041769042, 0.900497512437811, 0.9027431421446385, 0.913151364764268</t>
+        </is>
+      </c>
+      <c r="AV8" t="n">
+        <v>0.902410857220194</v>
+      </c>
+      <c r="AW8" t="n">
+        <v>0.9027431421446385</v>
+      </c>
+      <c r="AX8" t="n">
+        <v>0.005643865032366699</v>
+      </c>
+      <c r="AY8" t="inlineStr">
+        <is>
+          <t>0.8660714285714286, 0.9365079365079365, 0.9361702127659575, 0.9154228855721394, 0.923469387755102, 0.9282051282051282, 0.934010152284264</t>
+        </is>
+      </c>
+      <c r="AZ8" t="n">
+        <v>0.9199795902374223</v>
+      </c>
+      <c r="BA8" t="n">
+        <v>0.9282051282051282</v>
+      </c>
+      <c r="BB8" t="n">
+        <v>0.02311113143313012</v>
+      </c>
+      <c r="BC8" t="inlineStr">
+        <is>
+          <t>0.9463414634146341, 0.8634146341463415, 0.8543689320388349, 0.8932038834951457, 0.8786407766990292, 0.8786407766990292, 0.8932038834951457</t>
+        </is>
+      </c>
+      <c r="BD8" t="n">
+        <v>0.8868306214268801</v>
+      </c>
+      <c r="BE8" t="n">
+        <v>0.8786407766990292</v>
+      </c>
+      <c r="BF8" t="n">
+        <v>0.02766894624575639</v>
+      </c>
+      <c r="BG8" t="inlineStr">
+        <is>
+          <t>0.9372976473127563, 0.9515618314077879, 0.9390196752298307, 0.9434444539908927, 0.9364850932210671, 0.9465589827304751, 0.9486854540768108</t>
+        </is>
+      </c>
+      <c r="BH8" t="n">
+        <v>0.9432933054242316</v>
+      </c>
+      <c r="BI8" t="n">
+        <v>0.9434444539908927</v>
+      </c>
+      <c r="BJ8" t="n">
+        <v>0.005460178801644405</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>no_fragmentation</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>SVC_no_fragmentation_base</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>{'estimator': SVC(probability=True), 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Re', 'sedimentation_Stk'), 'log_features': ('relative_roughness',), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sign_sedimentation_Re', 'particle_liquid_density_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.7222222222222222</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.6842105263157895</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.9281818181818182</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.8888888888888888</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.8194444444444444</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.7468354430379747</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0.781456953642384</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0.9624898385785624</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>0.008935928344726562, 0.006967067718505859, 0.007485151290893555, 0.0068700313568115234, 0.007204771041870117, 0.006928920745849609, 0.006788015365600586</t>
+        </is>
+      </c>
+      <c r="P9" t="n">
+        <v>0.007311412266322545</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0.006967067718505859</v>
+      </c>
+      <c r="R9" t="n">
+        <v>0.0006983904395327948</v>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>0.005445241928100586, 0.005352973937988281, 0.0054247379302978516, 0.004976749420166016, 0.004960060119628906, 0.005160093307495117, 0.005090951919555664</t>
+        </is>
+      </c>
+      <c r="T9" t="n">
+        <v>0.005201544080461774</v>
+      </c>
+      <c r="U9" t="n">
+        <v>0.005160093307495117</v>
+      </c>
+      <c r="V9" t="n">
+        <v>0.0001908369058981177</v>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>0.8333333333333334, 0.7358490566037735, 0.8679245283018868, 0.8867924528301887, 0.8867924528301887, 0.8679245283018868, 0.8301886792452831</t>
+        </is>
+      </c>
+      <c r="X9" t="n">
+        <v>0.844115004492363</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>0.8679245283018868</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>0.04900177617977858</v>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>0.6666666666666665, 0.5, 0.6956521739130435, 0.7857142857142857, 0.75, 0.7200000000000001, 0.689655172413793</t>
+        </is>
+      </c>
+      <c r="AB9" t="n">
+        <v>0.6868126141011126</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>0.6956521739130435</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>0.08474045998405863</v>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>0.75, 0.5, 0.8888888888888888, 0.7857142857142857, 0.9, 0.8181818181818182, 0.6666666666666666</t>
+        </is>
+      </c>
+      <c r="AF9" t="n">
+        <v>0.75849309420738</v>
+      </c>
+      <c r="AG9" t="n">
+        <v>0.7857142857142857</v>
+      </c>
+      <c r="AH9" t="n">
+        <v>0.1290923865694569</v>
+      </c>
+      <c r="AI9" t="inlineStr">
+        <is>
+          <t>0.6, 0.5, 0.5714285714285714, 0.7857142857142857, 0.6428571428571429, 0.6428571428571429, 0.7142857142857143</t>
+        </is>
+      </c>
+      <c r="AJ9" t="n">
+        <v>0.636734693877551</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>0.6428571428571429</v>
+      </c>
+      <c r="AL9" t="n">
+        <v>0.08668065543508287</v>
+      </c>
+      <c r="AM9" t="inlineStr">
+        <is>
+          <t>0.9384615384615385, 0.8626373626373627, 0.9725274725274725, 0.9267399267399268, 0.9523809523809523, 0.9432234432234433, 0.9413919413919414</t>
+        </is>
+      </c>
+      <c r="AN9" t="n">
+        <v>0.9339089481946626</v>
+      </c>
+      <c r="AO9" t="n">
+        <v>0.9413919413919414</v>
+      </c>
+      <c r="AP9" t="n">
+        <v>0.03190862001703766</v>
+      </c>
+      <c r="AQ9" t="inlineStr">
+        <is>
+          <t>0.8805031446540881, 0.9028213166144201, 0.8683385579937304, 0.8840125391849529, 0.8808777429467085, 0.8840125391849529, 0.8746081504702194</t>
+        </is>
+      </c>
+      <c r="AR9" t="n">
+        <v>0.8821677130070105</v>
+      </c>
+      <c r="AS9" t="n">
+        <v>0.8808777429467085</v>
+      </c>
+      <c r="AT9" t="n">
+        <v>0.009900977108437748</v>
+      </c>
+      <c r="AU9" t="inlineStr">
+        <is>
+          <t>0.7532467532467533, 0.8248587570621468, 0.7272727272727274, 0.7836257309941521, 0.7790697674418604, 0.7784431137724551, 0.7368421052631579</t>
+        </is>
+      </c>
+      <c r="AV9" t="n">
+        <v>0.7690512792933218</v>
+      </c>
+      <c r="AW9" t="n">
+        <v>0.7784431137724551</v>
+      </c>
+      <c r="AX9" t="n">
+        <v>0.03058507390673511</v>
+      </c>
+      <c r="AY9" t="inlineStr">
+        <is>
+          <t>0.8285714285714286, 0.7934782608695652, 0.8115942028985508, 0.7790697674418605, 0.7701149425287356, 0.7926829268292683, 0.835820895522388</t>
+        </is>
+      </c>
+      <c r="AZ9" t="n">
+        <v>0.8016189178088281</v>
+      </c>
+      <c r="BA9" t="n">
+        <v>0.7934782608695652</v>
+      </c>
+      <c r="BB9" t="n">
+        <v>0.02281229712069013</v>
+      </c>
+      <c r="BC9" t="inlineStr">
+        <is>
+          <t>0.6904761904761905, 0.8588235294117647, 0.6588235294117647, 0.788235294117647, 0.788235294117647, 0.7647058823529411, 0.6588235294117647</t>
+        </is>
+      </c>
+      <c r="BD9" t="n">
+        <v>0.7440176070428172</v>
+      </c>
+      <c r="BE9" t="n">
+        <v>0.7647058823529411</v>
+      </c>
+      <c r="BF9" t="n">
+        <v>0.07061116591341229</v>
+      </c>
+      <c r="BG9" t="inlineStr">
+        <is>
+          <t>0.9595543345543346, 0.9641025641025641, 0.9572146807440925, 0.9567621920563096, 0.9577677224736049, 0.9569130216189041, 0.9638511814982402</t>
+        </is>
+      </c>
+      <c r="BH9" t="n">
+        <v>0.9594522424354358</v>
+      </c>
+      <c r="BI9" t="n">
+        <v>0.9577677224736049</v>
+      </c>
+      <c r="BJ9" t="n">
+        <v>0.002988427262158605</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CatBoostClassifier_splashing_base</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>{'estimator': &lt;catboost.core.CatBoostClassifier object at 0x16fb7af50&gt;, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Re', 'sedimentation_Stk'), 'log_features': ('relative_roughness',), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sign_sedimentation_Re', 'particle_liquid_density_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.8679245283018868</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.9583333333333334</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.910891089108911</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.9467592592592593</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.9966329966329966</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.9948186528497409</v>
+      </c>
+      <c r="L10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.9974025974025974</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0.9988839285714286</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>0.6066570281982422, 0.5708298683166504, 0.5453627109527588, 0.5702857971191406, 0.5615198612213135, 0.5314240455627441, 0.5659708976745605</t>
+        </is>
+      </c>
+      <c r="P10" t="n">
+        <v>0.5645786012922015</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>0.5659708976745605</v>
+      </c>
+      <c r="R10" t="n">
+        <v>0.02178470571524163</v>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>0.0053708553314208984, 0.0063610076904296875, 0.0051500797271728516, 0.005546092987060547, 0.004878997802734375, 0.005018711090087891, 0.005541801452636719</t>
+        </is>
+      </c>
+      <c r="T10" t="n">
+        <v>0.005409649440220424</v>
+      </c>
+      <c r="U10" t="n">
+        <v>0.005370855331420898</v>
+      </c>
+      <c r="V10" t="n">
+        <v>0.0004542606062731175</v>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>0.9629629629629629, 0.8679245283018868, 0.9056603773584906, 0.8301886792452831, 0.8867924528301887, 0.8867924528301887, 0.8679245283018868</t>
+        </is>
+      </c>
+      <c r="X10" t="n">
+        <v>0.8868922831186982</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>0.8867924528301887</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>0.03793577234399872</v>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>0.9722222222222222, 0.8985507246376812, 0.9275362318840579, 0.8656716417910447, 0.9090909090909091, 0.9090909090909091, 0.8985507246376812</t>
+        </is>
+      </c>
+      <c r="AB10" t="n">
+        <v>0.9115304804792151</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>0.9090909090909091</v>
+      </c>
+      <c r="AD10" t="n">
+        <v>0.03021720375687164</v>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>0.9459459459459459, 0.9117647058823529, 0.9142857142857143, 0.8787878787878788, 0.9375, 0.9375, 0.8857142857142857</t>
+        </is>
+      </c>
+      <c r="AF10" t="n">
+        <v>0.915928361516597</v>
+      </c>
+      <c r="AG10" t="n">
+        <v>0.9142857142857143</v>
+      </c>
+      <c r="AH10" t="n">
+        <v>0.02433124593359062</v>
+      </c>
+      <c r="AI10" t="inlineStr">
+        <is>
+          <t>1.0, 0.8857142857142857, 0.9411764705882353, 0.8529411764705882, 0.8823529411764706, 0.8823529411764706, 0.9117647058823529</t>
+        </is>
+      </c>
+      <c r="AJ10" t="n">
+        <v>0.9080432172869148</v>
+      </c>
+      <c r="AK10" t="n">
+        <v>0.8857142857142857</v>
+      </c>
+      <c r="AL10" t="n">
+        <v>0.04539117047431458</v>
+      </c>
+      <c r="AM10" t="inlineStr">
+        <is>
+          <t>1.0, 0.9396825396825397, 0.9736842105263158, 0.93343653250774, 0.9705882352941176, 0.9504643962848298, 0.9226006191950464</t>
+        </is>
+      </c>
+      <c r="AN10" t="n">
+        <v>0.9557795047843699</v>
+      </c>
+      <c r="AO10" t="n">
+        <v>0.9504643962848298</v>
+      </c>
+      <c r="AP10" t="n">
+        <v>0.02502210082274886</v>
+      </c>
+      <c r="AQ10" t="inlineStr">
+        <is>
+          <t>0.9874213836477987, 0.9937304075235109, 0.9905956112852664, 0.9905956112852664, 0.987460815047022, 0.9937304075235109, 0.9905956112852664</t>
+        </is>
+      </c>
+      <c r="AR10" t="n">
+        <v>0.9905899782282346</v>
+      </c>
+      <c r="AS10" t="n">
+        <v>0.9905956112852664</v>
+      </c>
+      <c r="AT10" t="n">
+        <v>0.002377163415894737</v>
+      </c>
+      <c r="AU10" t="inlineStr">
+        <is>
+          <t>0.9902912621359223, 0.9951456310679612, 0.9927360774818401, 0.9927007299270073, 0.9902912621359223, 0.9951456310679612, 0.9927360774818401</t>
+        </is>
+      </c>
+      <c r="AV10" t="n">
+        <v>0.9927209530426364</v>
+      </c>
+      <c r="AW10" t="n">
+        <v>0.9927360774818401</v>
+      </c>
+      <c r="AX10" t="n">
+        <v>0.001834813705181454</v>
+      </c>
+      <c r="AY10" t="inlineStr">
+        <is>
+          <t>0.9855072463768116, 0.9903381642512077, 0.9903381642512077, 0.9951219512195122, 0.9902912621359223, 0.9951456310679612, 0.9903381642512077</t>
+        </is>
+      </c>
+      <c r="AZ10" t="n">
+        <v>0.9910115119362616</v>
+      </c>
+      <c r="BA10" t="n">
+        <v>0.9903381642512077</v>
+      </c>
+      <c r="BB10" t="n">
+        <v>0.003074376650758704</v>
+      </c>
+      <c r="BC10" t="inlineStr">
+        <is>
+          <t>0.9951219512195122, 1.0, 0.9951456310679612, 0.9902912621359223, 0.9902912621359223, 0.9951456310679612, 0.9951456310679612</t>
+        </is>
+      </c>
+      <c r="BD10" t="n">
+        <v>0.994448766956463</v>
+      </c>
+      <c r="BE10" t="n">
+        <v>0.9951456310679612</v>
+      </c>
+      <c r="BF10" t="n">
+        <v>0.003100597103577546</v>
+      </c>
+      <c r="BG10" t="inlineStr">
+        <is>
+          <t>0.9979063241959854, 0.9986307231493367, 0.9984319958759343, 0.9985179139101297, 0.9984319958759343, 0.9999570409829023, 0.9984319958759343</t>
+        </is>
+      </c>
+      <c r="BH10" t="n">
+        <v>0.9986154271237367</v>
+      </c>
+      <c r="BI10" t="n">
+        <v>0.9984319958759343</v>
+      </c>
+      <c r="BJ10" t="n">
+        <v>0.0005871770933261723</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>no_fragmentation</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>CatBoostClassifier_no_fragmentation_base</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>{'estimator': &lt;catboost.core.CatBoostClassifier object at 0x16fb27f10&gt;, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Re', 'sedimentation_Stk'), 'log_features': ('relative_roughness',), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sign_sedimentation_Re', 'particle_liquid_density_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>0.9066666666666666</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.8095238095238095</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.8292682926829269</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.9781818181818182</v>
+      </c>
+      <c r="J11" t="n">
+        <v>1</v>
+      </c>
+      <c r="K11" t="n">
+        <v>1</v>
+      </c>
+      <c r="L11" t="n">
+        <v>1</v>
+      </c>
+      <c r="M11" t="n">
+        <v>1</v>
+      </c>
+      <c r="N11" t="n">
+        <v>1</v>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>0.5642380714416504, 0.5649821758270264, 0.5700709819793701, 0.5433738231658936, 0.5416419506072998, 0.5433840751647949, 0.5672628879547119</t>
+        </is>
+      </c>
+      <c r="P11" t="n">
+        <v>0.5564219951629639</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>0.5642380714416504</v>
+      </c>
+      <c r="R11" t="n">
+        <v>0.01193362240803832</v>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>0.0054111480712890625, 0.00581812858581543, 0.005033016204833984, 0.00533604621887207, 0.005205631256103516, 0.0053369998931884766, 0.0055849552154541016</t>
+        </is>
+      </c>
+      <c r="T11" t="n">
+        <v>0.005389417920793805</v>
+      </c>
+      <c r="U11" t="n">
+        <v>0.005336999893188477</v>
+      </c>
+      <c r="V11" t="n">
+        <v>0.0002357043477349292</v>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>0.9074074074074074, 0.8301886792452831, 0.9622641509433962, 0.8867924528301887, 0.8867924528301887, 0.9433962264150944, 0.8867924528301887</t>
+        </is>
+      </c>
+      <c r="X11" t="n">
+        <v>0.9005191175002497</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>0.8867924528301887</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>0.04001781509646558</v>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>0.8148148148148148, 0.7096774193548386, 0.9285714285714286, 0.7999999999999999, 0.7272727272727273, 0.888888888888889, 0.7857142857142857</t>
+        </is>
+      </c>
+      <c r="AB11" t="n">
+        <v>0.8078485092309977</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>0.7999999999999999</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>0.07355429314085414</v>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>0.9166666666666666, 0.6470588235294118, 0.9285714285714286, 0.75, 1.0, 0.9230769230769231, 0.7857142857142857</t>
+        </is>
+      </c>
+      <c r="AF11" t="n">
+        <v>0.8501554467941023</v>
+      </c>
+      <c r="AG11" t="n">
+        <v>0.9166666666666666</v>
+      </c>
+      <c r="AH11" t="n">
+        <v>0.1157434080450252</v>
+      </c>
+      <c r="AI11" t="inlineStr">
+        <is>
+          <t>0.7333333333333333, 0.7857142857142857, 0.9285714285714286, 0.8571428571428571, 0.5714285714285714, 0.8571428571428571, 0.7857142857142857</t>
+        </is>
+      </c>
+      <c r="AJ11" t="n">
+        <v>0.7884353741496598</v>
+      </c>
+      <c r="AK11" t="n">
+        <v>0.7857142857142857</v>
+      </c>
+      <c r="AL11" t="n">
+        <v>0.106383770352787</v>
+      </c>
+      <c r="AM11" t="inlineStr">
+        <is>
+          <t>0.9641025641025642, 0.9084249084249085, 0.9908424908424909, 0.9084249084249084, 0.989010989010989, 0.9688644688644689, 0.9761904761904763</t>
+        </is>
+      </c>
+      <c r="AN11" t="n">
+        <v>0.9579801151229724</v>
+      </c>
+      <c r="AO11" t="n">
+        <v>0.9688644688644689</v>
+      </c>
+      <c r="AP11" t="n">
+        <v>0.03260556193142309</v>
+      </c>
+      <c r="AQ11" t="inlineStr">
+        <is>
+          <t>0.9937106918238994, 1.0, 0.9968652037617555, 0.9968652037617555, 0.9937304075235109, 0.9968652037617555, 0.9905956112852664</t>
+        </is>
+      </c>
+      <c r="AR11" t="n">
+        <v>0.9955189031311348</v>
+      </c>
+      <c r="AS11" t="n">
+        <v>0.9968652037617555</v>
+      </c>
+      <c r="AT11" t="n">
+        <v>0.002834102341681714</v>
+      </c>
+      <c r="AU11" t="inlineStr">
+        <is>
+          <t>0.9880952380952381, 1.0, 0.9941520467836257, 0.9940828402366864, 0.9882352941176471, 0.9941520467836257, 0.9822485207100591</t>
+        </is>
+      </c>
+      <c r="AV11" t="n">
+        <v>0.9915665695324117</v>
+      </c>
+      <c r="AW11" t="n">
+        <v>0.9940828402366864</v>
+      </c>
+      <c r="AX11" t="n">
+        <v>0.005355868938882427</v>
+      </c>
+      <c r="AY11" t="inlineStr">
+        <is>
+          <t>0.9880952380952381, 1.0, 0.9883720930232558, 1.0, 0.9882352941176471, 0.9883720930232558, 0.9880952380952381</t>
+        </is>
+      </c>
+      <c r="AZ11" t="n">
+        <v>0.9915957080506621</v>
+      </c>
+      <c r="BA11" t="n">
+        <v>0.9883720930232558</v>
+      </c>
+      <c r="BB11" t="n">
+        <v>0.005316370884193521</v>
+      </c>
+      <c r="BC11" t="inlineStr">
+        <is>
+          <t>0.9880952380952381, 1.0, 1.0, 0.9882352941176471, 0.9882352941176471, 1.0, 0.9764705882352941</t>
+        </is>
+      </c>
+      <c r="BD11" t="n">
+        <v>0.991576630652261</v>
+      </c>
+      <c r="BE11" t="n">
+        <v>0.9882352941176471</v>
+      </c>
+      <c r="BF11" t="n">
+        <v>0.008241888868281137</v>
+      </c>
+      <c r="BG11" t="inlineStr">
+        <is>
+          <t>0.999949124949125, 1.0, 0.9998994469582705, 1.0, 0.9998491704374057, 0.9998994469582704, 0.9998994469582704</t>
+        </is>
+      </c>
+      <c r="BH11" t="n">
+        <v>0.9999280908944774</v>
+      </c>
+      <c r="BI11" t="n">
+        <v>0.9998994469582705</v>
+      </c>
+      <c r="BJ11" t="n">
+        <v>5.274484965747932e-05</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
           <t>XGBClassifier_splashing_base</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>{'estimator': XGBClassifier(base_score=None, booster=None, callbacks=None,
               colsample_bylevel=None, colsample_bynode=None,
@@ -2091,1093 +2971,433 @@
               num_parallel_tree=None, random_state=None, ...), 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Re', 'sedimentation_Stk'), 'log_features': ('relative_roughness',), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sign_sedimentation_Re', 'particle_liquid_density_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
         </is>
       </c>
-      <c r="E8" t="n">
+      <c r="E12" t="n">
         <v>0.8666666666666667</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F12" t="n">
         <v>0.8518518518518519</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G12" t="n">
         <v>0.9583333333333334</v>
       </c>
-      <c r="H8" t="n">
+      <c r="H12" t="n">
         <v>0.9019607843137256</v>
       </c>
-      <c r="I8" t="n">
+      <c r="I12" t="n">
         <v>0.9440586419753086</v>
       </c>
-      <c r="J8" t="n">
+      <c r="J12" t="n">
         <v>0.9966329966329966</v>
       </c>
-      <c r="K8" t="n">
+      <c r="K12" t="n">
         <v>0.9948186528497409</v>
       </c>
-      <c r="L8" t="n">
+      <c r="L12" t="n">
         <v>1</v>
       </c>
-      <c r="M8" t="n">
+      <c r="M12" t="n">
         <v>0.9974025974025974</v>
       </c>
-      <c r="N8" t="n">
+      <c r="N12" t="n">
         <v>0.9999751984126984</v>
       </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>0.08282208442687988, 0.09463286399841309, 0.08095884323120117, 0.0952138900756836, 0.09817290306091309, 0.07666778564453125, 0.07187414169311523</t>
-        </is>
-      </c>
-      <c r="P8" t="n">
-        <v>0.08576321601867676</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>0.08282208442687988</v>
-      </c>
-      <c r="R8" t="n">
-        <v>0.009481950674350216</v>
-      </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>0.009022951126098633, 0.007380962371826172, 0.008313179016113281, 0.009870052337646484, 0.008810043334960938, 0.006027936935424805, 0.00585174560546875</t>
-        </is>
-      </c>
-      <c r="T8" t="n">
-        <v>0.007896695818219866</v>
-      </c>
-      <c r="U8" t="n">
-        <v>0.008313179016113281</v>
-      </c>
-      <c r="V8" t="n">
-        <v>0.001419774178932221</v>
-      </c>
-      <c r="W8" t="inlineStr">
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>0.040197134017944336, 0.03922295570373535, 0.03351879119873047, 0.03398489952087402, 0.032292842864990234, 0.0335690975189209, 0.03051900863647461</t>
+        </is>
+      </c>
+      <c r="P12" t="n">
+        <v>0.03475781849452427</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>0.0335690975189209</v>
+      </c>
+      <c r="R12" t="n">
+        <v>0.003319054673175258</v>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>0.006788015365600586, 0.005930900573730469, 0.006511211395263672, 0.005742073059082031, 0.006432056427001953, 0.005510807037353516, 0.005647897720336914</t>
+        </is>
+      </c>
+      <c r="T12" t="n">
+        <v>0.006080423082624163</v>
+      </c>
+      <c r="U12" t="n">
+        <v>0.005930900573730469</v>
+      </c>
+      <c r="V12" t="n">
+        <v>0.0004564286464750315</v>
+      </c>
+      <c r="W12" t="inlineStr">
         <is>
           <t>0.9629629629629629, 0.8490566037735849, 0.9056603773584906, 0.8301886792452831, 0.8867924528301887, 0.8867924528301887, 0.8490566037735849</t>
         </is>
       </c>
-      <c r="X8" t="n">
+      <c r="X12" t="n">
         <v>0.8815014475391835</v>
       </c>
-      <c r="Y8" t="n">
+      <c r="Y12" t="n">
         <v>0.8867924528301887</v>
       </c>
-      <c r="Z8" t="n">
+      <c r="Z12" t="n">
         <v>0.04142800609502062</v>
       </c>
-      <c r="AA8" t="inlineStr">
+      <c r="AA12" t="inlineStr">
         <is>
           <t>0.9722222222222222, 0.8857142857142857, 0.9253731343283583, 0.8695652173913043, 0.9090909090909091, 0.90625, 0.8857142857142858</t>
         </is>
       </c>
-      <c r="AB8" t="n">
+      <c r="AB12" t="n">
         <v>0.9077042934944808</v>
       </c>
-      <c r="AC8" t="n">
+      <c r="AC12" t="n">
         <v>0.90625</v>
       </c>
-      <c r="AD8" t="n">
+      <c r="AD12" t="n">
         <v>0.03139722177532166</v>
       </c>
-      <c r="AE8" t="inlineStr">
+      <c r="AE12" t="inlineStr">
         <is>
           <t>0.9459459459459459, 0.8857142857142857, 0.9393939393939394, 0.8571428571428571, 0.9375, 0.9666666666666667, 0.8611111111111112</t>
         </is>
       </c>
-      <c r="AF8" t="n">
+      <c r="AF12" t="n">
         <v>0.9133535437106867</v>
       </c>
-      <c r="AG8" t="n">
+      <c r="AG12" t="n">
         <v>0.9375</v>
       </c>
-      <c r="AH8" t="n">
+      <c r="AH12" t="n">
         <v>0.0410897083958572</v>
       </c>
-      <c r="AI8" t="inlineStr">
+      <c r="AI12" t="inlineStr">
         <is>
           <t>1.0, 0.8857142857142857, 0.9117647058823529, 0.8823529411764706, 0.8823529411764706, 0.8529411764705882, 0.9117647058823529</t>
         </is>
       </c>
-      <c r="AJ8" t="n">
+      <c r="AJ12" t="n">
         <v>0.9038415366146458</v>
       </c>
-      <c r="AK8" t="n">
+      <c r="AK12" t="n">
         <v>0.8857142857142857</v>
       </c>
-      <c r="AL8" t="n">
+      <c r="AL12" t="n">
         <v>0.04344942323952641</v>
       </c>
-      <c r="AM8" t="inlineStr">
+      <c r="AM12" t="inlineStr">
         <is>
           <t>0.9984962406015038, 0.9333333333333333, 0.9520123839009289, 0.8978328173374612, 0.9659442724458205, 0.9342105263157896, 0.9256965944272446</t>
         </is>
       </c>
-      <c r="AN8" t="n">
+      <c r="AN12" t="n">
         <v>0.9439323097660115</v>
       </c>
-      <c r="AO8" t="n">
+      <c r="AO12" t="n">
         <v>0.9342105263157896</v>
       </c>
-      <c r="AP8" t="n">
+      <c r="AP12" t="n">
         <v>0.02974076696634106</v>
       </c>
-      <c r="AQ8" t="inlineStr">
+      <c r="AQ12" t="inlineStr">
         <is>
           <t>0.9968553459119497, 1.0, 0.9968652037617555, 0.9968652037617555, 0.9968652037617555, 1.0, 0.9968652037617555</t>
         </is>
       </c>
-      <c r="AR8" t="n">
+      <c r="AR12" t="n">
         <v>0.9977594515655674</v>
       </c>
-      <c r="AS8" t="n">
+      <c r="AS12" t="n">
         <v>0.9968652037617555</v>
       </c>
-      <c r="AT8" t="n">
+      <c r="AT12" t="n">
         <v>0.001417051170840857</v>
       </c>
-      <c r="AU8" t="inlineStr">
+      <c r="AU12" t="inlineStr">
         <is>
           <t>0.9975669099756691, 1.0, 0.9975786924939467, 0.9975786924939467, 0.9975786924939467, 1.0, 0.9975786924939467</t>
         </is>
       </c>
-      <c r="AV8" t="n">
+      <c r="AV12" t="n">
         <v>0.9982688114216364</v>
       </c>
-      <c r="AW8" t="n">
+      <c r="AW12" t="n">
         <v>0.9975786924939467</v>
       </c>
-      <c r="AX8" t="n">
+      <c r="AX12" t="n">
         <v>0.001094907038779773</v>
       </c>
-      <c r="AY8" t="inlineStr">
+      <c r="AY12" t="inlineStr">
         <is>
           <t>0.9951456310679612, 1.0, 0.9951690821256038, 0.9951690821256038, 0.9951690821256038, 1.0, 0.9951690821256038</t>
         </is>
       </c>
-      <c r="AZ8" t="n">
+      <c r="AZ12" t="n">
         <v>0.9965459942243395</v>
       </c>
-      <c r="BA8" t="n">
+      <c r="BA12" t="n">
         <v>0.9951690821256038</v>
       </c>
-      <c r="BB8" t="n">
+      <c r="BB12" t="n">
         <v>0.002184519446236978</v>
       </c>
-      <c r="BC8" t="inlineStr">
+      <c r="BC12" t="inlineStr">
         <is>
           <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
         </is>
       </c>
-      <c r="BD8" t="n">
+      <c r="BD12" t="n">
         <v>1</v>
       </c>
-      <c r="BE8" t="n">
+      <c r="BE12" t="n">
         <v>1</v>
       </c>
-      <c r="BF8" t="n">
+      <c r="BF12" t="n">
         <v>0</v>
       </c>
-      <c r="BG8" t="inlineStr">
+      <c r="BG12" t="inlineStr">
         <is>
           <t>0.9999784157133608, 1.0, 0.9999355614743535, 0.9999785204914512, 0.9999785204914512, 1.0, 0.9999785204914512</t>
         </is>
       </c>
-      <c r="BH8" t="n">
+      <c r="BH12" t="n">
         <v>0.9999785055231526</v>
       </c>
-      <c r="BI8" t="n">
+      <c r="BI12" t="n">
         <v>0.9999785204914512</v>
       </c>
-      <c r="BJ8" t="n">
+      <c r="BJ12" t="n">
         <v>1.988619454760789e-05</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>df_dimless</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>no_fragmentation</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>LogisticRegression_no_fragmentation_base</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>{'estimator': LogisticRegression(), 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Re', 'sedimentation_Stk'), 'log_features': ('relative_roughness',), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sign_sedimentation_Re', 'particle_liquid_density_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>0.8533333333333334</v>
-      </c>
-      <c r="F9" t="n">
-        <v>0.7368421052631579</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0.717948717948718</v>
-      </c>
-      <c r="I9" t="n">
-        <v>0.9254545454545455</v>
-      </c>
-      <c r="J9" t="n">
-        <v>0.8754208754208754</v>
-      </c>
-      <c r="K9" t="n">
-        <v>0.8181818181818182</v>
-      </c>
-      <c r="L9" t="n">
-        <v>0.6835443037974683</v>
-      </c>
-      <c r="M9" t="n">
-        <v>0.7448275862068965</v>
-      </c>
-      <c r="N9" t="n">
-        <v>0.9316571826733249</v>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>0.00896906852722168, 0.013093233108520508, 0.0, 0.008106708526611328, 0.010124683380126953, 0.0, 0.0</t>
-        </is>
-      </c>
-      <c r="P9" t="n">
-        <v>0.005756241934640067</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>0.008106708526611328</v>
-      </c>
-      <c r="R9" t="n">
-        <v>0.005184656369554661</v>
-      </c>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t>0.007524251937866211, 0.005464315414428711, 0.010611295700073242, 0.0, 0.0, 0.0, 0.010504722595214844</t>
-        </is>
-      </c>
-      <c r="T9" t="n">
-        <v>0.00487208366394043</v>
-      </c>
-      <c r="U9" t="n">
-        <v>0.005464315414428711</v>
-      </c>
-      <c r="V9" t="n">
-        <v>0.004523928583663451</v>
-      </c>
-      <c r="W9" t="inlineStr">
-        <is>
-          <t>0.8148148148148148, 0.7924528301886793, 0.9245283018867925, 0.8490566037735849, 0.8490566037735849, 0.8490566037735849, 0.8867924528301887</t>
-        </is>
-      </c>
-      <c r="X9" t="n">
-        <v>0.85225117300589</v>
-      </c>
-      <c r="Y9" t="n">
-        <v>0.8490566037735849</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>0.04039982656823135</v>
-      </c>
-      <c r="AA9" t="inlineStr">
-        <is>
-          <t>0.5833333333333334, 0.6206896551724138, 0.8571428571428571, 0.7333333333333334, 0.6363636363636364, 0.6666666666666666, 0.7999999999999999</t>
-        </is>
-      </c>
-      <c r="AB9" t="n">
-        <v>0.6996470688588915</v>
-      </c>
-      <c r="AC9" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="AD9" t="n">
-        <v>0.09324779318350135</v>
-      </c>
-      <c r="AE9" t="inlineStr">
-        <is>
-          <t>0.7777777777777778, 0.6, 0.8571428571428571, 0.6875, 0.875, 0.8, 0.75</t>
-        </is>
-      </c>
-      <c r="AF9" t="n">
-        <v>0.7639172335600907</v>
-      </c>
-      <c r="AG9" t="n">
-        <v>0.7777777777777778</v>
-      </c>
-      <c r="AH9" t="n">
-        <v>0.08898364299549143</v>
-      </c>
-      <c r="AI9" t="inlineStr">
-        <is>
-          <t>0.4666666666666667, 0.6428571428571429, 0.8571428571428571, 0.7857142857142857, 0.5, 0.5714285714285714, 0.8571428571428571</t>
-        </is>
-      </c>
-      <c r="AJ9" t="n">
-        <v>0.6687074829931972</v>
-      </c>
-      <c r="AK9" t="n">
-        <v>0.6428571428571429</v>
-      </c>
-      <c r="AL9" t="n">
-        <v>0.1531201700556019</v>
-      </c>
-      <c r="AM9" t="inlineStr">
-        <is>
-          <t>0.9418803418803419, 0.8498168498168499, 0.9578754578754578, 0.8864468864468865, 0.9560439560439561, 0.9212454212454212, 0.9633699633699634</t>
-        </is>
-      </c>
-      <c r="AN9" t="n">
-        <v>0.9252398395255538</v>
-      </c>
-      <c r="AO9" t="n">
-        <v>0.9418803418803419</v>
-      </c>
-      <c r="AP9" t="n">
-        <v>0.03955875522584676</v>
-      </c>
-      <c r="AQ9" t="inlineStr">
-        <is>
-          <t>0.8773584905660378, 0.877742946708464, 0.8589341692789969, 0.877742946708464, 0.8746081504702194, 0.8714733542319749, 0.8526645768025078</t>
-        </is>
-      </c>
-      <c r="AR9" t="n">
-        <v>0.8700749478238093</v>
-      </c>
-      <c r="AS9" t="n">
-        <v>0.8746081504702194</v>
-      </c>
-      <c r="AT9" t="n">
-        <v>0.009414197796548299</v>
-      </c>
-      <c r="AU9" t="inlineStr">
-        <is>
-          <t>0.7547169811320756, 0.7577639751552795, 0.7133757961783439, 0.751592356687898, 0.7468354430379747, 0.7453416149068324, 0.69281045751634</t>
-        </is>
-      </c>
-      <c r="AV9" t="n">
-        <v>0.737490946373535</v>
-      </c>
-      <c r="AW9" t="n">
-        <v>0.7468354430379747</v>
-      </c>
-      <c r="AX9" t="n">
-        <v>0.02278289116899502</v>
-      </c>
-      <c r="AY9" t="inlineStr">
-        <is>
-          <t>0.8, 0.8026315789473685, 0.7777777777777778, 0.8194444444444444, 0.8082191780821918, 0.7894736842105263, 0.7794117647058824</t>
-        </is>
-      </c>
-      <c r="AZ9" t="n">
-        <v>0.7967083468811701</v>
-      </c>
-      <c r="BA9" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="BB9" t="n">
-        <v>0.014168514244079</v>
-      </c>
-      <c r="BC9" t="inlineStr">
-        <is>
-          <t>0.7142857142857143, 0.7176470588235294, 0.6588235294117647, 0.6941176470588235, 0.6941176470588235, 0.7058823529411765, 0.6235294117647059</t>
-        </is>
-      </c>
-      <c r="BD9" t="n">
-        <v>0.6869147659063627</v>
-      </c>
-      <c r="BE9" t="n">
-        <v>0.6941176470588235</v>
-      </c>
-      <c r="BF9" t="n">
-        <v>0.03154134629409137</v>
-      </c>
-      <c r="BG9" t="inlineStr">
-        <is>
-          <t>0.9281135531135531, 0.9407742584213172, 0.9262443438914028, 0.9370035193564605, 0.9277526395173454, 0.9327300150829563, 0.9243841126194067</t>
-        </is>
-      </c>
-      <c r="BH9" t="n">
-        <v>0.9310003488574919</v>
-      </c>
-      <c r="BI9" t="n">
-        <v>0.9281135531135531</v>
-      </c>
-      <c r="BJ9" t="n">
-        <v>0.005604009792409489</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>df_dimless</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>no_fragmentation</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>KNeighborsClassifier_no_fragmentation_base</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>{'estimator': KNeighborsClassifier(), 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Re', 'sedimentation_Stk'), 'log_features': ('relative_roughness',), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sign_sedimentation_Re', 'particle_liquid_density_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>0.88</v>
-      </c>
-      <c r="F10" t="n">
-        <v>0.7894736842105263</v>
-      </c>
-      <c r="G10" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0.7692307692307692</v>
-      </c>
-      <c r="I10" t="n">
-        <v>0.9495454545454545</v>
-      </c>
-      <c r="J10" t="n">
-        <v>0.8922558922558923</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0.8309859154929577</v>
-      </c>
-      <c r="L10" t="n">
-        <v>0.7468354430379747</v>
-      </c>
-      <c r="M10" t="n">
-        <v>0.7866666666666666</v>
-      </c>
-      <c r="N10" t="n">
-        <v>0.9578155847172223</v>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>0.007361412048339844, 0.0034761428833007812, 0.0, 0.004326820373535156, 0.0, 0.01344752311706543, 0.00612187385559082</t>
-        </is>
-      </c>
-      <c r="P10" t="n">
-        <v>0.004961967468261719</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>0.004326820373535156</v>
-      </c>
-      <c r="R10" t="n">
-        <v>0.00432535218434897</v>
-      </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>0.010094881057739258, 0.002934694290161133, 0.013010263442993164, 0.004120349884033203, 0.0160982608795166, 0.0, 0.008006095886230469</t>
-        </is>
-      </c>
-      <c r="T10" t="n">
-        <v>0.007752077920096261</v>
-      </c>
-      <c r="U10" t="n">
-        <v>0.008006095886230469</v>
-      </c>
-      <c r="V10" t="n">
-        <v>0.005336556973224901</v>
-      </c>
-      <c r="W10" t="inlineStr">
-        <is>
-          <t>0.8888888888888888, 0.7735849056603774, 0.8679245283018868, 0.8301886792452831, 0.8490566037735849, 0.8490566037735849, 0.8867924528301887</t>
-        </is>
-      </c>
-      <c r="X10" t="n">
-        <v>0.8493560946391135</v>
-      </c>
-      <c r="Y10" t="n">
-        <v>0.8490566037735849</v>
-      </c>
-      <c r="Z10" t="n">
-        <v>0.03667999015847824</v>
-      </c>
-      <c r="AA10" t="inlineStr">
-        <is>
-          <t>0.8000000000000002, 0.5714285714285714, 0.7200000000000001, 0.6666666666666666, 0.6923076923076924, 0.6666666666666666, 0.8125000000000001</t>
-        </is>
-      </c>
-      <c r="AB10" t="n">
-        <v>0.7042242281527996</v>
-      </c>
-      <c r="AC10" t="n">
-        <v>0.6923076923076924</v>
-      </c>
-      <c r="AD10" t="n">
-        <v>0.07722263485750151</v>
-      </c>
-      <c r="AE10" t="inlineStr">
-        <is>
-          <t>0.8, 0.5714285714285714, 0.8181818181818182, 0.6923076923076923, 0.75, 0.8, 0.7222222222222222</t>
-        </is>
-      </c>
-      <c r="AF10" t="n">
-        <v>0.7363057577343292</v>
-      </c>
-      <c r="AG10" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="AH10" t="n">
-        <v>0.07957368269107451</v>
-      </c>
-      <c r="AI10" t="inlineStr">
-        <is>
-          <t>0.8, 0.5714285714285714, 0.6428571428571429, 0.6428571428571429, 0.6428571428571429, 0.5714285714285714, 0.9285714285714286</t>
-        </is>
-      </c>
-      <c r="AJ10" t="n">
-        <v>0.6857142857142857</v>
-      </c>
-      <c r="AK10" t="n">
-        <v>0.6428571428571429</v>
-      </c>
-      <c r="AL10" t="n">
-        <v>0.1216983797214333</v>
-      </c>
-      <c r="AM10" t="inlineStr">
-        <is>
-          <t>0.9444444444444444, 0.8772893772893773, 0.9487179487179488, 0.8946886446886448, 0.9010989010989011, 0.903846153846154, 0.9468864468864469</t>
-        </is>
-      </c>
-      <c r="AN10" t="n">
-        <v>0.9167102738531312</v>
-      </c>
-      <c r="AO10" t="n">
-        <v>0.903846153846154</v>
-      </c>
-      <c r="AP10" t="n">
-        <v>0.02713046960614661</v>
-      </c>
-      <c r="AQ10" t="inlineStr">
-        <is>
-          <t>0.89937106918239, 0.9059561128526645, 0.9122257053291536, 0.9028213166144201, 0.9059561128526645, 0.9028213166144201, 0.9028213166144201</t>
-        </is>
-      </c>
-      <c r="AR10" t="n">
-        <v>0.9045675642943048</v>
-      </c>
-      <c r="AS10" t="n">
-        <v>0.9028213166144201</v>
-      </c>
-      <c r="AT10" t="n">
-        <v>0.003754139860286498</v>
-      </c>
-      <c r="AU10" t="inlineStr">
-        <is>
-          <t>0.8117647058823529, 0.8255813953488372, 0.829268292682927, 0.8165680473372781, 0.8255813953488372, 0.822857142857143, 0.8143712574850299</t>
-        </is>
-      </c>
-      <c r="AV10" t="n">
-        <v>0.820856033848915</v>
-      </c>
-      <c r="AW10" t="n">
-        <v>0.822857142857143</v>
-      </c>
-      <c r="AX10" t="n">
-        <v>0.00612395781888402</v>
-      </c>
-      <c r="AY10" t="inlineStr">
-        <is>
-          <t>0.8023255813953488, 0.8160919540229885, 0.8607594936708861, 0.8214285714285714, 0.8160919540229885, 0.8, 0.8292682926829268</t>
-        </is>
-      </c>
-      <c r="AZ10" t="n">
-        <v>0.8208522638891014</v>
-      </c>
-      <c r="BA10" t="n">
-        <v>0.8160919540229885</v>
-      </c>
-      <c r="BB10" t="n">
-        <v>0.01884949652022786</v>
-      </c>
-      <c r="BC10" t="inlineStr">
-        <is>
-          <t>0.8214285714285714, 0.8352941176470589, 0.8, 0.8117647058823529, 0.8352941176470589, 0.8470588235294118, 0.8</t>
-        </is>
-      </c>
-      <c r="BD10" t="n">
-        <v>0.821548619447779</v>
-      </c>
-      <c r="BE10" t="n">
-        <v>0.8214285714285714</v>
-      </c>
-      <c r="BF10" t="n">
-        <v>0.01712589238622703</v>
-      </c>
-      <c r="BG10" t="inlineStr">
-        <is>
-          <t>0.9602920227920229, 0.9680744092508797, 0.9614379084967319, 0.9640020110608346, 0.9654600301659125, 0.9612116641528407, 0.9623428858722977</t>
-        </is>
-      </c>
-      <c r="BH10" t="n">
-        <v>0.9632601331130743</v>
-      </c>
-      <c r="BI10" t="n">
-        <v>0.9623428858722977</v>
-      </c>
-      <c r="BJ10" t="n">
-        <v>0.002556083322909469</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>df_dimless</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>no_fragmentation</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>SVC_no_fragmentation_base</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>{'estimator': SVC(probability=True), 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Re', 'sedimentation_Stk'), 'log_features': ('relative_roughness',), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sign_sedimentation_Re', 'particle_liquid_density_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="F11" t="n">
-        <v>0.7222222222222222</v>
-      </c>
-      <c r="G11" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="H11" t="n">
-        <v>0.6842105263157895</v>
-      </c>
-      <c r="I11" t="n">
-        <v>0.9281818181818182</v>
-      </c>
-      <c r="J11" t="n">
-        <v>0.8888888888888888</v>
-      </c>
-      <c r="K11" t="n">
-        <v>0.8194444444444444</v>
-      </c>
-      <c r="L11" t="n">
-        <v>0.7468354430379747</v>
-      </c>
-      <c r="M11" t="n">
-        <v>0.781456953642384</v>
-      </c>
-      <c r="N11" t="n">
-        <v>0.9624898385785624</v>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>0.008918046951293945, 0.015131235122680664, 0.00925302505493164, 0.005823373794555664, 0.015625, 0.015604257583618164, 0.026727914810180664</t>
-        </is>
-      </c>
-      <c r="P11" t="n">
-        <v>0.01386897904532296</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>0.01513123512268066</v>
-      </c>
-      <c r="R11" t="n">
-        <v>0.006364980577914103</v>
-      </c>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>0.029338359832763672, 0.008470535278320312, 0.011104106903076172, 0.010102987289428711, 0.0, 0.0, 0.0024471282958984375</t>
-        </is>
-      </c>
-      <c r="T11" t="n">
-        <v>0.00878044537135533</v>
-      </c>
-      <c r="U11" t="n">
-        <v>0.008470535278320312</v>
-      </c>
-      <c r="V11" t="n">
-        <v>0.009442879088229031</v>
-      </c>
-      <c r="W11" t="inlineStr">
-        <is>
-          <t>0.8333333333333334, 0.7358490566037735, 0.8679245283018868, 0.8867924528301887, 0.8867924528301887, 0.8679245283018868, 0.8301886792452831</t>
-        </is>
-      </c>
-      <c r="X11" t="n">
-        <v>0.844115004492363</v>
-      </c>
-      <c r="Y11" t="n">
-        <v>0.8679245283018868</v>
-      </c>
-      <c r="Z11" t="n">
-        <v>0.04900177617977858</v>
-      </c>
-      <c r="AA11" t="inlineStr">
-        <is>
-          <t>0.6666666666666665, 0.5, 0.6956521739130435, 0.7857142857142857, 0.75, 0.7200000000000001, 0.689655172413793</t>
-        </is>
-      </c>
-      <c r="AB11" t="n">
-        <v>0.6868126141011126</v>
-      </c>
-      <c r="AC11" t="n">
-        <v>0.6956521739130435</v>
-      </c>
-      <c r="AD11" t="n">
-        <v>0.08474045998405863</v>
-      </c>
-      <c r="AE11" t="inlineStr">
-        <is>
-          <t>0.75, 0.5, 0.8888888888888888, 0.7857142857142857, 0.9, 0.8181818181818182, 0.6666666666666666</t>
-        </is>
-      </c>
-      <c r="AF11" t="n">
-        <v>0.75849309420738</v>
-      </c>
-      <c r="AG11" t="n">
-        <v>0.7857142857142857</v>
-      </c>
-      <c r="AH11" t="n">
-        <v>0.1290923865694569</v>
-      </c>
-      <c r="AI11" t="inlineStr">
-        <is>
-          <t>0.6, 0.5, 0.5714285714285714, 0.7857142857142857, 0.6428571428571429, 0.6428571428571429, 0.7142857142857143</t>
-        </is>
-      </c>
-      <c r="AJ11" t="n">
-        <v>0.636734693877551</v>
-      </c>
-      <c r="AK11" t="n">
-        <v>0.6428571428571429</v>
-      </c>
-      <c r="AL11" t="n">
-        <v>0.08668065543508287</v>
-      </c>
-      <c r="AM11" t="inlineStr">
-        <is>
-          <t>0.9384615384615385, 0.8626373626373627, 0.9725274725274725, 0.9267399267399268, 0.9523809523809523, 0.9432234432234433, 0.9413919413919414</t>
-        </is>
-      </c>
-      <c r="AN11" t="n">
-        <v>0.9339089481946626</v>
-      </c>
-      <c r="AO11" t="n">
-        <v>0.9413919413919414</v>
-      </c>
-      <c r="AP11" t="n">
-        <v>0.03190862001703766</v>
-      </c>
-      <c r="AQ11" t="inlineStr">
-        <is>
-          <t>0.8805031446540881, 0.9028213166144201, 0.8683385579937304, 0.8840125391849529, 0.8808777429467085, 0.8840125391849529, 0.8746081504702194</t>
-        </is>
-      </c>
-      <c r="AR11" t="n">
-        <v>0.8821677130070105</v>
-      </c>
-      <c r="AS11" t="n">
-        <v>0.8808777429467085</v>
-      </c>
-      <c r="AT11" t="n">
-        <v>0.009900977108437748</v>
-      </c>
-      <c r="AU11" t="inlineStr">
-        <is>
-          <t>0.7532467532467533, 0.8248587570621468, 0.7272727272727274, 0.7836257309941521, 0.7790697674418604, 0.7784431137724551, 0.7368421052631579</t>
-        </is>
-      </c>
-      <c r="AV11" t="n">
-        <v>0.7690512792933218</v>
-      </c>
-      <c r="AW11" t="n">
-        <v>0.7784431137724551</v>
-      </c>
-      <c r="AX11" t="n">
-        <v>0.03058507390673511</v>
-      </c>
-      <c r="AY11" t="inlineStr">
-        <is>
-          <t>0.8285714285714286, 0.7934782608695652, 0.8115942028985508, 0.7790697674418605, 0.7701149425287356, 0.7926829268292683, 0.835820895522388</t>
-        </is>
-      </c>
-      <c r="AZ11" t="n">
-        <v>0.8016189178088281</v>
-      </c>
-      <c r="BA11" t="n">
-        <v>0.7934782608695652</v>
-      </c>
-      <c r="BB11" t="n">
-        <v>0.02281229712069013</v>
-      </c>
-      <c r="BC11" t="inlineStr">
-        <is>
-          <t>0.6904761904761905, 0.8588235294117647, 0.6588235294117647, 0.788235294117647, 0.788235294117647, 0.7647058823529411, 0.6588235294117647</t>
-        </is>
-      </c>
-      <c r="BD11" t="n">
-        <v>0.7440176070428172</v>
-      </c>
-      <c r="BE11" t="n">
-        <v>0.7647058823529411</v>
-      </c>
-      <c r="BF11" t="n">
-        <v>0.07061116591341229</v>
-      </c>
-      <c r="BG11" t="inlineStr">
-        <is>
-          <t>0.9595543345543346, 0.9641025641025641, 0.9572146807440925, 0.9567621920563096, 0.9577677224736049, 0.956913021618904, 0.9638511814982402</t>
-        </is>
-      </c>
-      <c r="BH11" t="n">
-        <v>0.9594522424354358</v>
-      </c>
-      <c r="BI11" t="n">
-        <v>0.9577677224736049</v>
-      </c>
-      <c r="BJ11" t="n">
-        <v>0.002988427262158618</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>df_dimless</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>no_fragmentation</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>XGBClassifier_no_fragmentation_base</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>{'estimator': XGBClassifier(base_score=None, booster=None, callbacks=None,
               colsample_bylevel=None, colsample_bynode=None,
-              colsample_bytree=None, early_stopping_rounds=None,
+              colsample_bytree=None, device=None, early_stopping_rounds=None,
               enable_categorical=False, eval_metric=None, feature_types=None,
-              gamma=None, gpu_id=None, grow_policy=None, importance_type=None,
+              gamma=None, grow_policy=None, importance_type=None,
               interaction_constraints=None, learning_rate=None, max_bin=None,
               max_cat_threshold=None, max_cat_to_onehot=None,
               max_delta_step=None, max_depth=None, max_leaves=None,
               min_child_weight=None, missing=nan, monotone_constraints=None,
-              n_estimators=100, n_jobs=None, num_parallel_tree=None,
-              predictor=None, random_state=None, ...), 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Re', 'sedimentation_Stk'), 'log_features': ('relative_roughness',), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sign_sedimentation_Re', 'particle_liquid_density_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>0.88</v>
-      </c>
-      <c r="F12" t="n">
-        <v>0.7619047619047619</v>
-      </c>
-      <c r="G12" t="n">
+              multi_strategy=None, n_estimators=None, n_jobs=None,
+              num_parallel_tree=None, random_state=None, ...), 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Re', 'sedimentation_Stk'), 'log_features': ('relative_roughness',), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sign_sedimentation_Re', 'particle_liquid_density_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>0.8666666666666667</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.7272727272727273</v>
+      </c>
+      <c r="G13" t="n">
         <v>0.8</v>
       </c>
-      <c r="H12" t="n">
-        <v>0.7804878048780488</v>
-      </c>
-      <c r="I12" t="n">
-        <v>0.9654545454545455</v>
-      </c>
-      <c r="J12" t="n">
+      <c r="H13" t="n">
+        <v>0.761904761904762</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="J13" t="n">
         <v>1</v>
       </c>
-      <c r="K12" t="n">
+      <c r="K13" t="n">
         <v>1</v>
       </c>
-      <c r="L12" t="n">
+      <c r="L13" t="n">
         <v>1</v>
       </c>
-      <c r="M12" t="n">
+      <c r="M13" t="n">
         <v>1</v>
       </c>
-      <c r="N12" t="n">
+      <c r="N13" t="n">
         <v>1</v>
       </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>0.07788205146789551, 0.05489039421081543, 0.06288433074951172, 0.057038068771362305, 0.04688525199890137, 0.07667183876037598, 0.0814962387084961</t>
-        </is>
-      </c>
-      <c r="P12" t="n">
-        <v>0.0653925963810512</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>0.06288433074951172</v>
-      </c>
-      <c r="R12" t="n">
-        <v>0.01237187286775673</v>
-      </c>
-      <c r="S12" t="inlineStr">
-        <is>
-          <t>0.019135475158691406, 0.01563429832458496, 0.016017913818359375, 0.01617717742919922, 0.015770435333251953, 0.015863656997680664, 0.013914346694946289</t>
-        </is>
-      </c>
-      <c r="T12" t="n">
-        <v>0.01607332910810198</v>
-      </c>
-      <c r="U12" t="n">
-        <v>0.01586365699768066</v>
-      </c>
-      <c r="V12" t="n">
-        <v>0.001433290613797244</v>
-      </c>
-      <c r="W12" t="inlineStr">
-        <is>
-          <t>0.9074074074074074, 0.8113207547169812, 0.9433962264150944, 0.8867924528301887, 0.9245283018867925, 0.8867924528301887, 0.9056603773584906</t>
-        </is>
-      </c>
-      <c r="X12" t="n">
-        <v>0.8951282819207348</v>
-      </c>
-      <c r="Y12" t="n">
-        <v>0.9056603773584906</v>
-      </c>
-      <c r="Z12" t="n">
-        <v>0.03894782463392368</v>
-      </c>
-      <c r="AA12" t="inlineStr">
-        <is>
-          <t>0.8, 0.6428571428571429, 0.88, 0.7999999999999999, 0.8571428571428571, 0.7857142857142857, 0.8275862068965518</t>
-        </is>
-      </c>
-      <c r="AB12" t="n">
-        <v>0.7990429275158339</v>
-      </c>
-      <c r="AC12" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AD12" t="n">
-        <v>0.07103103165205046</v>
-      </c>
-      <c r="AE12" t="inlineStr">
-        <is>
-          <t>1.0, 0.6428571428571429, 1.0, 0.75, 0.8571428571428571, 0.7857142857142857, 0.8</t>
-        </is>
-      </c>
-      <c r="AF12" t="n">
-        <v>0.8336734693877551</v>
-      </c>
-      <c r="AG12" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AH12" t="n">
-        <v>0.1211409730861799</v>
-      </c>
-      <c r="AI12" t="inlineStr">
-        <is>
-          <t>0.6666666666666666, 0.6428571428571429, 0.7857142857142857, 0.8571428571428571, 0.8571428571428571, 0.7857142857142857, 0.8571428571428571</t>
-        </is>
-      </c>
-      <c r="AJ12" t="n">
-        <v>0.7789115646258503</v>
-      </c>
-      <c r="AK12" t="n">
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>0.04003310203552246, 0.030820131301879883, 0.033125877380371094, 0.026775121688842773, 0.029233932495117188, 0.028567075729370117, 0.028364181518554688</t>
+        </is>
+      </c>
+      <c r="P13" t="n">
+        <v>0.0309884888785226</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>0.02923393249511719</v>
+      </c>
+      <c r="R13" t="n">
+        <v>0.004140099429056395</v>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>0.0064640045166015625, 0.0062122344970703125, 0.005652904510498047, 0.005545854568481445, 0.0057070255279541016, 0.005602836608886719, 0.005322933197021484</t>
+        </is>
+      </c>
+      <c r="T13" t="n">
+        <v>0.005786827632359096</v>
+      </c>
+      <c r="U13" t="n">
+        <v>0.005652904510498047</v>
+      </c>
+      <c r="V13" t="n">
+        <v>0.0003724363939755224</v>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>0.9074074074074074, 0.8301886792452831, 0.9433962264150944, 0.8867924528301887, 0.9245283018867925, 0.9245283018867925, 0.9245283018867925</t>
+        </is>
+      </c>
+      <c r="X13" t="n">
+        <v>0.9059099530797644</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>0.9245283018867925</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>0.03494195579170031</v>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>0.8, 0.689655172413793, 0.88, 0.7999999999999999, 0.8571428571428571, 0.8461538461538461, 0.8666666666666666</t>
+        </is>
+      </c>
+      <c r="AB13" t="n">
+        <v>0.8199455060538803</v>
+      </c>
+      <c r="AC13" t="n">
+        <v>0.8461538461538461</v>
+      </c>
+      <c r="AD13" t="n">
+        <v>0.06051109293167232</v>
+      </c>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>1.0, 0.6666666666666666, 1.0, 0.75, 0.8571428571428571, 0.9166666666666666, 0.8125</t>
+        </is>
+      </c>
+      <c r="AF13" t="n">
+        <v>0.8575680272108844</v>
+      </c>
+      <c r="AG13" t="n">
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="AH13" t="n">
+        <v>0.1159506672885783</v>
+      </c>
+      <c r="AI13" t="inlineStr">
+        <is>
+          <t>0.6666666666666666, 0.7142857142857143, 0.7857142857142857, 0.8571428571428571, 0.8571428571428571, 0.7857142857142857, 0.9285714285714286</t>
+        </is>
+      </c>
+      <c r="AJ13" t="n">
+        <v>0.7993197278911566</v>
+      </c>
+      <c r="AK13" t="n">
         <v>0.7857142857142857</v>
       </c>
-      <c r="AL12" t="n">
-        <v>0.08414501276770733</v>
-      </c>
-      <c r="AM12" t="inlineStr">
-        <is>
-          <t>0.9709401709401709, 0.8736263736263736, 0.9798534798534799, 0.9267399267399268, 0.9780219780219781, 0.967032967032967, 0.9780219780219781</t>
-        </is>
-      </c>
-      <c r="AN12" t="n">
-        <v>0.9534624106052678</v>
-      </c>
-      <c r="AO12" t="n">
-        <v>0.9709401709401709</v>
-      </c>
-      <c r="AP12" t="n">
-        <v>0.03680129906862034</v>
-      </c>
-      <c r="AQ12" t="inlineStr">
+      <c r="AL13" t="n">
+        <v>0.08331597764568634</v>
+      </c>
+      <c r="AM13" t="inlineStr">
+        <is>
+          <t>0.9675213675213675, 0.8937728937728937, 0.978021978021978, 0.9322344322344323, 0.9706959706959707, 0.9743589743589743, 0.9780219780219781</t>
+        </is>
+      </c>
+      <c r="AN13" t="n">
+        <v>0.956375370661085</v>
+      </c>
+      <c r="AO13" t="n">
+        <v>0.9706959706959707</v>
+      </c>
+      <c r="AP13" t="n">
+        <v>0.02949994933279096</v>
+      </c>
+      <c r="AQ13" t="inlineStr">
         <is>
           <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
         </is>
       </c>
-      <c r="AR12" t="n">
+      <c r="AR13" t="n">
         <v>1</v>
       </c>
-      <c r="AS12" t="n">
+      <c r="AS13" t="n">
         <v>1</v>
       </c>
-      <c r="AT12" t="n">
+      <c r="AT13" t="n">
         <v>0</v>
       </c>
-      <c r="AU12" t="inlineStr">
+      <c r="AU13" t="inlineStr">
         <is>
           <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
         </is>
       </c>
-      <c r="AV12" t="n">
+      <c r="AV13" t="n">
         <v>1</v>
       </c>
-      <c r="AW12" t="n">
+      <c r="AW13" t="n">
         <v>1</v>
       </c>
-      <c r="AX12" t="n">
+      <c r="AX13" t="n">
         <v>0</v>
       </c>
-      <c r="AY12" t="inlineStr">
+      <c r="AY13" t="inlineStr">
         <is>
           <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
         </is>
       </c>
-      <c r="AZ12" t="n">
+      <c r="AZ13" t="n">
         <v>1</v>
       </c>
-      <c r="BA12" t="n">
+      <c r="BA13" t="n">
         <v>1</v>
       </c>
-      <c r="BB12" t="n">
+      <c r="BB13" t="n">
         <v>0</v>
       </c>
-      <c r="BC12" t="inlineStr">
+      <c r="BC13" t="inlineStr">
         <is>
           <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
         </is>
       </c>
-      <c r="BD12" t="n">
+      <c r="BD13" t="n">
         <v>1</v>
       </c>
-      <c r="BE12" t="n">
+      <c r="BE13" t="n">
         <v>1</v>
       </c>
-      <c r="BF12" t="n">
+      <c r="BF13" t="n">
         <v>0</v>
       </c>
-      <c r="BG12" t="inlineStr">
-        <is>
-          <t>1.0, 1.0, 1.0, 0.9999999999999999, 1.0, 0.9999999999999999, 1.0</t>
-        </is>
-      </c>
-      <c r="BH12" t="n">
+      <c r="BG13" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 0.9999999999999999</t>
+        </is>
+      </c>
+      <c r="BH13" t="n">
         <v>1</v>
       </c>
-      <c r="BI12" t="n">
+      <c r="BI13" t="n">
         <v>1</v>
       </c>
-      <c r="BJ12" t="n">
-        <v>5.934391687221749e-17</v>
+      <c r="BJ13" t="n">
+        <v>4.196248604251576e-17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[ADD] New models, review IEEE
</commit_message>
<xml_diff>
--- a/results/metrics_modelling3.xlsx
+++ b/results/metrics_modelling3.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BJ53"/>
+  <dimension ref="A1:BJ59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12260,6 +12260,1326 @@
         <v>0.006631067788558371</v>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>AdaBoostClassifier_splashing_Stk_diam</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>{'estimator': AdaBoostClassifier(), 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>0.8133333333333334</v>
+      </c>
+      <c r="F54" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="G54" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="H54" t="n">
+        <v>0.8571428571428572</v>
+      </c>
+      <c r="I54" t="n">
+        <v>0.8815586419753086</v>
+      </c>
+      <c r="J54" t="n">
+        <v>0.9629629629629629</v>
+      </c>
+      <c r="K54" t="n">
+        <v>0.9593908629441624</v>
+      </c>
+      <c r="L54" t="n">
+        <v>0.984375</v>
+      </c>
+      <c r="M54" t="n">
+        <v>0.9717223650385605</v>
+      </c>
+      <c r="N54" t="n">
+        <v>0.9953621031746032</v>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>0.04229545593261719, 0.04643964767456055, 0.04575991630554199, 0.04851102828979492, 0.04134535789489746, 0.04512667655944824, 0.040598392486572266</t>
+        </is>
+      </c>
+      <c r="P54" t="n">
+        <v>0.04429663930620466</v>
+      </c>
+      <c r="Q54" t="n">
+        <v>0.04512667655944824</v>
+      </c>
+      <c r="R54" t="n">
+        <v>0.002714393570599508</v>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>0.01538991928100586, 0.015076637268066406, 0.010388374328613281, 0.01736736297607422, 0.013797998428344727, 0.012734413146972656, 0.014501333236694336</t>
+        </is>
+      </c>
+      <c r="T54" t="n">
+        <v>0.01417943409511021</v>
+      </c>
+      <c r="U54" t="n">
+        <v>0.01450133323669434</v>
+      </c>
+      <c r="V54" t="n">
+        <v>0.002040394583262948</v>
+      </c>
+      <c r="W54" t="inlineStr">
+        <is>
+          <t>0.8888888888888888, 0.8113207547169812, 0.9056603773584906, 0.7924528301886793, 0.9245283018867925, 0.8113207547169812, 0.8301886792452831</t>
+        </is>
+      </c>
+      <c r="X54" t="n">
+        <v>0.852051512428871</v>
+      </c>
+      <c r="Y54" t="n">
+        <v>0.8301886792452831</v>
+      </c>
+      <c r="Z54" t="n">
+        <v>0.04903608490660909</v>
+      </c>
+      <c r="AA54" t="inlineStr">
+        <is>
+          <t>0.9210526315789475, 0.8571428571428571, 0.9315068493150686, 0.8405797101449276, 0.9411764705882353, 0.84375, 0.8656716417910447</t>
+        </is>
+      </c>
+      <c r="AB54" t="n">
+        <v>0.8858400229372974</v>
+      </c>
+      <c r="AC54" t="n">
+        <v>0.8656716417910447</v>
+      </c>
+      <c r="AD54" t="n">
+        <v>0.04042252933524638</v>
+      </c>
+      <c r="AE54" t="inlineStr">
+        <is>
+          <t>0.8536585365853658, 0.8571428571428571, 0.8717948717948718, 0.8285714285714286, 0.9411764705882353, 0.9, 0.8787878787878788</t>
+        </is>
+      </c>
+      <c r="AF54" t="n">
+        <v>0.8758760062100911</v>
+      </c>
+      <c r="AG54" t="n">
+        <v>0.8717948717948718</v>
+      </c>
+      <c r="AH54" t="n">
+        <v>0.03370782503572691</v>
+      </c>
+      <c r="AI54" t="inlineStr">
+        <is>
+          <t>1.0, 0.8571428571428571, 1.0, 0.8529411764705882, 0.9411764705882353, 0.7941176470588235, 0.8529411764705882</t>
+        </is>
+      </c>
+      <c r="AJ54" t="n">
+        <v>0.8997599039615846</v>
+      </c>
+      <c r="AK54" t="n">
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="AL54" t="n">
+        <v>0.07480638944209077</v>
+      </c>
+      <c r="AM54" t="inlineStr">
+        <is>
+          <t>0.9353383458646617, 0.8714285714285714, 0.9226006191950464, 0.9009287925696594, 0.9411764705882353, 0.836687306501548, 0.8978328173374613</t>
+        </is>
+      </c>
+      <c r="AN54" t="n">
+        <v>0.9008561319264548</v>
+      </c>
+      <c r="AO54" t="n">
+        <v>0.9009287925696594</v>
+      </c>
+      <c r="AP54" t="n">
+        <v>0.03439339782656949</v>
+      </c>
+      <c r="AQ54" t="inlineStr">
+        <is>
+          <t>0.9276729559748428, 0.9247648902821317, 0.9278996865203761, 0.9247648902821317, 0.9153605015673981, 0.9498432601880877, 0.9310344827586207</t>
+        </is>
+      </c>
+      <c r="AR54" t="n">
+        <v>0.9287629525105128</v>
+      </c>
+      <c r="AS54" t="n">
+        <v>0.9276729559748428</v>
+      </c>
+      <c r="AT54" t="n">
+        <v>0.009732619941746736</v>
+      </c>
+      <c r="AU54" t="inlineStr">
+        <is>
+          <t>0.9440389294403893, 0.9411764705882352, 0.943765281173594, 0.9423076923076923, 0.9346246973365618, 0.9611650485436893, 0.9473684210526316</t>
+        </is>
+      </c>
+      <c r="AV54" t="n">
+        <v>0.9449209343489706</v>
+      </c>
+      <c r="AW54" t="n">
+        <v>0.943765281173594</v>
+      </c>
+      <c r="AX54" t="n">
+        <v>0.007548296340363749</v>
+      </c>
+      <c r="AY54" t="inlineStr">
+        <is>
+          <t>0.941747572815534, 0.9458128078817734, 0.9507389162561576, 0.9333333333333333, 0.9323671497584541, 0.9611650485436893, 0.9339622641509434</t>
+        </is>
+      </c>
+      <c r="AZ54" t="n">
+        <v>0.9427324418199835</v>
+      </c>
+      <c r="BA54" t="n">
+        <v>0.941747572815534</v>
+      </c>
+      <c r="BB54" t="n">
+        <v>0.009906864732307152</v>
+      </c>
+      <c r="BC54" t="inlineStr">
+        <is>
+          <t>0.9463414634146341, 0.9365853658536586, 0.9368932038834952, 0.9514563106796117, 0.9368932038834952, 0.9611650485436893, 0.9611650485436893</t>
+        </is>
+      </c>
+      <c r="BD54" t="n">
+        <v>0.9472142349717533</v>
+      </c>
+      <c r="BE54" t="n">
+        <v>0.9463414634146341</v>
+      </c>
+      <c r="BF54" t="n">
+        <v>0.0102401699157158</v>
+      </c>
+      <c r="BG54" t="inlineStr">
+        <is>
+          <t>0.9849341679257501, 0.9855370132648695, 0.9842984792507947, 0.9883366268579775, 0.9821934874130079, 0.9935991064524444, 0.9862960735458373</t>
+        </is>
+      </c>
+      <c r="BH54" t="n">
+        <v>0.986456422101526</v>
+      </c>
+      <c r="BI54" t="n">
+        <v>0.9855370132648695</v>
+      </c>
+      <c r="BJ54" t="n">
+        <v>0.00339265427510108</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>no_fragmentation</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>AdaBoostClassifier_no_fragmentation_Stk_diam</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>{'estimator': AdaBoostClassifier(), 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': (), 'passthrough_features': ('wettability', 'inclination', 'volume_fraction'), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>0.8666666666666667</v>
+      </c>
+      <c r="F55" t="n">
+        <v>0.7272727272727273</v>
+      </c>
+      <c r="G55" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H55" t="n">
+        <v>0.761904761904762</v>
+      </c>
+      <c r="I55" t="n">
+        <v>0.8945454545454545</v>
+      </c>
+      <c r="J55" t="n">
+        <v>0.9764309764309764</v>
+      </c>
+      <c r="K55" t="n">
+        <v>0.9615384615384616</v>
+      </c>
+      <c r="L55" t="n">
+        <v>0.9493670886075949</v>
+      </c>
+      <c r="M55" t="n">
+        <v>0.9554140127388535</v>
+      </c>
+      <c r="N55" t="n">
+        <v>0.9983451399372896</v>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>0.04655003547668457, 0.043056488037109375, 0.04389595985412598, 0.0430448055267334, 0.042558908462524414, 0.04320216178894043, 0.043022871017456055</t>
+        </is>
+      </c>
+      <c r="P55" t="n">
+        <v>0.04361874716622489</v>
+      </c>
+      <c r="Q55" t="n">
+        <v>0.04305648803710938</v>
+      </c>
+      <c r="R55" t="n">
+        <v>0.001251668155833141</v>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>0.011513233184814453, 0.012504100799560547, 0.012018680572509766, 0.010513067245483398, 0.012743234634399414, 0.012613534927368164, 0.010503053665161133</t>
+        </is>
+      </c>
+      <c r="T55" t="n">
+        <v>0.01177270071847098</v>
+      </c>
+      <c r="U55" t="n">
+        <v>0.01201868057250977</v>
+      </c>
+      <c r="V55" t="n">
+        <v>0.0008872424329106799</v>
+      </c>
+      <c r="W55" t="inlineStr">
+        <is>
+          <t>0.8518518518518519, 0.7924528301886793, 0.9245283018867925, 0.8113207547169812, 0.9056603773584906, 0.8679245283018868, 0.9056603773584906</t>
+        </is>
+      </c>
+      <c r="X55" t="n">
+        <v>0.8656284316661675</v>
+      </c>
+      <c r="Y55" t="n">
+        <v>0.8679245283018868</v>
+      </c>
+      <c r="Z55" t="n">
+        <v>0.04655774709538191</v>
+      </c>
+      <c r="AA55" t="inlineStr">
+        <is>
+          <t>0.7333333333333333, 0.5925925925925927, 0.8461538461538461, 0.6875000000000001, 0.8148148148148148, 0.7407407407407408, 0.8275862068965518</t>
+        </is>
+      </c>
+      <c r="AB55" t="n">
+        <v>0.7489602192188399</v>
+      </c>
+      <c r="AC55" t="n">
+        <v>0.7407407407407408</v>
+      </c>
+      <c r="AD55" t="n">
+        <v>0.08324269801375989</v>
+      </c>
+      <c r="AE55" t="inlineStr">
+        <is>
+          <t>0.7333333333333333, 0.6153846153846154, 0.9166666666666666, 0.6111111111111112, 0.8461538461538461, 0.7692307692307693, 0.8</t>
+        </is>
+      </c>
+      <c r="AF55" t="n">
+        <v>0.755982905982906</v>
+      </c>
+      <c r="AG55" t="n">
+        <v>0.7692307692307693</v>
+      </c>
+      <c r="AH55" t="n">
+        <v>0.1051066120353698</v>
+      </c>
+      <c r="AI55" t="inlineStr">
+        <is>
+          <t>0.7333333333333333, 0.5714285714285714, 0.7857142857142857, 0.7857142857142857, 0.7857142857142857, 0.7142857142857143, 0.8571428571428571</t>
+        </is>
+      </c>
+      <c r="AJ55" t="n">
+        <v>0.7476190476190475</v>
+      </c>
+      <c r="AK55" t="n">
+        <v>0.7857142857142857</v>
+      </c>
+      <c r="AL55" t="n">
+        <v>0.08341589690323446</v>
+      </c>
+      <c r="AM55" t="inlineStr">
+        <is>
+          <t>0.876923076923077, 0.8699633699633699, 0.9725274725274725, 0.8965201465201466, 0.946886446886447, 0.9120879120879121, 0.9413919413919414</t>
+        </is>
+      </c>
+      <c r="AN55" t="n">
+        <v>0.9166143380429095</v>
+      </c>
+      <c r="AO55" t="n">
+        <v>0.9120879120879121</v>
+      </c>
+      <c r="AP55" t="n">
+        <v>0.03552178990496289</v>
+      </c>
+      <c r="AQ55" t="inlineStr">
+        <is>
+          <t>0.9842767295597484, 0.9843260188087775, 0.9686520376175548, 0.9749216300940439, 0.9749216300940439, 0.9811912225705329, 0.9749216300940439</t>
+        </is>
+      </c>
+      <c r="AR55" t="n">
+        <v>0.9776015569769635</v>
+      </c>
+      <c r="AS55" t="n">
+        <v>0.9749216300940439</v>
+      </c>
+      <c r="AT55" t="n">
+        <v>0.005402406025743921</v>
+      </c>
+      <c r="AU55" t="inlineStr">
+        <is>
+          <t>0.970059880239521, 0.9710982658959537, 0.941860465116279, 0.9523809523809523, 0.9534883720930232, 0.9651162790697674, 0.9534883720930232</t>
+        </is>
+      </c>
+      <c r="AV55" t="n">
+        <v>0.9582132266983601</v>
+      </c>
+      <c r="AW55" t="n">
+        <v>0.9534883720930232</v>
+      </c>
+      <c r="AX55" t="n">
+        <v>0.01000068786525098</v>
+      </c>
+      <c r="AY55" t="inlineStr">
+        <is>
+          <t>0.9759036144578314, 0.9545454545454546, 0.9310344827586207, 0.963855421686747, 0.9425287356321839, 0.9540229885057471, 0.9425287356321839</t>
+        </is>
+      </c>
+      <c r="AZ55" t="n">
+        <v>0.9520599190312525</v>
+      </c>
+      <c r="BA55" t="n">
+        <v>0.9540229885057471</v>
+      </c>
+      <c r="BB55" t="n">
+        <v>0.01384321962691562</v>
+      </c>
+      <c r="BC55" t="inlineStr">
+        <is>
+          <t>0.9642857142857143, 0.9882352941176471, 0.9529411764705882, 0.9411764705882353, 0.9647058823529412, 0.9764705882352941, 0.9647058823529412</t>
+        </is>
+      </c>
+      <c r="BD55" t="n">
+        <v>0.9646458583433375</v>
+      </c>
+      <c r="BE55" t="n">
+        <v>0.9647058823529412</v>
+      </c>
+      <c r="BF55" t="n">
+        <v>0.01406228169870084</v>
+      </c>
+      <c r="BG55" t="inlineStr">
+        <is>
+          <t>0.9983465608465608, 0.998340874811463, 0.9959276018099548, 0.998265460030166, 0.9964303670186023, 0.9974358974358974, 0.9966817496229261</t>
+        </is>
+      </c>
+      <c r="BH55" t="n">
+        <v>0.9973469302250815</v>
+      </c>
+      <c r="BI55" t="n">
+        <v>0.9974358974358974</v>
+      </c>
+      <c r="BJ55" t="n">
+        <v>0.000936242175825913</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>RandomForestClassifier_splashing_Stk_diam</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>{'estimator': RandomForestClassifier(), 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>0.8666666666666667</v>
+      </c>
+      <c r="F56" t="n">
+        <v>0.8518518518518519</v>
+      </c>
+      <c r="G56" t="n">
+        <v>0.9583333333333334</v>
+      </c>
+      <c r="H56" t="n">
+        <v>0.9019607843137256</v>
+      </c>
+      <c r="I56" t="n">
+        <v>0.9540895061728395</v>
+      </c>
+      <c r="J56" t="n">
+        <v>0.9966329966329966</v>
+      </c>
+      <c r="K56" t="n">
+        <v>0.9948186528497409</v>
+      </c>
+      <c r="L56" t="n">
+        <v>1</v>
+      </c>
+      <c r="M56" t="n">
+        <v>0.9974025974025974</v>
+      </c>
+      <c r="N56" t="n">
+        <v>0.9999751984126984</v>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>0.08300065994262695, 0.08986687660217285, 0.08384990692138672, 0.0838019847869873, 0.08411645889282227, 0.08526420593261719, 0.08512067794799805</t>
+        </is>
+      </c>
+      <c r="P56" t="n">
+        <v>0.08500296728951591</v>
+      </c>
+      <c r="Q56" t="n">
+        <v>0.08411645889282227</v>
+      </c>
+      <c r="R56" t="n">
+        <v>0.002114803410730603</v>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>0.01667308807373047, 0.014289140701293945, 0.012070417404174805, 0.012803792953491211, 0.011937856674194336, 0.012521743774414062, 0.01160287857055664</t>
+        </is>
+      </c>
+      <c r="T56" t="n">
+        <v>0.0131284168788365</v>
+      </c>
+      <c r="U56" t="n">
+        <v>0.01252174377441406</v>
+      </c>
+      <c r="V56" t="n">
+        <v>0.00165828957663176</v>
+      </c>
+      <c r="W56" t="inlineStr">
+        <is>
+          <t>0.9444444444444444, 0.9056603773584906, 0.9056603773584906, 0.8490566037735849, 0.9245283018867925, 0.8490566037735849, 0.8113207547169812</t>
+        </is>
+      </c>
+      <c r="X56" t="n">
+        <v>0.8842467804731956</v>
+      </c>
+      <c r="Y56" t="n">
+        <v>0.9056603773584906</v>
+      </c>
+      <c r="Z56" t="n">
+        <v>0.04465478103184949</v>
+      </c>
+      <c r="AA56" t="inlineStr">
+        <is>
+          <t>0.958904109589041, 0.9275362318840579, 0.9295774647887325, 0.8787878787878787, 0.9411764705882353, 0.8709677419354839, 0.861111111111111</t>
+        </is>
+      </c>
+      <c r="AB56" t="n">
+        <v>0.9097230012406486</v>
+      </c>
+      <c r="AC56" t="n">
+        <v>0.9275362318840579</v>
+      </c>
+      <c r="AD56" t="n">
+        <v>0.03574049493633244</v>
+      </c>
+      <c r="AE56" t="inlineStr">
+        <is>
+          <t>0.9210526315789473, 0.9411764705882353, 0.8918918918918919, 0.90625, 0.9411764705882353, 0.9642857142857143, 0.8157894736842105</t>
+        </is>
+      </c>
+      <c r="AF56" t="n">
+        <v>0.9116603789453193</v>
+      </c>
+      <c r="AG56" t="n">
+        <v>0.9210526315789473</v>
+      </c>
+      <c r="AH56" t="n">
+        <v>0.04505763835239565</v>
+      </c>
+      <c r="AI56" t="inlineStr">
+        <is>
+          <t>1.0, 0.9142857142857143, 0.9705882352941176, 0.8529411764705882, 0.9411764705882353, 0.7941176470588235, 0.9117647058823529</t>
+        </is>
+      </c>
+      <c r="AJ56" t="n">
+        <v>0.912124849939976</v>
+      </c>
+      <c r="AK56" t="n">
+        <v>0.9142857142857143</v>
+      </c>
+      <c r="AL56" t="n">
+        <v>0.06482637499291748</v>
+      </c>
+      <c r="AM56" t="inlineStr">
+        <is>
+          <t>0.9962406015037594, 0.9531746031746031, 0.9876160990712075, 0.9210526315789473, 0.9396284829721362, 0.93343653250774, 0.9303405572755418</t>
+        </is>
+      </c>
+      <c r="AN56" t="n">
+        <v>0.9516413582977049</v>
+      </c>
+      <c r="AO56" t="n">
+        <v>0.9396284829721362</v>
+      </c>
+      <c r="AP56" t="n">
+        <v>0.02712601410933079</v>
+      </c>
+      <c r="AQ56" t="inlineStr">
+        <is>
+          <t>0.9968553459119497, 1.0, 0.9968652037617555, 0.9968652037617555, 0.9968652037617555, 1.0, 0.9968652037617555</t>
+        </is>
+      </c>
+      <c r="AR56" t="n">
+        <v>0.9977594515655674</v>
+      </c>
+      <c r="AS56" t="n">
+        <v>0.9968652037617555</v>
+      </c>
+      <c r="AT56" t="n">
+        <v>0.001417051170840857</v>
+      </c>
+      <c r="AU56" t="inlineStr">
+        <is>
+          <t>0.9975669099756691, 1.0, 0.9975786924939467, 0.9975786924939467, 0.9975786924939467, 1.0, 0.9975786924939467</t>
+        </is>
+      </c>
+      <c r="AV56" t="n">
+        <v>0.9982688114216364</v>
+      </c>
+      <c r="AW56" t="n">
+        <v>0.9975786924939467</v>
+      </c>
+      <c r="AX56" t="n">
+        <v>0.001094907038779773</v>
+      </c>
+      <c r="AY56" t="inlineStr">
+        <is>
+          <t>0.9951456310679612, 1.0, 0.9951690821256038, 0.9951690821256038, 0.9951690821256038, 1.0, 0.9951690821256038</t>
+        </is>
+      </c>
+      <c r="AZ56" t="n">
+        <v>0.9965459942243395</v>
+      </c>
+      <c r="BA56" t="n">
+        <v>0.9951690821256038</v>
+      </c>
+      <c r="BB56" t="n">
+        <v>0.002184519446236978</v>
+      </c>
+      <c r="BC56" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="BD56" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE56" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF56" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG56" t="inlineStr">
+        <is>
+          <t>0.9999784157133607, 0.9999999999999999, 0.9999785204914512, 0.9999785204914511, 0.9999785204914512, 1.0, 0.9999785204914512</t>
+        </is>
+      </c>
+      <c r="BH56" t="n">
+        <v>0.999984642525595</v>
+      </c>
+      <c r="BI56" t="n">
+        <v>0.9999785204914512</v>
+      </c>
+      <c r="BJ56" t="n">
+        <v>9.712984233428587e-06</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>no_fragmentation</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>RandomForestClassifier_no_fragmentation_Stk_diam</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>{'estimator': RandomForestClassifier(), 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': (), 'passthrough_features': ('wettability', 'inclination', 'volume_fraction'), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>0.9466666666666667</v>
+      </c>
+      <c r="F57" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G57" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H57" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="I57" t="n">
+        <v>0.9836363636363636</v>
+      </c>
+      <c r="J57" t="n">
+        <v>1</v>
+      </c>
+      <c r="K57" t="n">
+        <v>1</v>
+      </c>
+      <c r="L57" t="n">
+        <v>1</v>
+      </c>
+      <c r="M57" t="n">
+        <v>1</v>
+      </c>
+      <c r="N57" t="n">
+        <v>1</v>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>0.07860326766967773, 0.07773756980895996, 0.07647180557250977, 0.08232712745666504, 0.08237171173095703, 0.0821986198425293, 0.07474780082702637</t>
+        </is>
+      </c>
+      <c r="P57" t="n">
+        <v>0.07920827184404645</v>
+      </c>
+      <c r="Q57" t="n">
+        <v>0.07860326766967773</v>
+      </c>
+      <c r="R57" t="n">
+        <v>0.002893091210809317</v>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>0.009609460830688477, 0.012346744537353516, 0.01396632194519043, 0.009385347366333008, 0.011641263961791992, 0.011887550354003906, 0.013554096221923828</t>
+        </is>
+      </c>
+      <c r="T57" t="n">
+        <v>0.01177011217389788</v>
+      </c>
+      <c r="U57" t="n">
+        <v>0.01188755035400391</v>
+      </c>
+      <c r="V57" t="n">
+        <v>0.001635514437545498</v>
+      </c>
+      <c r="W57" t="inlineStr">
+        <is>
+          <t>0.8333333333333334, 0.7924528301886793, 0.9056603773584906, 0.8113207547169812, 0.9433962264150944, 0.9433962264150944, 0.9433962264150944</t>
+        </is>
+      </c>
+      <c r="X57" t="n">
+        <v>0.8818508535489668</v>
+      </c>
+      <c r="Y57" t="n">
+        <v>0.9056603773584906</v>
+      </c>
+      <c r="Z57" t="n">
+        <v>0.06239373065756213</v>
+      </c>
+      <c r="AA57" t="inlineStr">
+        <is>
+          <t>0.6666666666666665, 0.6206896551724138, 0.8148148148148148, 0.6428571428571429, 0.88, 0.888888888888889, 0.896551724137931</t>
+        </is>
+      </c>
+      <c r="AB57" t="n">
+        <v>0.7729241275054084</v>
+      </c>
+      <c r="AC57" t="n">
+        <v>0.8148148148148148</v>
+      </c>
+      <c r="AD57" t="n">
+        <v>0.1154711366108976</v>
+      </c>
+      <c r="AE57" t="inlineStr">
+        <is>
+          <t>0.75, 0.6, 0.8461538461538461, 0.6428571428571429, 1.0, 0.9230769230769231, 0.8666666666666667</t>
+        </is>
+      </c>
+      <c r="AF57" t="n">
+        <v>0.8041077969649398</v>
+      </c>
+      <c r="AG57" t="n">
+        <v>0.8461538461538461</v>
+      </c>
+      <c r="AH57" t="n">
+        <v>0.1356457100227356</v>
+      </c>
+      <c r="AI57" t="inlineStr">
+        <is>
+          <t>0.6, 0.6428571428571429, 0.7857142857142857, 0.6428571428571429, 0.7857142857142857, 0.8571428571428571, 0.9285714285714286</t>
+        </is>
+      </c>
+      <c r="AJ57" t="n">
+        <v>0.7489795918367347</v>
+      </c>
+      <c r="AK57" t="n">
+        <v>0.7857142857142857</v>
+      </c>
+      <c r="AL57" t="n">
+        <v>0.1142492653247217</v>
+      </c>
+      <c r="AM57" t="inlineStr">
+        <is>
+          <t>0.9521367521367521, 0.8589743589743589, 0.9752747252747253, 0.9175824175824177, 0.9908424908424909, 0.9093406593406593, 0.9871794871794871</t>
+        </is>
+      </c>
+      <c r="AN57" t="n">
+        <v>0.941618698761556</v>
+      </c>
+      <c r="AO57" t="n">
+        <v>0.9521367521367521</v>
+      </c>
+      <c r="AP57" t="n">
+        <v>0.04502670042190914</v>
+      </c>
+      <c r="AQ57" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="AR57" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS57" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU57" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="AV57" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW57" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY57" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="AZ57" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA57" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC57" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="BD57" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE57" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG57" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="BH57" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI57" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ57" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>LGBMClassifier_splashing_Stk_diam</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>{'estimator': LGBMClassifier(), 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="F58" t="n">
+        <v>0.8823529411764706</v>
+      </c>
+      <c r="G58" t="n">
+        <v>0.9375</v>
+      </c>
+      <c r="H58" t="n">
+        <v>0.9090909090909091</v>
+      </c>
+      <c r="I58" t="n">
+        <v>0.9517746913580247</v>
+      </c>
+      <c r="J58" t="n">
+        <v>0.9966329966329966</v>
+      </c>
+      <c r="K58" t="n">
+        <v>0.9948186528497409</v>
+      </c>
+      <c r="L58" t="n">
+        <v>1</v>
+      </c>
+      <c r="M58" t="n">
+        <v>0.9974025974025974</v>
+      </c>
+      <c r="N58" t="n">
+        <v>0.9999751984126984</v>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>0.13146328926086426, 0.01901865005493164, 0.020598173141479492, 0.01701521873474121, 0.0210115909576416, 0.022017240524291992, 0.018513917922973633</t>
+        </is>
+      </c>
+      <c r="P58" t="n">
+        <v>0.03566258294241769</v>
+      </c>
+      <c r="Q58" t="n">
+        <v>0.02059817314147949</v>
+      </c>
+      <c r="R58" t="n">
+        <v>0.03914146525364429</v>
+      </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>0.011510848999023438, 0.010015487670898438, 0.011011838912963867, 0.009507179260253906, 0.008506298065185547, 0.010508298873901367, 0.01151418685913086</t>
+        </is>
+      </c>
+      <c r="T58" t="n">
+        <v>0.01036773409162249</v>
+      </c>
+      <c r="U58" t="n">
+        <v>0.01050829887390137</v>
+      </c>
+      <c r="V58" t="n">
+        <v>0.00102715079973434</v>
+      </c>
+      <c r="W58" t="inlineStr">
+        <is>
+          <t>0.9629629629629629, 0.8490566037735849, 0.9433962264150944, 0.8490566037735849, 0.9056603773584906, 0.8679245283018868, 0.8867924528301887</t>
+        </is>
+      </c>
+      <c r="X58" t="n">
+        <v>0.8949785364879705</v>
+      </c>
+      <c r="Y58" t="n">
+        <v>0.8867924528301887</v>
+      </c>
+      <c r="Z58" t="n">
+        <v>0.04157065551294201</v>
+      </c>
+      <c r="AA58" t="inlineStr">
+        <is>
+          <t>0.9722222222222222, 0.888888888888889, 0.9565217391304348, 0.8823529411764706, 0.9253731343283583, 0.8923076923076922, 0.9142857142857143</t>
+        </is>
+      </c>
+      <c r="AB58" t="n">
+        <v>0.9188503331913973</v>
+      </c>
+      <c r="AC58" t="n">
+        <v>0.9142857142857143</v>
+      </c>
+      <c r="AD58" t="n">
+        <v>0.03221653434902594</v>
+      </c>
+      <c r="AE58" t="inlineStr">
+        <is>
+          <t>0.9459459459459459, 0.8648648648648649, 0.9428571428571428, 0.8823529411764706, 0.9393939393939394, 0.9354838709677419, 0.8888888888888888</t>
+        </is>
+      </c>
+      <c r="AF58" t="n">
+        <v>0.9142553705849993</v>
+      </c>
+      <c r="AG58" t="n">
+        <v>0.9354838709677419</v>
+      </c>
+      <c r="AH58" t="n">
+        <v>0.03163541475077126</v>
+      </c>
+      <c r="AI58" t="inlineStr">
+        <is>
+          <t>1.0, 0.9142857142857143, 0.9705882352941176, 0.8823529411764706, 0.9117647058823529, 0.8529411764705882, 0.9411764705882353</t>
+        </is>
+      </c>
+      <c r="AJ58" t="n">
+        <v>0.9247298919567827</v>
+      </c>
+      <c r="AK58" t="n">
+        <v>0.9142857142857143</v>
+      </c>
+      <c r="AL58" t="n">
+        <v>0.04669914237959417</v>
+      </c>
+      <c r="AM58" t="inlineStr">
+        <is>
+          <t>0.9954887218045113, 0.9523809523809523, 0.9845201238390093, 0.9458204334365325, 0.9427244582043344, 0.9202786377708978, 0.9256965944272446</t>
+        </is>
+      </c>
+      <c r="AN58" t="n">
+        <v>0.9524157031233546</v>
+      </c>
+      <c r="AO58" t="n">
+        <v>0.9458204334365325</v>
+      </c>
+      <c r="AP58" t="n">
+        <v>0.02610445918315244</v>
+      </c>
+      <c r="AQ58" t="inlineStr">
+        <is>
+          <t>0.9968553459119497, 1.0, 0.9968652037617555, 0.9968652037617555, 0.9968652037617555, 1.0, 0.9968652037617555</t>
+        </is>
+      </c>
+      <c r="AR58" t="n">
+        <v>0.9977594515655674</v>
+      </c>
+      <c r="AS58" t="n">
+        <v>0.9968652037617555</v>
+      </c>
+      <c r="AT58" t="n">
+        <v>0.001417051170840857</v>
+      </c>
+      <c r="AU58" t="inlineStr">
+        <is>
+          <t>0.9975669099756691, 1.0, 0.9975786924939467, 0.9975786924939467, 0.9975786924939467, 1.0, 0.9975786924939467</t>
+        </is>
+      </c>
+      <c r="AV58" t="n">
+        <v>0.9982688114216364</v>
+      </c>
+      <c r="AW58" t="n">
+        <v>0.9975786924939467</v>
+      </c>
+      <c r="AX58" t="n">
+        <v>0.001094907038779773</v>
+      </c>
+      <c r="AY58" t="inlineStr">
+        <is>
+          <t>0.9951456310679612, 1.0, 0.9951690821256038, 0.9951690821256038, 0.9951690821256038, 1.0, 0.9951690821256038</t>
+        </is>
+      </c>
+      <c r="AZ58" t="n">
+        <v>0.9965459942243395</v>
+      </c>
+      <c r="BA58" t="n">
+        <v>0.9951690821256038</v>
+      </c>
+      <c r="BB58" t="n">
+        <v>0.002184519446236978</v>
+      </c>
+      <c r="BC58" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="BD58" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE58" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF58" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG58" t="inlineStr">
+        <is>
+          <t>0.9999784157133607, 1.0, 0.9999785204914512, 0.9999785204914512, 0.9999785204914511, 1.0, 0.9999785204914511</t>
+        </is>
+      </c>
+      <c r="BH58" t="n">
+        <v>0.999984642525595</v>
+      </c>
+      <c r="BI58" t="n">
+        <v>0.9999785204914512</v>
+      </c>
+      <c r="BJ58" t="n">
+        <v>9.712984233463661e-06</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>no_fragmentation</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>LGBMClassifier_no_fragmentation_Stk_diam</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>{'estimator': LGBMClassifier(), 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': (), 'passthrough_features': ('wettability', 'inclination', 'volume_fraction'), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>0.9333333333333333</v>
+      </c>
+      <c r="F59" t="n">
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="G59" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H59" t="n">
+        <v>0.8780487804878048</v>
+      </c>
+      <c r="I59" t="n">
+        <v>0.9854545454545455</v>
+      </c>
+      <c r="J59" t="n">
+        <v>1</v>
+      </c>
+      <c r="K59" t="n">
+        <v>1</v>
+      </c>
+      <c r="L59" t="n">
+        <v>1</v>
+      </c>
+      <c r="M59" t="n">
+        <v>1</v>
+      </c>
+      <c r="N59" t="n">
+        <v>1</v>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>0.019602537155151367, 0.014482259750366211, 0.02073359489440918, 0.01558375358581543, 0.014885902404785156, 0.013393163681030273, 0.015613317489624023</t>
+        </is>
+      </c>
+      <c r="P59" t="n">
+        <v>0.01632778985159738</v>
+      </c>
+      <c r="Q59" t="n">
+        <v>0.01558375358581543</v>
+      </c>
+      <c r="R59" t="n">
+        <v>0.002543793573807909</v>
+      </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>0.009006738662719727, 0.006963491439819336, 0.007121086120605469, 0.00627446174621582, 0.012955904006958008, 0.0137939453125, 0.010265588760375977</t>
+        </is>
+      </c>
+      <c r="T59" t="n">
+        <v>0.009483030864170619</v>
+      </c>
+      <c r="U59" t="n">
+        <v>0.009006738662719727</v>
+      </c>
+      <c r="V59" t="n">
+        <v>0.002769885506555768</v>
+      </c>
+      <c r="W59" t="inlineStr">
+        <is>
+          <t>0.8518518518518519, 0.9056603773584906, 0.9433962264150944, 0.8867924528301887, 0.9245283018867925, 0.9245283018867925, 0.9433962264150944</t>
+        </is>
+      </c>
+      <c r="X59" t="n">
+        <v>0.9114505340920437</v>
+      </c>
+      <c r="Y59" t="n">
+        <v>0.9245283018867925</v>
+      </c>
+      <c r="Z59" t="n">
+        <v>0.03065163791537664</v>
+      </c>
+      <c r="AA59" t="inlineStr">
+        <is>
+          <t>0.6666666666666667, 0.8275862068965518, 0.88, 0.7999999999999999, 0.8461538461538461, 0.8571428571428571, 0.896551724137931</t>
+        </is>
+      </c>
+      <c r="AB59" t="n">
+        <v>0.8248716144282646</v>
+      </c>
+      <c r="AC59" t="n">
+        <v>0.8461538461538461</v>
+      </c>
+      <c r="AD59" t="n">
+        <v>0.07103954153456497</v>
+      </c>
+      <c r="AE59" t="inlineStr">
+        <is>
+          <t>0.8888888888888888, 0.8, 1.0, 0.75, 0.9166666666666666, 0.8571428571428571, 0.8666666666666667</t>
+        </is>
+      </c>
+      <c r="AF59" t="n">
+        <v>0.8684807256235827</v>
+      </c>
+      <c r="AG59" t="n">
+        <v>0.8666666666666667</v>
+      </c>
+      <c r="AH59" t="n">
+        <v>0.07454129035294924</v>
+      </c>
+      <c r="AI59" t="inlineStr">
+        <is>
+          <t>0.5333333333333333, 0.8571428571428571, 0.7857142857142857, 0.8571428571428571, 0.7857142857142857, 0.8571428571428571, 0.9285714285714286</t>
+        </is>
+      </c>
+      <c r="AJ59" t="n">
+        <v>0.8006802721088435</v>
+      </c>
+      <c r="AK59" t="n">
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="AL59" t="n">
+        <v>0.1182265172078387</v>
+      </c>
+      <c r="AM59" t="inlineStr">
+        <is>
+          <t>0.958974358974359, 0.9322344322344323, 0.990842490842491, 0.9377289377289377, 0.9816849816849818, 0.9139194139194139, 0.9816849816849818</t>
+        </is>
+      </c>
+      <c r="AN59" t="n">
+        <v>0.9567242281527996</v>
+      </c>
+      <c r="AO59" t="n">
+        <v>0.958974358974359</v>
+      </c>
+      <c r="AP59" t="n">
+        <v>0.02727641748426234</v>
+      </c>
+      <c r="AQ59" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="AR59" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS59" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU59" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="AV59" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW59" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY59" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="AZ59" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA59" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB59" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC59" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="BD59" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE59" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF59" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG59" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="BH59" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI59" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ59" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
[ADD] Ablation study updates
</commit_message>
<xml_diff>
--- a/results/metrics_modelling3.xlsx
+++ b/results/metrics_modelling3.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BJ59"/>
+  <dimension ref="A1:DH60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -739,6 +739,256 @@
           <t>cv_train_roc_auc_std</t>
         </is>
       </c>
+      <c r="BK1" s="1" t="inlineStr">
+        <is>
+          <t>holdout_test_f1_macro</t>
+        </is>
+      </c>
+      <c r="BL1" s="1" t="inlineStr">
+        <is>
+          <t>holdout_test_accuracy_balanced</t>
+        </is>
+      </c>
+      <c r="BM1" s="1" t="inlineStr">
+        <is>
+          <t>holdout_test_precision_class_0</t>
+        </is>
+      </c>
+      <c r="BN1" s="1" t="inlineStr">
+        <is>
+          <t>holdout_test_recall_class_0</t>
+        </is>
+      </c>
+      <c r="BO1" s="1" t="inlineStr">
+        <is>
+          <t>holdout_test_f1_class_0</t>
+        </is>
+      </c>
+      <c r="BP1" s="1" t="inlineStr">
+        <is>
+          <t>holdout_train_f1_macro</t>
+        </is>
+      </c>
+      <c r="BQ1" s="1" t="inlineStr">
+        <is>
+          <t>holdout_train_accuracy_balanced</t>
+        </is>
+      </c>
+      <c r="BR1" s="1" t="inlineStr">
+        <is>
+          <t>holdout_train_precision_class_0</t>
+        </is>
+      </c>
+      <c r="BS1" s="1" t="inlineStr">
+        <is>
+          <t>holdout_train_recall_class_0</t>
+        </is>
+      </c>
+      <c r="BT1" s="1" t="inlineStr">
+        <is>
+          <t>holdout_train_f1_class_0</t>
+        </is>
+      </c>
+      <c r="BU1" s="1" t="inlineStr">
+        <is>
+          <t>cv_test_accuracy_balanced</t>
+        </is>
+      </c>
+      <c r="BV1" s="1" t="inlineStr">
+        <is>
+          <t>cv_test_accuracy_balanced_mean</t>
+        </is>
+      </c>
+      <c r="BW1" s="1" t="inlineStr">
+        <is>
+          <t>cv_test_accuracy_balanced_median</t>
+        </is>
+      </c>
+      <c r="BX1" s="1" t="inlineStr">
+        <is>
+          <t>cv_test_accuracy_balanced_std</t>
+        </is>
+      </c>
+      <c r="BY1" s="1" t="inlineStr">
+        <is>
+          <t>cv_test_f1_class_0</t>
+        </is>
+      </c>
+      <c r="BZ1" s="1" t="inlineStr">
+        <is>
+          <t>cv_test_f1_class_0_mean</t>
+        </is>
+      </c>
+      <c r="CA1" s="1" t="inlineStr">
+        <is>
+          <t>cv_test_f1_class_0_median</t>
+        </is>
+      </c>
+      <c r="CB1" s="1" t="inlineStr">
+        <is>
+          <t>cv_test_f1_class_0_std</t>
+        </is>
+      </c>
+      <c r="CC1" s="1" t="inlineStr">
+        <is>
+          <t>cv_test_f1_macro</t>
+        </is>
+      </c>
+      <c r="CD1" s="1" t="inlineStr">
+        <is>
+          <t>cv_test_f1_macro_mean</t>
+        </is>
+      </c>
+      <c r="CE1" s="1" t="inlineStr">
+        <is>
+          <t>cv_test_f1_macro_median</t>
+        </is>
+      </c>
+      <c r="CF1" s="1" t="inlineStr">
+        <is>
+          <t>cv_test_f1_macro_std</t>
+        </is>
+      </c>
+      <c r="CG1" s="1" t="inlineStr">
+        <is>
+          <t>cv_test_precision_class_0</t>
+        </is>
+      </c>
+      <c r="CH1" s="1" t="inlineStr">
+        <is>
+          <t>cv_test_precision_class_0_mean</t>
+        </is>
+      </c>
+      <c r="CI1" s="1" t="inlineStr">
+        <is>
+          <t>cv_test_precision_class_0_median</t>
+        </is>
+      </c>
+      <c r="CJ1" s="1" t="inlineStr">
+        <is>
+          <t>cv_test_precision_class_0_std</t>
+        </is>
+      </c>
+      <c r="CK1" s="1" t="inlineStr">
+        <is>
+          <t>cv_test_recall_class_0</t>
+        </is>
+      </c>
+      <c r="CL1" s="1" t="inlineStr">
+        <is>
+          <t>cv_test_recall_class_0_mean</t>
+        </is>
+      </c>
+      <c r="CM1" s="1" t="inlineStr">
+        <is>
+          <t>cv_test_recall_class_0_median</t>
+        </is>
+      </c>
+      <c r="CN1" s="1" t="inlineStr">
+        <is>
+          <t>cv_test_recall_class_0_std</t>
+        </is>
+      </c>
+      <c r="CO1" s="1" t="inlineStr">
+        <is>
+          <t>cv_train_accuracy_balanced</t>
+        </is>
+      </c>
+      <c r="CP1" s="1" t="inlineStr">
+        <is>
+          <t>cv_train_accuracy_balanced_mean</t>
+        </is>
+      </c>
+      <c r="CQ1" s="1" t="inlineStr">
+        <is>
+          <t>cv_train_accuracy_balanced_median</t>
+        </is>
+      </c>
+      <c r="CR1" s="1" t="inlineStr">
+        <is>
+          <t>cv_train_accuracy_balanced_std</t>
+        </is>
+      </c>
+      <c r="CS1" s="1" t="inlineStr">
+        <is>
+          <t>cv_train_f1_class_0</t>
+        </is>
+      </c>
+      <c r="CT1" s="1" t="inlineStr">
+        <is>
+          <t>cv_train_f1_class_0_mean</t>
+        </is>
+      </c>
+      <c r="CU1" s="1" t="inlineStr">
+        <is>
+          <t>cv_train_f1_class_0_median</t>
+        </is>
+      </c>
+      <c r="CV1" s="1" t="inlineStr">
+        <is>
+          <t>cv_train_f1_class_0_std</t>
+        </is>
+      </c>
+      <c r="CW1" s="1" t="inlineStr">
+        <is>
+          <t>cv_train_f1_macro</t>
+        </is>
+      </c>
+      <c r="CX1" s="1" t="inlineStr">
+        <is>
+          <t>cv_train_f1_macro_mean</t>
+        </is>
+      </c>
+      <c r="CY1" s="1" t="inlineStr">
+        <is>
+          <t>cv_train_f1_macro_median</t>
+        </is>
+      </c>
+      <c r="CZ1" s="1" t="inlineStr">
+        <is>
+          <t>cv_train_f1_macro_std</t>
+        </is>
+      </c>
+      <c r="DA1" s="1" t="inlineStr">
+        <is>
+          <t>cv_train_precision_class_0</t>
+        </is>
+      </c>
+      <c r="DB1" s="1" t="inlineStr">
+        <is>
+          <t>cv_train_precision_class_0_mean</t>
+        </is>
+      </c>
+      <c r="DC1" s="1" t="inlineStr">
+        <is>
+          <t>cv_train_precision_class_0_median</t>
+        </is>
+      </c>
+      <c r="DD1" s="1" t="inlineStr">
+        <is>
+          <t>cv_train_precision_class_0_std</t>
+        </is>
+      </c>
+      <c r="DE1" s="1" t="inlineStr">
+        <is>
+          <t>cv_train_recall_class_0</t>
+        </is>
+      </c>
+      <c r="DF1" s="1" t="inlineStr">
+        <is>
+          <t>cv_train_recall_class_0_mean</t>
+        </is>
+      </c>
+      <c r="DG1" s="1" t="inlineStr">
+        <is>
+          <t>cv_train_recall_class_0_median</t>
+        </is>
+      </c>
+      <c r="DH1" s="1" t="inlineStr">
+        <is>
+          <t>cv_train_recall_class_0_std</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -959,6 +1209,56 @@
       <c r="BJ2" t="n">
         <v>0.006878900544216725</v>
       </c>
+      <c r="BK2" t="inlineStr"/>
+      <c r="BL2" t="inlineStr"/>
+      <c r="BM2" t="inlineStr"/>
+      <c r="BN2" t="inlineStr"/>
+      <c r="BO2" t="inlineStr"/>
+      <c r="BP2" t="inlineStr"/>
+      <c r="BQ2" t="inlineStr"/>
+      <c r="BR2" t="inlineStr"/>
+      <c r="BS2" t="inlineStr"/>
+      <c r="BT2" t="inlineStr"/>
+      <c r="BU2" t="inlineStr"/>
+      <c r="BV2" t="inlineStr"/>
+      <c r="BW2" t="inlineStr"/>
+      <c r="BX2" t="inlineStr"/>
+      <c r="BY2" t="inlineStr"/>
+      <c r="BZ2" t="inlineStr"/>
+      <c r="CA2" t="inlineStr"/>
+      <c r="CB2" t="inlineStr"/>
+      <c r="CC2" t="inlineStr"/>
+      <c r="CD2" t="inlineStr"/>
+      <c r="CE2" t="inlineStr"/>
+      <c r="CF2" t="inlineStr"/>
+      <c r="CG2" t="inlineStr"/>
+      <c r="CH2" t="inlineStr"/>
+      <c r="CI2" t="inlineStr"/>
+      <c r="CJ2" t="inlineStr"/>
+      <c r="CK2" t="inlineStr"/>
+      <c r="CL2" t="inlineStr"/>
+      <c r="CM2" t="inlineStr"/>
+      <c r="CN2" t="inlineStr"/>
+      <c r="CO2" t="inlineStr"/>
+      <c r="CP2" t="inlineStr"/>
+      <c r="CQ2" t="inlineStr"/>
+      <c r="CR2" t="inlineStr"/>
+      <c r="CS2" t="inlineStr"/>
+      <c r="CT2" t="inlineStr"/>
+      <c r="CU2" t="inlineStr"/>
+      <c r="CV2" t="inlineStr"/>
+      <c r="CW2" t="inlineStr"/>
+      <c r="CX2" t="inlineStr"/>
+      <c r="CY2" t="inlineStr"/>
+      <c r="CZ2" t="inlineStr"/>
+      <c r="DA2" t="inlineStr"/>
+      <c r="DB2" t="inlineStr"/>
+      <c r="DC2" t="inlineStr"/>
+      <c r="DD2" t="inlineStr"/>
+      <c r="DE2" t="inlineStr"/>
+      <c r="DF2" t="inlineStr"/>
+      <c r="DG2" t="inlineStr"/>
+      <c r="DH2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1179,6 +1479,56 @@
       <c r="BJ3" t="n">
         <v>0.005635428789683134</v>
       </c>
+      <c r="BK3" t="inlineStr"/>
+      <c r="BL3" t="inlineStr"/>
+      <c r="BM3" t="inlineStr"/>
+      <c r="BN3" t="inlineStr"/>
+      <c r="BO3" t="inlineStr"/>
+      <c r="BP3" t="inlineStr"/>
+      <c r="BQ3" t="inlineStr"/>
+      <c r="BR3" t="inlineStr"/>
+      <c r="BS3" t="inlineStr"/>
+      <c r="BT3" t="inlineStr"/>
+      <c r="BU3" t="inlineStr"/>
+      <c r="BV3" t="inlineStr"/>
+      <c r="BW3" t="inlineStr"/>
+      <c r="BX3" t="inlineStr"/>
+      <c r="BY3" t="inlineStr"/>
+      <c r="BZ3" t="inlineStr"/>
+      <c r="CA3" t="inlineStr"/>
+      <c r="CB3" t="inlineStr"/>
+      <c r="CC3" t="inlineStr"/>
+      <c r="CD3" t="inlineStr"/>
+      <c r="CE3" t="inlineStr"/>
+      <c r="CF3" t="inlineStr"/>
+      <c r="CG3" t="inlineStr"/>
+      <c r="CH3" t="inlineStr"/>
+      <c r="CI3" t="inlineStr"/>
+      <c r="CJ3" t="inlineStr"/>
+      <c r="CK3" t="inlineStr"/>
+      <c r="CL3" t="inlineStr"/>
+      <c r="CM3" t="inlineStr"/>
+      <c r="CN3" t="inlineStr"/>
+      <c r="CO3" t="inlineStr"/>
+      <c r="CP3" t="inlineStr"/>
+      <c r="CQ3" t="inlineStr"/>
+      <c r="CR3" t="inlineStr"/>
+      <c r="CS3" t="inlineStr"/>
+      <c r="CT3" t="inlineStr"/>
+      <c r="CU3" t="inlineStr"/>
+      <c r="CV3" t="inlineStr"/>
+      <c r="CW3" t="inlineStr"/>
+      <c r="CX3" t="inlineStr"/>
+      <c r="CY3" t="inlineStr"/>
+      <c r="CZ3" t="inlineStr"/>
+      <c r="DA3" t="inlineStr"/>
+      <c r="DB3" t="inlineStr"/>
+      <c r="DC3" t="inlineStr"/>
+      <c r="DD3" t="inlineStr"/>
+      <c r="DE3" t="inlineStr"/>
+      <c r="DF3" t="inlineStr"/>
+      <c r="DG3" t="inlineStr"/>
+      <c r="DH3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1399,6 +1749,56 @@
       <c r="BJ4" t="n">
         <v>0.007603060102699606</v>
       </c>
+      <c r="BK4" t="inlineStr"/>
+      <c r="BL4" t="inlineStr"/>
+      <c r="BM4" t="inlineStr"/>
+      <c r="BN4" t="inlineStr"/>
+      <c r="BO4" t="inlineStr"/>
+      <c r="BP4" t="inlineStr"/>
+      <c r="BQ4" t="inlineStr"/>
+      <c r="BR4" t="inlineStr"/>
+      <c r="BS4" t="inlineStr"/>
+      <c r="BT4" t="inlineStr"/>
+      <c r="BU4" t="inlineStr"/>
+      <c r="BV4" t="inlineStr"/>
+      <c r="BW4" t="inlineStr"/>
+      <c r="BX4" t="inlineStr"/>
+      <c r="BY4" t="inlineStr"/>
+      <c r="BZ4" t="inlineStr"/>
+      <c r="CA4" t="inlineStr"/>
+      <c r="CB4" t="inlineStr"/>
+      <c r="CC4" t="inlineStr"/>
+      <c r="CD4" t="inlineStr"/>
+      <c r="CE4" t="inlineStr"/>
+      <c r="CF4" t="inlineStr"/>
+      <c r="CG4" t="inlineStr"/>
+      <c r="CH4" t="inlineStr"/>
+      <c r="CI4" t="inlineStr"/>
+      <c r="CJ4" t="inlineStr"/>
+      <c r="CK4" t="inlineStr"/>
+      <c r="CL4" t="inlineStr"/>
+      <c r="CM4" t="inlineStr"/>
+      <c r="CN4" t="inlineStr"/>
+      <c r="CO4" t="inlineStr"/>
+      <c r="CP4" t="inlineStr"/>
+      <c r="CQ4" t="inlineStr"/>
+      <c r="CR4" t="inlineStr"/>
+      <c r="CS4" t="inlineStr"/>
+      <c r="CT4" t="inlineStr"/>
+      <c r="CU4" t="inlineStr"/>
+      <c r="CV4" t="inlineStr"/>
+      <c r="CW4" t="inlineStr"/>
+      <c r="CX4" t="inlineStr"/>
+      <c r="CY4" t="inlineStr"/>
+      <c r="CZ4" t="inlineStr"/>
+      <c r="DA4" t="inlineStr"/>
+      <c r="DB4" t="inlineStr"/>
+      <c r="DC4" t="inlineStr"/>
+      <c r="DD4" t="inlineStr"/>
+      <c r="DE4" t="inlineStr"/>
+      <c r="DF4" t="inlineStr"/>
+      <c r="DG4" t="inlineStr"/>
+      <c r="DH4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1619,6 +2019,56 @@
       <c r="BJ5" t="n">
         <v>0.005604009792409489</v>
       </c>
+      <c r="BK5" t="inlineStr"/>
+      <c r="BL5" t="inlineStr"/>
+      <c r="BM5" t="inlineStr"/>
+      <c r="BN5" t="inlineStr"/>
+      <c r="BO5" t="inlineStr"/>
+      <c r="BP5" t="inlineStr"/>
+      <c r="BQ5" t="inlineStr"/>
+      <c r="BR5" t="inlineStr"/>
+      <c r="BS5" t="inlineStr"/>
+      <c r="BT5" t="inlineStr"/>
+      <c r="BU5" t="inlineStr"/>
+      <c r="BV5" t="inlineStr"/>
+      <c r="BW5" t="inlineStr"/>
+      <c r="BX5" t="inlineStr"/>
+      <c r="BY5" t="inlineStr"/>
+      <c r="BZ5" t="inlineStr"/>
+      <c r="CA5" t="inlineStr"/>
+      <c r="CB5" t="inlineStr"/>
+      <c r="CC5" t="inlineStr"/>
+      <c r="CD5" t="inlineStr"/>
+      <c r="CE5" t="inlineStr"/>
+      <c r="CF5" t="inlineStr"/>
+      <c r="CG5" t="inlineStr"/>
+      <c r="CH5" t="inlineStr"/>
+      <c r="CI5" t="inlineStr"/>
+      <c r="CJ5" t="inlineStr"/>
+      <c r="CK5" t="inlineStr"/>
+      <c r="CL5" t="inlineStr"/>
+      <c r="CM5" t="inlineStr"/>
+      <c r="CN5" t="inlineStr"/>
+      <c r="CO5" t="inlineStr"/>
+      <c r="CP5" t="inlineStr"/>
+      <c r="CQ5" t="inlineStr"/>
+      <c r="CR5" t="inlineStr"/>
+      <c r="CS5" t="inlineStr"/>
+      <c r="CT5" t="inlineStr"/>
+      <c r="CU5" t="inlineStr"/>
+      <c r="CV5" t="inlineStr"/>
+      <c r="CW5" t="inlineStr"/>
+      <c r="CX5" t="inlineStr"/>
+      <c r="CY5" t="inlineStr"/>
+      <c r="CZ5" t="inlineStr"/>
+      <c r="DA5" t="inlineStr"/>
+      <c r="DB5" t="inlineStr"/>
+      <c r="DC5" t="inlineStr"/>
+      <c r="DD5" t="inlineStr"/>
+      <c r="DE5" t="inlineStr"/>
+      <c r="DF5" t="inlineStr"/>
+      <c r="DG5" t="inlineStr"/>
+      <c r="DH5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1839,6 +2289,56 @@
       <c r="BJ6" t="n">
         <v>0.002061603425119283</v>
       </c>
+      <c r="BK6" t="inlineStr"/>
+      <c r="BL6" t="inlineStr"/>
+      <c r="BM6" t="inlineStr"/>
+      <c r="BN6" t="inlineStr"/>
+      <c r="BO6" t="inlineStr"/>
+      <c r="BP6" t="inlineStr"/>
+      <c r="BQ6" t="inlineStr"/>
+      <c r="BR6" t="inlineStr"/>
+      <c r="BS6" t="inlineStr"/>
+      <c r="BT6" t="inlineStr"/>
+      <c r="BU6" t="inlineStr"/>
+      <c r="BV6" t="inlineStr"/>
+      <c r="BW6" t="inlineStr"/>
+      <c r="BX6" t="inlineStr"/>
+      <c r="BY6" t="inlineStr"/>
+      <c r="BZ6" t="inlineStr"/>
+      <c r="CA6" t="inlineStr"/>
+      <c r="CB6" t="inlineStr"/>
+      <c r="CC6" t="inlineStr"/>
+      <c r="CD6" t="inlineStr"/>
+      <c r="CE6" t="inlineStr"/>
+      <c r="CF6" t="inlineStr"/>
+      <c r="CG6" t="inlineStr"/>
+      <c r="CH6" t="inlineStr"/>
+      <c r="CI6" t="inlineStr"/>
+      <c r="CJ6" t="inlineStr"/>
+      <c r="CK6" t="inlineStr"/>
+      <c r="CL6" t="inlineStr"/>
+      <c r="CM6" t="inlineStr"/>
+      <c r="CN6" t="inlineStr"/>
+      <c r="CO6" t="inlineStr"/>
+      <c r="CP6" t="inlineStr"/>
+      <c r="CQ6" t="inlineStr"/>
+      <c r="CR6" t="inlineStr"/>
+      <c r="CS6" t="inlineStr"/>
+      <c r="CT6" t="inlineStr"/>
+      <c r="CU6" t="inlineStr"/>
+      <c r="CV6" t="inlineStr"/>
+      <c r="CW6" t="inlineStr"/>
+      <c r="CX6" t="inlineStr"/>
+      <c r="CY6" t="inlineStr"/>
+      <c r="CZ6" t="inlineStr"/>
+      <c r="DA6" t="inlineStr"/>
+      <c r="DB6" t="inlineStr"/>
+      <c r="DC6" t="inlineStr"/>
+      <c r="DD6" t="inlineStr"/>
+      <c r="DE6" t="inlineStr"/>
+      <c r="DF6" t="inlineStr"/>
+      <c r="DG6" t="inlineStr"/>
+      <c r="DH6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2059,6 +2559,56 @@
       <c r="BJ7" t="n">
         <v>0.002556083322909469</v>
       </c>
+      <c r="BK7" t="inlineStr"/>
+      <c r="BL7" t="inlineStr"/>
+      <c r="BM7" t="inlineStr"/>
+      <c r="BN7" t="inlineStr"/>
+      <c r="BO7" t="inlineStr"/>
+      <c r="BP7" t="inlineStr"/>
+      <c r="BQ7" t="inlineStr"/>
+      <c r="BR7" t="inlineStr"/>
+      <c r="BS7" t="inlineStr"/>
+      <c r="BT7" t="inlineStr"/>
+      <c r="BU7" t="inlineStr"/>
+      <c r="BV7" t="inlineStr"/>
+      <c r="BW7" t="inlineStr"/>
+      <c r="BX7" t="inlineStr"/>
+      <c r="BY7" t="inlineStr"/>
+      <c r="BZ7" t="inlineStr"/>
+      <c r="CA7" t="inlineStr"/>
+      <c r="CB7" t="inlineStr"/>
+      <c r="CC7" t="inlineStr"/>
+      <c r="CD7" t="inlineStr"/>
+      <c r="CE7" t="inlineStr"/>
+      <c r="CF7" t="inlineStr"/>
+      <c r="CG7" t="inlineStr"/>
+      <c r="CH7" t="inlineStr"/>
+      <c r="CI7" t="inlineStr"/>
+      <c r="CJ7" t="inlineStr"/>
+      <c r="CK7" t="inlineStr"/>
+      <c r="CL7" t="inlineStr"/>
+      <c r="CM7" t="inlineStr"/>
+      <c r="CN7" t="inlineStr"/>
+      <c r="CO7" t="inlineStr"/>
+      <c r="CP7" t="inlineStr"/>
+      <c r="CQ7" t="inlineStr"/>
+      <c r="CR7" t="inlineStr"/>
+      <c r="CS7" t="inlineStr"/>
+      <c r="CT7" t="inlineStr"/>
+      <c r="CU7" t="inlineStr"/>
+      <c r="CV7" t="inlineStr"/>
+      <c r="CW7" t="inlineStr"/>
+      <c r="CX7" t="inlineStr"/>
+      <c r="CY7" t="inlineStr"/>
+      <c r="CZ7" t="inlineStr"/>
+      <c r="DA7" t="inlineStr"/>
+      <c r="DB7" t="inlineStr"/>
+      <c r="DC7" t="inlineStr"/>
+      <c r="DD7" t="inlineStr"/>
+      <c r="DE7" t="inlineStr"/>
+      <c r="DF7" t="inlineStr"/>
+      <c r="DG7" t="inlineStr"/>
+      <c r="DH7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2279,6 +2829,56 @@
       <c r="BJ8" t="n">
         <v>0.005460178801644405</v>
       </c>
+      <c r="BK8" t="inlineStr"/>
+      <c r="BL8" t="inlineStr"/>
+      <c r="BM8" t="inlineStr"/>
+      <c r="BN8" t="inlineStr"/>
+      <c r="BO8" t="inlineStr"/>
+      <c r="BP8" t="inlineStr"/>
+      <c r="BQ8" t="inlineStr"/>
+      <c r="BR8" t="inlineStr"/>
+      <c r="BS8" t="inlineStr"/>
+      <c r="BT8" t="inlineStr"/>
+      <c r="BU8" t="inlineStr"/>
+      <c r="BV8" t="inlineStr"/>
+      <c r="BW8" t="inlineStr"/>
+      <c r="BX8" t="inlineStr"/>
+      <c r="BY8" t="inlineStr"/>
+      <c r="BZ8" t="inlineStr"/>
+      <c r="CA8" t="inlineStr"/>
+      <c r="CB8" t="inlineStr"/>
+      <c r="CC8" t="inlineStr"/>
+      <c r="CD8" t="inlineStr"/>
+      <c r="CE8" t="inlineStr"/>
+      <c r="CF8" t="inlineStr"/>
+      <c r="CG8" t="inlineStr"/>
+      <c r="CH8" t="inlineStr"/>
+      <c r="CI8" t="inlineStr"/>
+      <c r="CJ8" t="inlineStr"/>
+      <c r="CK8" t="inlineStr"/>
+      <c r="CL8" t="inlineStr"/>
+      <c r="CM8" t="inlineStr"/>
+      <c r="CN8" t="inlineStr"/>
+      <c r="CO8" t="inlineStr"/>
+      <c r="CP8" t="inlineStr"/>
+      <c r="CQ8" t="inlineStr"/>
+      <c r="CR8" t="inlineStr"/>
+      <c r="CS8" t="inlineStr"/>
+      <c r="CT8" t="inlineStr"/>
+      <c r="CU8" t="inlineStr"/>
+      <c r="CV8" t="inlineStr"/>
+      <c r="CW8" t="inlineStr"/>
+      <c r="CX8" t="inlineStr"/>
+      <c r="CY8" t="inlineStr"/>
+      <c r="CZ8" t="inlineStr"/>
+      <c r="DA8" t="inlineStr"/>
+      <c r="DB8" t="inlineStr"/>
+      <c r="DC8" t="inlineStr"/>
+      <c r="DD8" t="inlineStr"/>
+      <c r="DE8" t="inlineStr"/>
+      <c r="DF8" t="inlineStr"/>
+      <c r="DG8" t="inlineStr"/>
+      <c r="DH8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2499,6 +3099,56 @@
       <c r="BJ9" t="n">
         <v>0.002988427262158605</v>
       </c>
+      <c r="BK9" t="inlineStr"/>
+      <c r="BL9" t="inlineStr"/>
+      <c r="BM9" t="inlineStr"/>
+      <c r="BN9" t="inlineStr"/>
+      <c r="BO9" t="inlineStr"/>
+      <c r="BP9" t="inlineStr"/>
+      <c r="BQ9" t="inlineStr"/>
+      <c r="BR9" t="inlineStr"/>
+      <c r="BS9" t="inlineStr"/>
+      <c r="BT9" t="inlineStr"/>
+      <c r="BU9" t="inlineStr"/>
+      <c r="BV9" t="inlineStr"/>
+      <c r="BW9" t="inlineStr"/>
+      <c r="BX9" t="inlineStr"/>
+      <c r="BY9" t="inlineStr"/>
+      <c r="BZ9" t="inlineStr"/>
+      <c r="CA9" t="inlineStr"/>
+      <c r="CB9" t="inlineStr"/>
+      <c r="CC9" t="inlineStr"/>
+      <c r="CD9" t="inlineStr"/>
+      <c r="CE9" t="inlineStr"/>
+      <c r="CF9" t="inlineStr"/>
+      <c r="CG9" t="inlineStr"/>
+      <c r="CH9" t="inlineStr"/>
+      <c r="CI9" t="inlineStr"/>
+      <c r="CJ9" t="inlineStr"/>
+      <c r="CK9" t="inlineStr"/>
+      <c r="CL9" t="inlineStr"/>
+      <c r="CM9" t="inlineStr"/>
+      <c r="CN9" t="inlineStr"/>
+      <c r="CO9" t="inlineStr"/>
+      <c r="CP9" t="inlineStr"/>
+      <c r="CQ9" t="inlineStr"/>
+      <c r="CR9" t="inlineStr"/>
+      <c r="CS9" t="inlineStr"/>
+      <c r="CT9" t="inlineStr"/>
+      <c r="CU9" t="inlineStr"/>
+      <c r="CV9" t="inlineStr"/>
+      <c r="CW9" t="inlineStr"/>
+      <c r="CX9" t="inlineStr"/>
+      <c r="CY9" t="inlineStr"/>
+      <c r="CZ9" t="inlineStr"/>
+      <c r="DA9" t="inlineStr"/>
+      <c r="DB9" t="inlineStr"/>
+      <c r="DC9" t="inlineStr"/>
+      <c r="DD9" t="inlineStr"/>
+      <c r="DE9" t="inlineStr"/>
+      <c r="DF9" t="inlineStr"/>
+      <c r="DG9" t="inlineStr"/>
+      <c r="DH9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2719,6 +3369,56 @@
       <c r="BJ10" t="n">
         <v>0.0005871770933261723</v>
       </c>
+      <c r="BK10" t="inlineStr"/>
+      <c r="BL10" t="inlineStr"/>
+      <c r="BM10" t="inlineStr"/>
+      <c r="BN10" t="inlineStr"/>
+      <c r="BO10" t="inlineStr"/>
+      <c r="BP10" t="inlineStr"/>
+      <c r="BQ10" t="inlineStr"/>
+      <c r="BR10" t="inlineStr"/>
+      <c r="BS10" t="inlineStr"/>
+      <c r="BT10" t="inlineStr"/>
+      <c r="BU10" t="inlineStr"/>
+      <c r="BV10" t="inlineStr"/>
+      <c r="BW10" t="inlineStr"/>
+      <c r="BX10" t="inlineStr"/>
+      <c r="BY10" t="inlineStr"/>
+      <c r="BZ10" t="inlineStr"/>
+      <c r="CA10" t="inlineStr"/>
+      <c r="CB10" t="inlineStr"/>
+      <c r="CC10" t="inlineStr"/>
+      <c r="CD10" t="inlineStr"/>
+      <c r="CE10" t="inlineStr"/>
+      <c r="CF10" t="inlineStr"/>
+      <c r="CG10" t="inlineStr"/>
+      <c r="CH10" t="inlineStr"/>
+      <c r="CI10" t="inlineStr"/>
+      <c r="CJ10" t="inlineStr"/>
+      <c r="CK10" t="inlineStr"/>
+      <c r="CL10" t="inlineStr"/>
+      <c r="CM10" t="inlineStr"/>
+      <c r="CN10" t="inlineStr"/>
+      <c r="CO10" t="inlineStr"/>
+      <c r="CP10" t="inlineStr"/>
+      <c r="CQ10" t="inlineStr"/>
+      <c r="CR10" t="inlineStr"/>
+      <c r="CS10" t="inlineStr"/>
+      <c r="CT10" t="inlineStr"/>
+      <c r="CU10" t="inlineStr"/>
+      <c r="CV10" t="inlineStr"/>
+      <c r="CW10" t="inlineStr"/>
+      <c r="CX10" t="inlineStr"/>
+      <c r="CY10" t="inlineStr"/>
+      <c r="CZ10" t="inlineStr"/>
+      <c r="DA10" t="inlineStr"/>
+      <c r="DB10" t="inlineStr"/>
+      <c r="DC10" t="inlineStr"/>
+      <c r="DD10" t="inlineStr"/>
+      <c r="DE10" t="inlineStr"/>
+      <c r="DF10" t="inlineStr"/>
+      <c r="DG10" t="inlineStr"/>
+      <c r="DH10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2939,6 +3639,56 @@
       <c r="BJ11" t="n">
         <v>5.274484965747932e-05</v>
       </c>
+      <c r="BK11" t="inlineStr"/>
+      <c r="BL11" t="inlineStr"/>
+      <c r="BM11" t="inlineStr"/>
+      <c r="BN11" t="inlineStr"/>
+      <c r="BO11" t="inlineStr"/>
+      <c r="BP11" t="inlineStr"/>
+      <c r="BQ11" t="inlineStr"/>
+      <c r="BR11" t="inlineStr"/>
+      <c r="BS11" t="inlineStr"/>
+      <c r="BT11" t="inlineStr"/>
+      <c r="BU11" t="inlineStr"/>
+      <c r="BV11" t="inlineStr"/>
+      <c r="BW11" t="inlineStr"/>
+      <c r="BX11" t="inlineStr"/>
+      <c r="BY11" t="inlineStr"/>
+      <c r="BZ11" t="inlineStr"/>
+      <c r="CA11" t="inlineStr"/>
+      <c r="CB11" t="inlineStr"/>
+      <c r="CC11" t="inlineStr"/>
+      <c r="CD11" t="inlineStr"/>
+      <c r="CE11" t="inlineStr"/>
+      <c r="CF11" t="inlineStr"/>
+      <c r="CG11" t="inlineStr"/>
+      <c r="CH11" t="inlineStr"/>
+      <c r="CI11" t="inlineStr"/>
+      <c r="CJ11" t="inlineStr"/>
+      <c r="CK11" t="inlineStr"/>
+      <c r="CL11" t="inlineStr"/>
+      <c r="CM11" t="inlineStr"/>
+      <c r="CN11" t="inlineStr"/>
+      <c r="CO11" t="inlineStr"/>
+      <c r="CP11" t="inlineStr"/>
+      <c r="CQ11" t="inlineStr"/>
+      <c r="CR11" t="inlineStr"/>
+      <c r="CS11" t="inlineStr"/>
+      <c r="CT11" t="inlineStr"/>
+      <c r="CU11" t="inlineStr"/>
+      <c r="CV11" t="inlineStr"/>
+      <c r="CW11" t="inlineStr"/>
+      <c r="CX11" t="inlineStr"/>
+      <c r="CY11" t="inlineStr"/>
+      <c r="CZ11" t="inlineStr"/>
+      <c r="DA11" t="inlineStr"/>
+      <c r="DB11" t="inlineStr"/>
+      <c r="DC11" t="inlineStr"/>
+      <c r="DD11" t="inlineStr"/>
+      <c r="DE11" t="inlineStr"/>
+      <c r="DF11" t="inlineStr"/>
+      <c r="DG11" t="inlineStr"/>
+      <c r="DH11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3169,6 +3919,56 @@
       <c r="BJ12" t="n">
         <v>1.988619454760789e-05</v>
       </c>
+      <c r="BK12" t="inlineStr"/>
+      <c r="BL12" t="inlineStr"/>
+      <c r="BM12" t="inlineStr"/>
+      <c r="BN12" t="inlineStr"/>
+      <c r="BO12" t="inlineStr"/>
+      <c r="BP12" t="inlineStr"/>
+      <c r="BQ12" t="inlineStr"/>
+      <c r="BR12" t="inlineStr"/>
+      <c r="BS12" t="inlineStr"/>
+      <c r="BT12" t="inlineStr"/>
+      <c r="BU12" t="inlineStr"/>
+      <c r="BV12" t="inlineStr"/>
+      <c r="BW12" t="inlineStr"/>
+      <c r="BX12" t="inlineStr"/>
+      <c r="BY12" t="inlineStr"/>
+      <c r="BZ12" t="inlineStr"/>
+      <c r="CA12" t="inlineStr"/>
+      <c r="CB12" t="inlineStr"/>
+      <c r="CC12" t="inlineStr"/>
+      <c r="CD12" t="inlineStr"/>
+      <c r="CE12" t="inlineStr"/>
+      <c r="CF12" t="inlineStr"/>
+      <c r="CG12" t="inlineStr"/>
+      <c r="CH12" t="inlineStr"/>
+      <c r="CI12" t="inlineStr"/>
+      <c r="CJ12" t="inlineStr"/>
+      <c r="CK12" t="inlineStr"/>
+      <c r="CL12" t="inlineStr"/>
+      <c r="CM12" t="inlineStr"/>
+      <c r="CN12" t="inlineStr"/>
+      <c r="CO12" t="inlineStr"/>
+      <c r="CP12" t="inlineStr"/>
+      <c r="CQ12" t="inlineStr"/>
+      <c r="CR12" t="inlineStr"/>
+      <c r="CS12" t="inlineStr"/>
+      <c r="CT12" t="inlineStr"/>
+      <c r="CU12" t="inlineStr"/>
+      <c r="CV12" t="inlineStr"/>
+      <c r="CW12" t="inlineStr"/>
+      <c r="CX12" t="inlineStr"/>
+      <c r="CY12" t="inlineStr"/>
+      <c r="CZ12" t="inlineStr"/>
+      <c r="DA12" t="inlineStr"/>
+      <c r="DB12" t="inlineStr"/>
+      <c r="DC12" t="inlineStr"/>
+      <c r="DD12" t="inlineStr"/>
+      <c r="DE12" t="inlineStr"/>
+      <c r="DF12" t="inlineStr"/>
+      <c r="DG12" t="inlineStr"/>
+      <c r="DH12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3399,6 +4199,56 @@
       <c r="BJ13" t="n">
         <v>4.196248604251576e-17</v>
       </c>
+      <c r="BK13" t="inlineStr"/>
+      <c r="BL13" t="inlineStr"/>
+      <c r="BM13" t="inlineStr"/>
+      <c r="BN13" t="inlineStr"/>
+      <c r="BO13" t="inlineStr"/>
+      <c r="BP13" t="inlineStr"/>
+      <c r="BQ13" t="inlineStr"/>
+      <c r="BR13" t="inlineStr"/>
+      <c r="BS13" t="inlineStr"/>
+      <c r="BT13" t="inlineStr"/>
+      <c r="BU13" t="inlineStr"/>
+      <c r="BV13" t="inlineStr"/>
+      <c r="BW13" t="inlineStr"/>
+      <c r="BX13" t="inlineStr"/>
+      <c r="BY13" t="inlineStr"/>
+      <c r="BZ13" t="inlineStr"/>
+      <c r="CA13" t="inlineStr"/>
+      <c r="CB13" t="inlineStr"/>
+      <c r="CC13" t="inlineStr"/>
+      <c r="CD13" t="inlineStr"/>
+      <c r="CE13" t="inlineStr"/>
+      <c r="CF13" t="inlineStr"/>
+      <c r="CG13" t="inlineStr"/>
+      <c r="CH13" t="inlineStr"/>
+      <c r="CI13" t="inlineStr"/>
+      <c r="CJ13" t="inlineStr"/>
+      <c r="CK13" t="inlineStr"/>
+      <c r="CL13" t="inlineStr"/>
+      <c r="CM13" t="inlineStr"/>
+      <c r="CN13" t="inlineStr"/>
+      <c r="CO13" t="inlineStr"/>
+      <c r="CP13" t="inlineStr"/>
+      <c r="CQ13" t="inlineStr"/>
+      <c r="CR13" t="inlineStr"/>
+      <c r="CS13" t="inlineStr"/>
+      <c r="CT13" t="inlineStr"/>
+      <c r="CU13" t="inlineStr"/>
+      <c r="CV13" t="inlineStr"/>
+      <c r="CW13" t="inlineStr"/>
+      <c r="CX13" t="inlineStr"/>
+      <c r="CY13" t="inlineStr"/>
+      <c r="CZ13" t="inlineStr"/>
+      <c r="DA13" t="inlineStr"/>
+      <c r="DB13" t="inlineStr"/>
+      <c r="DC13" t="inlineStr"/>
+      <c r="DD13" t="inlineStr"/>
+      <c r="DE13" t="inlineStr"/>
+      <c r="DF13" t="inlineStr"/>
+      <c r="DG13" t="inlineStr"/>
+      <c r="DH13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3619,6 +4469,56 @@
       <c r="BJ14" t="n">
         <v>0.007205630596929708</v>
       </c>
+      <c r="BK14" t="inlineStr"/>
+      <c r="BL14" t="inlineStr"/>
+      <c r="BM14" t="inlineStr"/>
+      <c r="BN14" t="inlineStr"/>
+      <c r="BO14" t="inlineStr"/>
+      <c r="BP14" t="inlineStr"/>
+      <c r="BQ14" t="inlineStr"/>
+      <c r="BR14" t="inlineStr"/>
+      <c r="BS14" t="inlineStr"/>
+      <c r="BT14" t="inlineStr"/>
+      <c r="BU14" t="inlineStr"/>
+      <c r="BV14" t="inlineStr"/>
+      <c r="BW14" t="inlineStr"/>
+      <c r="BX14" t="inlineStr"/>
+      <c r="BY14" t="inlineStr"/>
+      <c r="BZ14" t="inlineStr"/>
+      <c r="CA14" t="inlineStr"/>
+      <c r="CB14" t="inlineStr"/>
+      <c r="CC14" t="inlineStr"/>
+      <c r="CD14" t="inlineStr"/>
+      <c r="CE14" t="inlineStr"/>
+      <c r="CF14" t="inlineStr"/>
+      <c r="CG14" t="inlineStr"/>
+      <c r="CH14" t="inlineStr"/>
+      <c r="CI14" t="inlineStr"/>
+      <c r="CJ14" t="inlineStr"/>
+      <c r="CK14" t="inlineStr"/>
+      <c r="CL14" t="inlineStr"/>
+      <c r="CM14" t="inlineStr"/>
+      <c r="CN14" t="inlineStr"/>
+      <c r="CO14" t="inlineStr"/>
+      <c r="CP14" t="inlineStr"/>
+      <c r="CQ14" t="inlineStr"/>
+      <c r="CR14" t="inlineStr"/>
+      <c r="CS14" t="inlineStr"/>
+      <c r="CT14" t="inlineStr"/>
+      <c r="CU14" t="inlineStr"/>
+      <c r="CV14" t="inlineStr"/>
+      <c r="CW14" t="inlineStr"/>
+      <c r="CX14" t="inlineStr"/>
+      <c r="CY14" t="inlineStr"/>
+      <c r="CZ14" t="inlineStr"/>
+      <c r="DA14" t="inlineStr"/>
+      <c r="DB14" t="inlineStr"/>
+      <c r="DC14" t="inlineStr"/>
+      <c r="DD14" t="inlineStr"/>
+      <c r="DE14" t="inlineStr"/>
+      <c r="DF14" t="inlineStr"/>
+      <c r="DG14" t="inlineStr"/>
+      <c r="DH14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3839,6 +4739,56 @@
       <c r="BJ15" t="n">
         <v>0.006311578643324333</v>
       </c>
+      <c r="BK15" t="inlineStr"/>
+      <c r="BL15" t="inlineStr"/>
+      <c r="BM15" t="inlineStr"/>
+      <c r="BN15" t="inlineStr"/>
+      <c r="BO15" t="inlineStr"/>
+      <c r="BP15" t="inlineStr"/>
+      <c r="BQ15" t="inlineStr"/>
+      <c r="BR15" t="inlineStr"/>
+      <c r="BS15" t="inlineStr"/>
+      <c r="BT15" t="inlineStr"/>
+      <c r="BU15" t="inlineStr"/>
+      <c r="BV15" t="inlineStr"/>
+      <c r="BW15" t="inlineStr"/>
+      <c r="BX15" t="inlineStr"/>
+      <c r="BY15" t="inlineStr"/>
+      <c r="BZ15" t="inlineStr"/>
+      <c r="CA15" t="inlineStr"/>
+      <c r="CB15" t="inlineStr"/>
+      <c r="CC15" t="inlineStr"/>
+      <c r="CD15" t="inlineStr"/>
+      <c r="CE15" t="inlineStr"/>
+      <c r="CF15" t="inlineStr"/>
+      <c r="CG15" t="inlineStr"/>
+      <c r="CH15" t="inlineStr"/>
+      <c r="CI15" t="inlineStr"/>
+      <c r="CJ15" t="inlineStr"/>
+      <c r="CK15" t="inlineStr"/>
+      <c r="CL15" t="inlineStr"/>
+      <c r="CM15" t="inlineStr"/>
+      <c r="CN15" t="inlineStr"/>
+      <c r="CO15" t="inlineStr"/>
+      <c r="CP15" t="inlineStr"/>
+      <c r="CQ15" t="inlineStr"/>
+      <c r="CR15" t="inlineStr"/>
+      <c r="CS15" t="inlineStr"/>
+      <c r="CT15" t="inlineStr"/>
+      <c r="CU15" t="inlineStr"/>
+      <c r="CV15" t="inlineStr"/>
+      <c r="CW15" t="inlineStr"/>
+      <c r="CX15" t="inlineStr"/>
+      <c r="CY15" t="inlineStr"/>
+      <c r="CZ15" t="inlineStr"/>
+      <c r="DA15" t="inlineStr"/>
+      <c r="DB15" t="inlineStr"/>
+      <c r="DC15" t="inlineStr"/>
+      <c r="DD15" t="inlineStr"/>
+      <c r="DE15" t="inlineStr"/>
+      <c r="DF15" t="inlineStr"/>
+      <c r="DG15" t="inlineStr"/>
+      <c r="DH15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -4059,6 +5009,56 @@
       <c r="BJ16" t="n">
         <v>0.007001423478172876</v>
       </c>
+      <c r="BK16" t="inlineStr"/>
+      <c r="BL16" t="inlineStr"/>
+      <c r="BM16" t="inlineStr"/>
+      <c r="BN16" t="inlineStr"/>
+      <c r="BO16" t="inlineStr"/>
+      <c r="BP16" t="inlineStr"/>
+      <c r="BQ16" t="inlineStr"/>
+      <c r="BR16" t="inlineStr"/>
+      <c r="BS16" t="inlineStr"/>
+      <c r="BT16" t="inlineStr"/>
+      <c r="BU16" t="inlineStr"/>
+      <c r="BV16" t="inlineStr"/>
+      <c r="BW16" t="inlineStr"/>
+      <c r="BX16" t="inlineStr"/>
+      <c r="BY16" t="inlineStr"/>
+      <c r="BZ16" t="inlineStr"/>
+      <c r="CA16" t="inlineStr"/>
+      <c r="CB16" t="inlineStr"/>
+      <c r="CC16" t="inlineStr"/>
+      <c r="CD16" t="inlineStr"/>
+      <c r="CE16" t="inlineStr"/>
+      <c r="CF16" t="inlineStr"/>
+      <c r="CG16" t="inlineStr"/>
+      <c r="CH16" t="inlineStr"/>
+      <c r="CI16" t="inlineStr"/>
+      <c r="CJ16" t="inlineStr"/>
+      <c r="CK16" t="inlineStr"/>
+      <c r="CL16" t="inlineStr"/>
+      <c r="CM16" t="inlineStr"/>
+      <c r="CN16" t="inlineStr"/>
+      <c r="CO16" t="inlineStr"/>
+      <c r="CP16" t="inlineStr"/>
+      <c r="CQ16" t="inlineStr"/>
+      <c r="CR16" t="inlineStr"/>
+      <c r="CS16" t="inlineStr"/>
+      <c r="CT16" t="inlineStr"/>
+      <c r="CU16" t="inlineStr"/>
+      <c r="CV16" t="inlineStr"/>
+      <c r="CW16" t="inlineStr"/>
+      <c r="CX16" t="inlineStr"/>
+      <c r="CY16" t="inlineStr"/>
+      <c r="CZ16" t="inlineStr"/>
+      <c r="DA16" t="inlineStr"/>
+      <c r="DB16" t="inlineStr"/>
+      <c r="DC16" t="inlineStr"/>
+      <c r="DD16" t="inlineStr"/>
+      <c r="DE16" t="inlineStr"/>
+      <c r="DF16" t="inlineStr"/>
+      <c r="DG16" t="inlineStr"/>
+      <c r="DH16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -4279,6 +5279,56 @@
       <c r="BJ17" t="n">
         <v>0.005684785794350271</v>
       </c>
+      <c r="BK17" t="inlineStr"/>
+      <c r="BL17" t="inlineStr"/>
+      <c r="BM17" t="inlineStr"/>
+      <c r="BN17" t="inlineStr"/>
+      <c r="BO17" t="inlineStr"/>
+      <c r="BP17" t="inlineStr"/>
+      <c r="BQ17" t="inlineStr"/>
+      <c r="BR17" t="inlineStr"/>
+      <c r="BS17" t="inlineStr"/>
+      <c r="BT17" t="inlineStr"/>
+      <c r="BU17" t="inlineStr"/>
+      <c r="BV17" t="inlineStr"/>
+      <c r="BW17" t="inlineStr"/>
+      <c r="BX17" t="inlineStr"/>
+      <c r="BY17" t="inlineStr"/>
+      <c r="BZ17" t="inlineStr"/>
+      <c r="CA17" t="inlineStr"/>
+      <c r="CB17" t="inlineStr"/>
+      <c r="CC17" t="inlineStr"/>
+      <c r="CD17" t="inlineStr"/>
+      <c r="CE17" t="inlineStr"/>
+      <c r="CF17" t="inlineStr"/>
+      <c r="CG17" t="inlineStr"/>
+      <c r="CH17" t="inlineStr"/>
+      <c r="CI17" t="inlineStr"/>
+      <c r="CJ17" t="inlineStr"/>
+      <c r="CK17" t="inlineStr"/>
+      <c r="CL17" t="inlineStr"/>
+      <c r="CM17" t="inlineStr"/>
+      <c r="CN17" t="inlineStr"/>
+      <c r="CO17" t="inlineStr"/>
+      <c r="CP17" t="inlineStr"/>
+      <c r="CQ17" t="inlineStr"/>
+      <c r="CR17" t="inlineStr"/>
+      <c r="CS17" t="inlineStr"/>
+      <c r="CT17" t="inlineStr"/>
+      <c r="CU17" t="inlineStr"/>
+      <c r="CV17" t="inlineStr"/>
+      <c r="CW17" t="inlineStr"/>
+      <c r="CX17" t="inlineStr"/>
+      <c r="CY17" t="inlineStr"/>
+      <c r="CZ17" t="inlineStr"/>
+      <c r="DA17" t="inlineStr"/>
+      <c r="DB17" t="inlineStr"/>
+      <c r="DC17" t="inlineStr"/>
+      <c r="DD17" t="inlineStr"/>
+      <c r="DE17" t="inlineStr"/>
+      <c r="DF17" t="inlineStr"/>
+      <c r="DG17" t="inlineStr"/>
+      <c r="DH17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4499,6 +5549,56 @@
       <c r="BJ18" t="n">
         <v>0.002800999199045301</v>
       </c>
+      <c r="BK18" t="inlineStr"/>
+      <c r="BL18" t="inlineStr"/>
+      <c r="BM18" t="inlineStr"/>
+      <c r="BN18" t="inlineStr"/>
+      <c r="BO18" t="inlineStr"/>
+      <c r="BP18" t="inlineStr"/>
+      <c r="BQ18" t="inlineStr"/>
+      <c r="BR18" t="inlineStr"/>
+      <c r="BS18" t="inlineStr"/>
+      <c r="BT18" t="inlineStr"/>
+      <c r="BU18" t="inlineStr"/>
+      <c r="BV18" t="inlineStr"/>
+      <c r="BW18" t="inlineStr"/>
+      <c r="BX18" t="inlineStr"/>
+      <c r="BY18" t="inlineStr"/>
+      <c r="BZ18" t="inlineStr"/>
+      <c r="CA18" t="inlineStr"/>
+      <c r="CB18" t="inlineStr"/>
+      <c r="CC18" t="inlineStr"/>
+      <c r="CD18" t="inlineStr"/>
+      <c r="CE18" t="inlineStr"/>
+      <c r="CF18" t="inlineStr"/>
+      <c r="CG18" t="inlineStr"/>
+      <c r="CH18" t="inlineStr"/>
+      <c r="CI18" t="inlineStr"/>
+      <c r="CJ18" t="inlineStr"/>
+      <c r="CK18" t="inlineStr"/>
+      <c r="CL18" t="inlineStr"/>
+      <c r="CM18" t="inlineStr"/>
+      <c r="CN18" t="inlineStr"/>
+      <c r="CO18" t="inlineStr"/>
+      <c r="CP18" t="inlineStr"/>
+      <c r="CQ18" t="inlineStr"/>
+      <c r="CR18" t="inlineStr"/>
+      <c r="CS18" t="inlineStr"/>
+      <c r="CT18" t="inlineStr"/>
+      <c r="CU18" t="inlineStr"/>
+      <c r="CV18" t="inlineStr"/>
+      <c r="CW18" t="inlineStr"/>
+      <c r="CX18" t="inlineStr"/>
+      <c r="CY18" t="inlineStr"/>
+      <c r="CZ18" t="inlineStr"/>
+      <c r="DA18" t="inlineStr"/>
+      <c r="DB18" t="inlineStr"/>
+      <c r="DC18" t="inlineStr"/>
+      <c r="DD18" t="inlineStr"/>
+      <c r="DE18" t="inlineStr"/>
+      <c r="DF18" t="inlineStr"/>
+      <c r="DG18" t="inlineStr"/>
+      <c r="DH18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4719,6 +5819,56 @@
       <c r="BJ19" t="n">
         <v>0.004564434495284856</v>
       </c>
+      <c r="BK19" t="inlineStr"/>
+      <c r="BL19" t="inlineStr"/>
+      <c r="BM19" t="inlineStr"/>
+      <c r="BN19" t="inlineStr"/>
+      <c r="BO19" t="inlineStr"/>
+      <c r="BP19" t="inlineStr"/>
+      <c r="BQ19" t="inlineStr"/>
+      <c r="BR19" t="inlineStr"/>
+      <c r="BS19" t="inlineStr"/>
+      <c r="BT19" t="inlineStr"/>
+      <c r="BU19" t="inlineStr"/>
+      <c r="BV19" t="inlineStr"/>
+      <c r="BW19" t="inlineStr"/>
+      <c r="BX19" t="inlineStr"/>
+      <c r="BY19" t="inlineStr"/>
+      <c r="BZ19" t="inlineStr"/>
+      <c r="CA19" t="inlineStr"/>
+      <c r="CB19" t="inlineStr"/>
+      <c r="CC19" t="inlineStr"/>
+      <c r="CD19" t="inlineStr"/>
+      <c r="CE19" t="inlineStr"/>
+      <c r="CF19" t="inlineStr"/>
+      <c r="CG19" t="inlineStr"/>
+      <c r="CH19" t="inlineStr"/>
+      <c r="CI19" t="inlineStr"/>
+      <c r="CJ19" t="inlineStr"/>
+      <c r="CK19" t="inlineStr"/>
+      <c r="CL19" t="inlineStr"/>
+      <c r="CM19" t="inlineStr"/>
+      <c r="CN19" t="inlineStr"/>
+      <c r="CO19" t="inlineStr"/>
+      <c r="CP19" t="inlineStr"/>
+      <c r="CQ19" t="inlineStr"/>
+      <c r="CR19" t="inlineStr"/>
+      <c r="CS19" t="inlineStr"/>
+      <c r="CT19" t="inlineStr"/>
+      <c r="CU19" t="inlineStr"/>
+      <c r="CV19" t="inlineStr"/>
+      <c r="CW19" t="inlineStr"/>
+      <c r="CX19" t="inlineStr"/>
+      <c r="CY19" t="inlineStr"/>
+      <c r="CZ19" t="inlineStr"/>
+      <c r="DA19" t="inlineStr"/>
+      <c r="DB19" t="inlineStr"/>
+      <c r="DC19" t="inlineStr"/>
+      <c r="DD19" t="inlineStr"/>
+      <c r="DE19" t="inlineStr"/>
+      <c r="DF19" t="inlineStr"/>
+      <c r="DG19" t="inlineStr"/>
+      <c r="DH19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4939,6 +6089,56 @@
       <c r="BJ20" t="n">
         <v>0.005477492640031644</v>
       </c>
+      <c r="BK20" t="inlineStr"/>
+      <c r="BL20" t="inlineStr"/>
+      <c r="BM20" t="inlineStr"/>
+      <c r="BN20" t="inlineStr"/>
+      <c r="BO20" t="inlineStr"/>
+      <c r="BP20" t="inlineStr"/>
+      <c r="BQ20" t="inlineStr"/>
+      <c r="BR20" t="inlineStr"/>
+      <c r="BS20" t="inlineStr"/>
+      <c r="BT20" t="inlineStr"/>
+      <c r="BU20" t="inlineStr"/>
+      <c r="BV20" t="inlineStr"/>
+      <c r="BW20" t="inlineStr"/>
+      <c r="BX20" t="inlineStr"/>
+      <c r="BY20" t="inlineStr"/>
+      <c r="BZ20" t="inlineStr"/>
+      <c r="CA20" t="inlineStr"/>
+      <c r="CB20" t="inlineStr"/>
+      <c r="CC20" t="inlineStr"/>
+      <c r="CD20" t="inlineStr"/>
+      <c r="CE20" t="inlineStr"/>
+      <c r="CF20" t="inlineStr"/>
+      <c r="CG20" t="inlineStr"/>
+      <c r="CH20" t="inlineStr"/>
+      <c r="CI20" t="inlineStr"/>
+      <c r="CJ20" t="inlineStr"/>
+      <c r="CK20" t="inlineStr"/>
+      <c r="CL20" t="inlineStr"/>
+      <c r="CM20" t="inlineStr"/>
+      <c r="CN20" t="inlineStr"/>
+      <c r="CO20" t="inlineStr"/>
+      <c r="CP20" t="inlineStr"/>
+      <c r="CQ20" t="inlineStr"/>
+      <c r="CR20" t="inlineStr"/>
+      <c r="CS20" t="inlineStr"/>
+      <c r="CT20" t="inlineStr"/>
+      <c r="CU20" t="inlineStr"/>
+      <c r="CV20" t="inlineStr"/>
+      <c r="CW20" t="inlineStr"/>
+      <c r="CX20" t="inlineStr"/>
+      <c r="CY20" t="inlineStr"/>
+      <c r="CZ20" t="inlineStr"/>
+      <c r="DA20" t="inlineStr"/>
+      <c r="DB20" t="inlineStr"/>
+      <c r="DC20" t="inlineStr"/>
+      <c r="DD20" t="inlineStr"/>
+      <c r="DE20" t="inlineStr"/>
+      <c r="DF20" t="inlineStr"/>
+      <c r="DG20" t="inlineStr"/>
+      <c r="DH20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5159,6 +6359,56 @@
       <c r="BJ21" t="n">
         <v>0.003730130754326795</v>
       </c>
+      <c r="BK21" t="inlineStr"/>
+      <c r="BL21" t="inlineStr"/>
+      <c r="BM21" t="inlineStr"/>
+      <c r="BN21" t="inlineStr"/>
+      <c r="BO21" t="inlineStr"/>
+      <c r="BP21" t="inlineStr"/>
+      <c r="BQ21" t="inlineStr"/>
+      <c r="BR21" t="inlineStr"/>
+      <c r="BS21" t="inlineStr"/>
+      <c r="BT21" t="inlineStr"/>
+      <c r="BU21" t="inlineStr"/>
+      <c r="BV21" t="inlineStr"/>
+      <c r="BW21" t="inlineStr"/>
+      <c r="BX21" t="inlineStr"/>
+      <c r="BY21" t="inlineStr"/>
+      <c r="BZ21" t="inlineStr"/>
+      <c r="CA21" t="inlineStr"/>
+      <c r="CB21" t="inlineStr"/>
+      <c r="CC21" t="inlineStr"/>
+      <c r="CD21" t="inlineStr"/>
+      <c r="CE21" t="inlineStr"/>
+      <c r="CF21" t="inlineStr"/>
+      <c r="CG21" t="inlineStr"/>
+      <c r="CH21" t="inlineStr"/>
+      <c r="CI21" t="inlineStr"/>
+      <c r="CJ21" t="inlineStr"/>
+      <c r="CK21" t="inlineStr"/>
+      <c r="CL21" t="inlineStr"/>
+      <c r="CM21" t="inlineStr"/>
+      <c r="CN21" t="inlineStr"/>
+      <c r="CO21" t="inlineStr"/>
+      <c r="CP21" t="inlineStr"/>
+      <c r="CQ21" t="inlineStr"/>
+      <c r="CR21" t="inlineStr"/>
+      <c r="CS21" t="inlineStr"/>
+      <c r="CT21" t="inlineStr"/>
+      <c r="CU21" t="inlineStr"/>
+      <c r="CV21" t="inlineStr"/>
+      <c r="CW21" t="inlineStr"/>
+      <c r="CX21" t="inlineStr"/>
+      <c r="CY21" t="inlineStr"/>
+      <c r="CZ21" t="inlineStr"/>
+      <c r="DA21" t="inlineStr"/>
+      <c r="DB21" t="inlineStr"/>
+      <c r="DC21" t="inlineStr"/>
+      <c r="DD21" t="inlineStr"/>
+      <c r="DE21" t="inlineStr"/>
+      <c r="DF21" t="inlineStr"/>
+      <c r="DG21" t="inlineStr"/>
+      <c r="DH21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -5379,6 +6629,56 @@
       <c r="BJ22" t="n">
         <v>0.0004372399597870666</v>
       </c>
+      <c r="BK22" t="inlineStr"/>
+      <c r="BL22" t="inlineStr"/>
+      <c r="BM22" t="inlineStr"/>
+      <c r="BN22" t="inlineStr"/>
+      <c r="BO22" t="inlineStr"/>
+      <c r="BP22" t="inlineStr"/>
+      <c r="BQ22" t="inlineStr"/>
+      <c r="BR22" t="inlineStr"/>
+      <c r="BS22" t="inlineStr"/>
+      <c r="BT22" t="inlineStr"/>
+      <c r="BU22" t="inlineStr"/>
+      <c r="BV22" t="inlineStr"/>
+      <c r="BW22" t="inlineStr"/>
+      <c r="BX22" t="inlineStr"/>
+      <c r="BY22" t="inlineStr"/>
+      <c r="BZ22" t="inlineStr"/>
+      <c r="CA22" t="inlineStr"/>
+      <c r="CB22" t="inlineStr"/>
+      <c r="CC22" t="inlineStr"/>
+      <c r="CD22" t="inlineStr"/>
+      <c r="CE22" t="inlineStr"/>
+      <c r="CF22" t="inlineStr"/>
+      <c r="CG22" t="inlineStr"/>
+      <c r="CH22" t="inlineStr"/>
+      <c r="CI22" t="inlineStr"/>
+      <c r="CJ22" t="inlineStr"/>
+      <c r="CK22" t="inlineStr"/>
+      <c r="CL22" t="inlineStr"/>
+      <c r="CM22" t="inlineStr"/>
+      <c r="CN22" t="inlineStr"/>
+      <c r="CO22" t="inlineStr"/>
+      <c r="CP22" t="inlineStr"/>
+      <c r="CQ22" t="inlineStr"/>
+      <c r="CR22" t="inlineStr"/>
+      <c r="CS22" t="inlineStr"/>
+      <c r="CT22" t="inlineStr"/>
+      <c r="CU22" t="inlineStr"/>
+      <c r="CV22" t="inlineStr"/>
+      <c r="CW22" t="inlineStr"/>
+      <c r="CX22" t="inlineStr"/>
+      <c r="CY22" t="inlineStr"/>
+      <c r="CZ22" t="inlineStr"/>
+      <c r="DA22" t="inlineStr"/>
+      <c r="DB22" t="inlineStr"/>
+      <c r="DC22" t="inlineStr"/>
+      <c r="DD22" t="inlineStr"/>
+      <c r="DE22" t="inlineStr"/>
+      <c r="DF22" t="inlineStr"/>
+      <c r="DG22" t="inlineStr"/>
+      <c r="DH22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -5599,6 +6899,56 @@
       <c r="BJ23" t="n">
         <v>3.522174730037765e-05</v>
       </c>
+      <c r="BK23" t="inlineStr"/>
+      <c r="BL23" t="inlineStr"/>
+      <c r="BM23" t="inlineStr"/>
+      <c r="BN23" t="inlineStr"/>
+      <c r="BO23" t="inlineStr"/>
+      <c r="BP23" t="inlineStr"/>
+      <c r="BQ23" t="inlineStr"/>
+      <c r="BR23" t="inlineStr"/>
+      <c r="BS23" t="inlineStr"/>
+      <c r="BT23" t="inlineStr"/>
+      <c r="BU23" t="inlineStr"/>
+      <c r="BV23" t="inlineStr"/>
+      <c r="BW23" t="inlineStr"/>
+      <c r="BX23" t="inlineStr"/>
+      <c r="BY23" t="inlineStr"/>
+      <c r="BZ23" t="inlineStr"/>
+      <c r="CA23" t="inlineStr"/>
+      <c r="CB23" t="inlineStr"/>
+      <c r="CC23" t="inlineStr"/>
+      <c r="CD23" t="inlineStr"/>
+      <c r="CE23" t="inlineStr"/>
+      <c r="CF23" t="inlineStr"/>
+      <c r="CG23" t="inlineStr"/>
+      <c r="CH23" t="inlineStr"/>
+      <c r="CI23" t="inlineStr"/>
+      <c r="CJ23" t="inlineStr"/>
+      <c r="CK23" t="inlineStr"/>
+      <c r="CL23" t="inlineStr"/>
+      <c r="CM23" t="inlineStr"/>
+      <c r="CN23" t="inlineStr"/>
+      <c r="CO23" t="inlineStr"/>
+      <c r="CP23" t="inlineStr"/>
+      <c r="CQ23" t="inlineStr"/>
+      <c r="CR23" t="inlineStr"/>
+      <c r="CS23" t="inlineStr"/>
+      <c r="CT23" t="inlineStr"/>
+      <c r="CU23" t="inlineStr"/>
+      <c r="CV23" t="inlineStr"/>
+      <c r="CW23" t="inlineStr"/>
+      <c r="CX23" t="inlineStr"/>
+      <c r="CY23" t="inlineStr"/>
+      <c r="CZ23" t="inlineStr"/>
+      <c r="DA23" t="inlineStr"/>
+      <c r="DB23" t="inlineStr"/>
+      <c r="DC23" t="inlineStr"/>
+      <c r="DD23" t="inlineStr"/>
+      <c r="DE23" t="inlineStr"/>
+      <c r="DF23" t="inlineStr"/>
+      <c r="DG23" t="inlineStr"/>
+      <c r="DH23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5829,6 +7179,56 @@
       <c r="BJ24" t="n">
         <v>9.712984233463661e-06</v>
       </c>
+      <c r="BK24" t="inlineStr"/>
+      <c r="BL24" t="inlineStr"/>
+      <c r="BM24" t="inlineStr"/>
+      <c r="BN24" t="inlineStr"/>
+      <c r="BO24" t="inlineStr"/>
+      <c r="BP24" t="inlineStr"/>
+      <c r="BQ24" t="inlineStr"/>
+      <c r="BR24" t="inlineStr"/>
+      <c r="BS24" t="inlineStr"/>
+      <c r="BT24" t="inlineStr"/>
+      <c r="BU24" t="inlineStr"/>
+      <c r="BV24" t="inlineStr"/>
+      <c r="BW24" t="inlineStr"/>
+      <c r="BX24" t="inlineStr"/>
+      <c r="BY24" t="inlineStr"/>
+      <c r="BZ24" t="inlineStr"/>
+      <c r="CA24" t="inlineStr"/>
+      <c r="CB24" t="inlineStr"/>
+      <c r="CC24" t="inlineStr"/>
+      <c r="CD24" t="inlineStr"/>
+      <c r="CE24" t="inlineStr"/>
+      <c r="CF24" t="inlineStr"/>
+      <c r="CG24" t="inlineStr"/>
+      <c r="CH24" t="inlineStr"/>
+      <c r="CI24" t="inlineStr"/>
+      <c r="CJ24" t="inlineStr"/>
+      <c r="CK24" t="inlineStr"/>
+      <c r="CL24" t="inlineStr"/>
+      <c r="CM24" t="inlineStr"/>
+      <c r="CN24" t="inlineStr"/>
+      <c r="CO24" t="inlineStr"/>
+      <c r="CP24" t="inlineStr"/>
+      <c r="CQ24" t="inlineStr"/>
+      <c r="CR24" t="inlineStr"/>
+      <c r="CS24" t="inlineStr"/>
+      <c r="CT24" t="inlineStr"/>
+      <c r="CU24" t="inlineStr"/>
+      <c r="CV24" t="inlineStr"/>
+      <c r="CW24" t="inlineStr"/>
+      <c r="CX24" t="inlineStr"/>
+      <c r="CY24" t="inlineStr"/>
+      <c r="CZ24" t="inlineStr"/>
+      <c r="DA24" t="inlineStr"/>
+      <c r="DB24" t="inlineStr"/>
+      <c r="DC24" t="inlineStr"/>
+      <c r="DD24" t="inlineStr"/>
+      <c r="DE24" t="inlineStr"/>
+      <c r="DF24" t="inlineStr"/>
+      <c r="DG24" t="inlineStr"/>
+      <c r="DH24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -6059,6 +7459,56 @@
       <c r="BJ25" t="n">
         <v>0</v>
       </c>
+      <c r="BK25" t="inlineStr"/>
+      <c r="BL25" t="inlineStr"/>
+      <c r="BM25" t="inlineStr"/>
+      <c r="BN25" t="inlineStr"/>
+      <c r="BO25" t="inlineStr"/>
+      <c r="BP25" t="inlineStr"/>
+      <c r="BQ25" t="inlineStr"/>
+      <c r="BR25" t="inlineStr"/>
+      <c r="BS25" t="inlineStr"/>
+      <c r="BT25" t="inlineStr"/>
+      <c r="BU25" t="inlineStr"/>
+      <c r="BV25" t="inlineStr"/>
+      <c r="BW25" t="inlineStr"/>
+      <c r="BX25" t="inlineStr"/>
+      <c r="BY25" t="inlineStr"/>
+      <c r="BZ25" t="inlineStr"/>
+      <c r="CA25" t="inlineStr"/>
+      <c r="CB25" t="inlineStr"/>
+      <c r="CC25" t="inlineStr"/>
+      <c r="CD25" t="inlineStr"/>
+      <c r="CE25" t="inlineStr"/>
+      <c r="CF25" t="inlineStr"/>
+      <c r="CG25" t="inlineStr"/>
+      <c r="CH25" t="inlineStr"/>
+      <c r="CI25" t="inlineStr"/>
+      <c r="CJ25" t="inlineStr"/>
+      <c r="CK25" t="inlineStr"/>
+      <c r="CL25" t="inlineStr"/>
+      <c r="CM25" t="inlineStr"/>
+      <c r="CN25" t="inlineStr"/>
+      <c r="CO25" t="inlineStr"/>
+      <c r="CP25" t="inlineStr"/>
+      <c r="CQ25" t="inlineStr"/>
+      <c r="CR25" t="inlineStr"/>
+      <c r="CS25" t="inlineStr"/>
+      <c r="CT25" t="inlineStr"/>
+      <c r="CU25" t="inlineStr"/>
+      <c r="CV25" t="inlineStr"/>
+      <c r="CW25" t="inlineStr"/>
+      <c r="CX25" t="inlineStr"/>
+      <c r="CY25" t="inlineStr"/>
+      <c r="CZ25" t="inlineStr"/>
+      <c r="DA25" t="inlineStr"/>
+      <c r="DB25" t="inlineStr"/>
+      <c r="DC25" t="inlineStr"/>
+      <c r="DD25" t="inlineStr"/>
+      <c r="DE25" t="inlineStr"/>
+      <c r="DF25" t="inlineStr"/>
+      <c r="DG25" t="inlineStr"/>
+      <c r="DH25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -6279,6 +7729,56 @@
       <c r="BJ26" t="n">
         <v>0.006864583551809107</v>
       </c>
+      <c r="BK26" t="inlineStr"/>
+      <c r="BL26" t="inlineStr"/>
+      <c r="BM26" t="inlineStr"/>
+      <c r="BN26" t="inlineStr"/>
+      <c r="BO26" t="inlineStr"/>
+      <c r="BP26" t="inlineStr"/>
+      <c r="BQ26" t="inlineStr"/>
+      <c r="BR26" t="inlineStr"/>
+      <c r="BS26" t="inlineStr"/>
+      <c r="BT26" t="inlineStr"/>
+      <c r="BU26" t="inlineStr"/>
+      <c r="BV26" t="inlineStr"/>
+      <c r="BW26" t="inlineStr"/>
+      <c r="BX26" t="inlineStr"/>
+      <c r="BY26" t="inlineStr"/>
+      <c r="BZ26" t="inlineStr"/>
+      <c r="CA26" t="inlineStr"/>
+      <c r="CB26" t="inlineStr"/>
+      <c r="CC26" t="inlineStr"/>
+      <c r="CD26" t="inlineStr"/>
+      <c r="CE26" t="inlineStr"/>
+      <c r="CF26" t="inlineStr"/>
+      <c r="CG26" t="inlineStr"/>
+      <c r="CH26" t="inlineStr"/>
+      <c r="CI26" t="inlineStr"/>
+      <c r="CJ26" t="inlineStr"/>
+      <c r="CK26" t="inlineStr"/>
+      <c r="CL26" t="inlineStr"/>
+      <c r="CM26" t="inlineStr"/>
+      <c r="CN26" t="inlineStr"/>
+      <c r="CO26" t="inlineStr"/>
+      <c r="CP26" t="inlineStr"/>
+      <c r="CQ26" t="inlineStr"/>
+      <c r="CR26" t="inlineStr"/>
+      <c r="CS26" t="inlineStr"/>
+      <c r="CT26" t="inlineStr"/>
+      <c r="CU26" t="inlineStr"/>
+      <c r="CV26" t="inlineStr"/>
+      <c r="CW26" t="inlineStr"/>
+      <c r="CX26" t="inlineStr"/>
+      <c r="CY26" t="inlineStr"/>
+      <c r="CZ26" t="inlineStr"/>
+      <c r="DA26" t="inlineStr"/>
+      <c r="DB26" t="inlineStr"/>
+      <c r="DC26" t="inlineStr"/>
+      <c r="DD26" t="inlineStr"/>
+      <c r="DE26" t="inlineStr"/>
+      <c r="DF26" t="inlineStr"/>
+      <c r="DG26" t="inlineStr"/>
+      <c r="DH26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -6499,6 +7999,56 @@
       <c r="BJ27" t="n">
         <v>0.00633123507806117</v>
       </c>
+      <c r="BK27" t="inlineStr"/>
+      <c r="BL27" t="inlineStr"/>
+      <c r="BM27" t="inlineStr"/>
+      <c r="BN27" t="inlineStr"/>
+      <c r="BO27" t="inlineStr"/>
+      <c r="BP27" t="inlineStr"/>
+      <c r="BQ27" t="inlineStr"/>
+      <c r="BR27" t="inlineStr"/>
+      <c r="BS27" t="inlineStr"/>
+      <c r="BT27" t="inlineStr"/>
+      <c r="BU27" t="inlineStr"/>
+      <c r="BV27" t="inlineStr"/>
+      <c r="BW27" t="inlineStr"/>
+      <c r="BX27" t="inlineStr"/>
+      <c r="BY27" t="inlineStr"/>
+      <c r="BZ27" t="inlineStr"/>
+      <c r="CA27" t="inlineStr"/>
+      <c r="CB27" t="inlineStr"/>
+      <c r="CC27" t="inlineStr"/>
+      <c r="CD27" t="inlineStr"/>
+      <c r="CE27" t="inlineStr"/>
+      <c r="CF27" t="inlineStr"/>
+      <c r="CG27" t="inlineStr"/>
+      <c r="CH27" t="inlineStr"/>
+      <c r="CI27" t="inlineStr"/>
+      <c r="CJ27" t="inlineStr"/>
+      <c r="CK27" t="inlineStr"/>
+      <c r="CL27" t="inlineStr"/>
+      <c r="CM27" t="inlineStr"/>
+      <c r="CN27" t="inlineStr"/>
+      <c r="CO27" t="inlineStr"/>
+      <c r="CP27" t="inlineStr"/>
+      <c r="CQ27" t="inlineStr"/>
+      <c r="CR27" t="inlineStr"/>
+      <c r="CS27" t="inlineStr"/>
+      <c r="CT27" t="inlineStr"/>
+      <c r="CU27" t="inlineStr"/>
+      <c r="CV27" t="inlineStr"/>
+      <c r="CW27" t="inlineStr"/>
+      <c r="CX27" t="inlineStr"/>
+      <c r="CY27" t="inlineStr"/>
+      <c r="CZ27" t="inlineStr"/>
+      <c r="DA27" t="inlineStr"/>
+      <c r="DB27" t="inlineStr"/>
+      <c r="DC27" t="inlineStr"/>
+      <c r="DD27" t="inlineStr"/>
+      <c r="DE27" t="inlineStr"/>
+      <c r="DF27" t="inlineStr"/>
+      <c r="DG27" t="inlineStr"/>
+      <c r="DH27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -6719,6 +8269,56 @@
       <c r="BJ28" t="n">
         <v>0.006998243955679154</v>
       </c>
+      <c r="BK28" t="inlineStr"/>
+      <c r="BL28" t="inlineStr"/>
+      <c r="BM28" t="inlineStr"/>
+      <c r="BN28" t="inlineStr"/>
+      <c r="BO28" t="inlineStr"/>
+      <c r="BP28" t="inlineStr"/>
+      <c r="BQ28" t="inlineStr"/>
+      <c r="BR28" t="inlineStr"/>
+      <c r="BS28" t="inlineStr"/>
+      <c r="BT28" t="inlineStr"/>
+      <c r="BU28" t="inlineStr"/>
+      <c r="BV28" t="inlineStr"/>
+      <c r="BW28" t="inlineStr"/>
+      <c r="BX28" t="inlineStr"/>
+      <c r="BY28" t="inlineStr"/>
+      <c r="BZ28" t="inlineStr"/>
+      <c r="CA28" t="inlineStr"/>
+      <c r="CB28" t="inlineStr"/>
+      <c r="CC28" t="inlineStr"/>
+      <c r="CD28" t="inlineStr"/>
+      <c r="CE28" t="inlineStr"/>
+      <c r="CF28" t="inlineStr"/>
+      <c r="CG28" t="inlineStr"/>
+      <c r="CH28" t="inlineStr"/>
+      <c r="CI28" t="inlineStr"/>
+      <c r="CJ28" t="inlineStr"/>
+      <c r="CK28" t="inlineStr"/>
+      <c r="CL28" t="inlineStr"/>
+      <c r="CM28" t="inlineStr"/>
+      <c r="CN28" t="inlineStr"/>
+      <c r="CO28" t="inlineStr"/>
+      <c r="CP28" t="inlineStr"/>
+      <c r="CQ28" t="inlineStr"/>
+      <c r="CR28" t="inlineStr"/>
+      <c r="CS28" t="inlineStr"/>
+      <c r="CT28" t="inlineStr"/>
+      <c r="CU28" t="inlineStr"/>
+      <c r="CV28" t="inlineStr"/>
+      <c r="CW28" t="inlineStr"/>
+      <c r="CX28" t="inlineStr"/>
+      <c r="CY28" t="inlineStr"/>
+      <c r="CZ28" t="inlineStr"/>
+      <c r="DA28" t="inlineStr"/>
+      <c r="DB28" t="inlineStr"/>
+      <c r="DC28" t="inlineStr"/>
+      <c r="DD28" t="inlineStr"/>
+      <c r="DE28" t="inlineStr"/>
+      <c r="DF28" t="inlineStr"/>
+      <c r="DG28" t="inlineStr"/>
+      <c r="DH28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -6939,6 +8539,56 @@
       <c r="BJ29" t="n">
         <v>0.005979998658646051</v>
       </c>
+      <c r="BK29" t="inlineStr"/>
+      <c r="BL29" t="inlineStr"/>
+      <c r="BM29" t="inlineStr"/>
+      <c r="BN29" t="inlineStr"/>
+      <c r="BO29" t="inlineStr"/>
+      <c r="BP29" t="inlineStr"/>
+      <c r="BQ29" t="inlineStr"/>
+      <c r="BR29" t="inlineStr"/>
+      <c r="BS29" t="inlineStr"/>
+      <c r="BT29" t="inlineStr"/>
+      <c r="BU29" t="inlineStr"/>
+      <c r="BV29" t="inlineStr"/>
+      <c r="BW29" t="inlineStr"/>
+      <c r="BX29" t="inlineStr"/>
+      <c r="BY29" t="inlineStr"/>
+      <c r="BZ29" t="inlineStr"/>
+      <c r="CA29" t="inlineStr"/>
+      <c r="CB29" t="inlineStr"/>
+      <c r="CC29" t="inlineStr"/>
+      <c r="CD29" t="inlineStr"/>
+      <c r="CE29" t="inlineStr"/>
+      <c r="CF29" t="inlineStr"/>
+      <c r="CG29" t="inlineStr"/>
+      <c r="CH29" t="inlineStr"/>
+      <c r="CI29" t="inlineStr"/>
+      <c r="CJ29" t="inlineStr"/>
+      <c r="CK29" t="inlineStr"/>
+      <c r="CL29" t="inlineStr"/>
+      <c r="CM29" t="inlineStr"/>
+      <c r="CN29" t="inlineStr"/>
+      <c r="CO29" t="inlineStr"/>
+      <c r="CP29" t="inlineStr"/>
+      <c r="CQ29" t="inlineStr"/>
+      <c r="CR29" t="inlineStr"/>
+      <c r="CS29" t="inlineStr"/>
+      <c r="CT29" t="inlineStr"/>
+      <c r="CU29" t="inlineStr"/>
+      <c r="CV29" t="inlineStr"/>
+      <c r="CW29" t="inlineStr"/>
+      <c r="CX29" t="inlineStr"/>
+      <c r="CY29" t="inlineStr"/>
+      <c r="CZ29" t="inlineStr"/>
+      <c r="DA29" t="inlineStr"/>
+      <c r="DB29" t="inlineStr"/>
+      <c r="DC29" t="inlineStr"/>
+      <c r="DD29" t="inlineStr"/>
+      <c r="DE29" t="inlineStr"/>
+      <c r="DF29" t="inlineStr"/>
+      <c r="DG29" t="inlineStr"/>
+      <c r="DH29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -7159,6 +8809,56 @@
       <c r="BJ30" t="n">
         <v>0.003593501616458011</v>
       </c>
+      <c r="BK30" t="inlineStr"/>
+      <c r="BL30" t="inlineStr"/>
+      <c r="BM30" t="inlineStr"/>
+      <c r="BN30" t="inlineStr"/>
+      <c r="BO30" t="inlineStr"/>
+      <c r="BP30" t="inlineStr"/>
+      <c r="BQ30" t="inlineStr"/>
+      <c r="BR30" t="inlineStr"/>
+      <c r="BS30" t="inlineStr"/>
+      <c r="BT30" t="inlineStr"/>
+      <c r="BU30" t="inlineStr"/>
+      <c r="BV30" t="inlineStr"/>
+      <c r="BW30" t="inlineStr"/>
+      <c r="BX30" t="inlineStr"/>
+      <c r="BY30" t="inlineStr"/>
+      <c r="BZ30" t="inlineStr"/>
+      <c r="CA30" t="inlineStr"/>
+      <c r="CB30" t="inlineStr"/>
+      <c r="CC30" t="inlineStr"/>
+      <c r="CD30" t="inlineStr"/>
+      <c r="CE30" t="inlineStr"/>
+      <c r="CF30" t="inlineStr"/>
+      <c r="CG30" t="inlineStr"/>
+      <c r="CH30" t="inlineStr"/>
+      <c r="CI30" t="inlineStr"/>
+      <c r="CJ30" t="inlineStr"/>
+      <c r="CK30" t="inlineStr"/>
+      <c r="CL30" t="inlineStr"/>
+      <c r="CM30" t="inlineStr"/>
+      <c r="CN30" t="inlineStr"/>
+      <c r="CO30" t="inlineStr"/>
+      <c r="CP30" t="inlineStr"/>
+      <c r="CQ30" t="inlineStr"/>
+      <c r="CR30" t="inlineStr"/>
+      <c r="CS30" t="inlineStr"/>
+      <c r="CT30" t="inlineStr"/>
+      <c r="CU30" t="inlineStr"/>
+      <c r="CV30" t="inlineStr"/>
+      <c r="CW30" t="inlineStr"/>
+      <c r="CX30" t="inlineStr"/>
+      <c r="CY30" t="inlineStr"/>
+      <c r="CZ30" t="inlineStr"/>
+      <c r="DA30" t="inlineStr"/>
+      <c r="DB30" t="inlineStr"/>
+      <c r="DC30" t="inlineStr"/>
+      <c r="DD30" t="inlineStr"/>
+      <c r="DE30" t="inlineStr"/>
+      <c r="DF30" t="inlineStr"/>
+      <c r="DG30" t="inlineStr"/>
+      <c r="DH30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -7379,6 +9079,56 @@
       <c r="BJ31" t="n">
         <v>0.00331515533222134</v>
       </c>
+      <c r="BK31" t="inlineStr"/>
+      <c r="BL31" t="inlineStr"/>
+      <c r="BM31" t="inlineStr"/>
+      <c r="BN31" t="inlineStr"/>
+      <c r="BO31" t="inlineStr"/>
+      <c r="BP31" t="inlineStr"/>
+      <c r="BQ31" t="inlineStr"/>
+      <c r="BR31" t="inlineStr"/>
+      <c r="BS31" t="inlineStr"/>
+      <c r="BT31" t="inlineStr"/>
+      <c r="BU31" t="inlineStr"/>
+      <c r="BV31" t="inlineStr"/>
+      <c r="BW31" t="inlineStr"/>
+      <c r="BX31" t="inlineStr"/>
+      <c r="BY31" t="inlineStr"/>
+      <c r="BZ31" t="inlineStr"/>
+      <c r="CA31" t="inlineStr"/>
+      <c r="CB31" t="inlineStr"/>
+      <c r="CC31" t="inlineStr"/>
+      <c r="CD31" t="inlineStr"/>
+      <c r="CE31" t="inlineStr"/>
+      <c r="CF31" t="inlineStr"/>
+      <c r="CG31" t="inlineStr"/>
+      <c r="CH31" t="inlineStr"/>
+      <c r="CI31" t="inlineStr"/>
+      <c r="CJ31" t="inlineStr"/>
+      <c r="CK31" t="inlineStr"/>
+      <c r="CL31" t="inlineStr"/>
+      <c r="CM31" t="inlineStr"/>
+      <c r="CN31" t="inlineStr"/>
+      <c r="CO31" t="inlineStr"/>
+      <c r="CP31" t="inlineStr"/>
+      <c r="CQ31" t="inlineStr"/>
+      <c r="CR31" t="inlineStr"/>
+      <c r="CS31" t="inlineStr"/>
+      <c r="CT31" t="inlineStr"/>
+      <c r="CU31" t="inlineStr"/>
+      <c r="CV31" t="inlineStr"/>
+      <c r="CW31" t="inlineStr"/>
+      <c r="CX31" t="inlineStr"/>
+      <c r="CY31" t="inlineStr"/>
+      <c r="CZ31" t="inlineStr"/>
+      <c r="DA31" t="inlineStr"/>
+      <c r="DB31" t="inlineStr"/>
+      <c r="DC31" t="inlineStr"/>
+      <c r="DD31" t="inlineStr"/>
+      <c r="DE31" t="inlineStr"/>
+      <c r="DF31" t="inlineStr"/>
+      <c r="DG31" t="inlineStr"/>
+      <c r="DH31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -7599,6 +9349,56 @@
       <c r="BJ32" t="n">
         <v>0.005858666205929211</v>
       </c>
+      <c r="BK32" t="inlineStr"/>
+      <c r="BL32" t="inlineStr"/>
+      <c r="BM32" t="inlineStr"/>
+      <c r="BN32" t="inlineStr"/>
+      <c r="BO32" t="inlineStr"/>
+      <c r="BP32" t="inlineStr"/>
+      <c r="BQ32" t="inlineStr"/>
+      <c r="BR32" t="inlineStr"/>
+      <c r="BS32" t="inlineStr"/>
+      <c r="BT32" t="inlineStr"/>
+      <c r="BU32" t="inlineStr"/>
+      <c r="BV32" t="inlineStr"/>
+      <c r="BW32" t="inlineStr"/>
+      <c r="BX32" t="inlineStr"/>
+      <c r="BY32" t="inlineStr"/>
+      <c r="BZ32" t="inlineStr"/>
+      <c r="CA32" t="inlineStr"/>
+      <c r="CB32" t="inlineStr"/>
+      <c r="CC32" t="inlineStr"/>
+      <c r="CD32" t="inlineStr"/>
+      <c r="CE32" t="inlineStr"/>
+      <c r="CF32" t="inlineStr"/>
+      <c r="CG32" t="inlineStr"/>
+      <c r="CH32" t="inlineStr"/>
+      <c r="CI32" t="inlineStr"/>
+      <c r="CJ32" t="inlineStr"/>
+      <c r="CK32" t="inlineStr"/>
+      <c r="CL32" t="inlineStr"/>
+      <c r="CM32" t="inlineStr"/>
+      <c r="CN32" t="inlineStr"/>
+      <c r="CO32" t="inlineStr"/>
+      <c r="CP32" t="inlineStr"/>
+      <c r="CQ32" t="inlineStr"/>
+      <c r="CR32" t="inlineStr"/>
+      <c r="CS32" t="inlineStr"/>
+      <c r="CT32" t="inlineStr"/>
+      <c r="CU32" t="inlineStr"/>
+      <c r="CV32" t="inlineStr"/>
+      <c r="CW32" t="inlineStr"/>
+      <c r="CX32" t="inlineStr"/>
+      <c r="CY32" t="inlineStr"/>
+      <c r="CZ32" t="inlineStr"/>
+      <c r="DA32" t="inlineStr"/>
+      <c r="DB32" t="inlineStr"/>
+      <c r="DC32" t="inlineStr"/>
+      <c r="DD32" t="inlineStr"/>
+      <c r="DE32" t="inlineStr"/>
+      <c r="DF32" t="inlineStr"/>
+      <c r="DG32" t="inlineStr"/>
+      <c r="DH32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -7819,6 +9619,56 @@
       <c r="BJ33" t="n">
         <v>0.004119140442349333</v>
       </c>
+      <c r="BK33" t="inlineStr"/>
+      <c r="BL33" t="inlineStr"/>
+      <c r="BM33" t="inlineStr"/>
+      <c r="BN33" t="inlineStr"/>
+      <c r="BO33" t="inlineStr"/>
+      <c r="BP33" t="inlineStr"/>
+      <c r="BQ33" t="inlineStr"/>
+      <c r="BR33" t="inlineStr"/>
+      <c r="BS33" t="inlineStr"/>
+      <c r="BT33" t="inlineStr"/>
+      <c r="BU33" t="inlineStr"/>
+      <c r="BV33" t="inlineStr"/>
+      <c r="BW33" t="inlineStr"/>
+      <c r="BX33" t="inlineStr"/>
+      <c r="BY33" t="inlineStr"/>
+      <c r="BZ33" t="inlineStr"/>
+      <c r="CA33" t="inlineStr"/>
+      <c r="CB33" t="inlineStr"/>
+      <c r="CC33" t="inlineStr"/>
+      <c r="CD33" t="inlineStr"/>
+      <c r="CE33" t="inlineStr"/>
+      <c r="CF33" t="inlineStr"/>
+      <c r="CG33" t="inlineStr"/>
+      <c r="CH33" t="inlineStr"/>
+      <c r="CI33" t="inlineStr"/>
+      <c r="CJ33" t="inlineStr"/>
+      <c r="CK33" t="inlineStr"/>
+      <c r="CL33" t="inlineStr"/>
+      <c r="CM33" t="inlineStr"/>
+      <c r="CN33" t="inlineStr"/>
+      <c r="CO33" t="inlineStr"/>
+      <c r="CP33" t="inlineStr"/>
+      <c r="CQ33" t="inlineStr"/>
+      <c r="CR33" t="inlineStr"/>
+      <c r="CS33" t="inlineStr"/>
+      <c r="CT33" t="inlineStr"/>
+      <c r="CU33" t="inlineStr"/>
+      <c r="CV33" t="inlineStr"/>
+      <c r="CW33" t="inlineStr"/>
+      <c r="CX33" t="inlineStr"/>
+      <c r="CY33" t="inlineStr"/>
+      <c r="CZ33" t="inlineStr"/>
+      <c r="DA33" t="inlineStr"/>
+      <c r="DB33" t="inlineStr"/>
+      <c r="DC33" t="inlineStr"/>
+      <c r="DD33" t="inlineStr"/>
+      <c r="DE33" t="inlineStr"/>
+      <c r="DF33" t="inlineStr"/>
+      <c r="DG33" t="inlineStr"/>
+      <c r="DH33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -8039,6 +9889,56 @@
       <c r="BJ34" t="n">
         <v>0.0002469013067630454</v>
       </c>
+      <c r="BK34" t="inlineStr"/>
+      <c r="BL34" t="inlineStr"/>
+      <c r="BM34" t="inlineStr"/>
+      <c r="BN34" t="inlineStr"/>
+      <c r="BO34" t="inlineStr"/>
+      <c r="BP34" t="inlineStr"/>
+      <c r="BQ34" t="inlineStr"/>
+      <c r="BR34" t="inlineStr"/>
+      <c r="BS34" t="inlineStr"/>
+      <c r="BT34" t="inlineStr"/>
+      <c r="BU34" t="inlineStr"/>
+      <c r="BV34" t="inlineStr"/>
+      <c r="BW34" t="inlineStr"/>
+      <c r="BX34" t="inlineStr"/>
+      <c r="BY34" t="inlineStr"/>
+      <c r="BZ34" t="inlineStr"/>
+      <c r="CA34" t="inlineStr"/>
+      <c r="CB34" t="inlineStr"/>
+      <c r="CC34" t="inlineStr"/>
+      <c r="CD34" t="inlineStr"/>
+      <c r="CE34" t="inlineStr"/>
+      <c r="CF34" t="inlineStr"/>
+      <c r="CG34" t="inlineStr"/>
+      <c r="CH34" t="inlineStr"/>
+      <c r="CI34" t="inlineStr"/>
+      <c r="CJ34" t="inlineStr"/>
+      <c r="CK34" t="inlineStr"/>
+      <c r="CL34" t="inlineStr"/>
+      <c r="CM34" t="inlineStr"/>
+      <c r="CN34" t="inlineStr"/>
+      <c r="CO34" t="inlineStr"/>
+      <c r="CP34" t="inlineStr"/>
+      <c r="CQ34" t="inlineStr"/>
+      <c r="CR34" t="inlineStr"/>
+      <c r="CS34" t="inlineStr"/>
+      <c r="CT34" t="inlineStr"/>
+      <c r="CU34" t="inlineStr"/>
+      <c r="CV34" t="inlineStr"/>
+      <c r="CW34" t="inlineStr"/>
+      <c r="CX34" t="inlineStr"/>
+      <c r="CY34" t="inlineStr"/>
+      <c r="CZ34" t="inlineStr"/>
+      <c r="DA34" t="inlineStr"/>
+      <c r="DB34" t="inlineStr"/>
+      <c r="DC34" t="inlineStr"/>
+      <c r="DD34" t="inlineStr"/>
+      <c r="DE34" t="inlineStr"/>
+      <c r="DF34" t="inlineStr"/>
+      <c r="DG34" t="inlineStr"/>
+      <c r="DH34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -8259,6 +10159,56 @@
       <c r="BJ35" t="n">
         <v>3.550147888793166e-05</v>
       </c>
+      <c r="BK35" t="inlineStr"/>
+      <c r="BL35" t="inlineStr"/>
+      <c r="BM35" t="inlineStr"/>
+      <c r="BN35" t="inlineStr"/>
+      <c r="BO35" t="inlineStr"/>
+      <c r="BP35" t="inlineStr"/>
+      <c r="BQ35" t="inlineStr"/>
+      <c r="BR35" t="inlineStr"/>
+      <c r="BS35" t="inlineStr"/>
+      <c r="BT35" t="inlineStr"/>
+      <c r="BU35" t="inlineStr"/>
+      <c r="BV35" t="inlineStr"/>
+      <c r="BW35" t="inlineStr"/>
+      <c r="BX35" t="inlineStr"/>
+      <c r="BY35" t="inlineStr"/>
+      <c r="BZ35" t="inlineStr"/>
+      <c r="CA35" t="inlineStr"/>
+      <c r="CB35" t="inlineStr"/>
+      <c r="CC35" t="inlineStr"/>
+      <c r="CD35" t="inlineStr"/>
+      <c r="CE35" t="inlineStr"/>
+      <c r="CF35" t="inlineStr"/>
+      <c r="CG35" t="inlineStr"/>
+      <c r="CH35" t="inlineStr"/>
+      <c r="CI35" t="inlineStr"/>
+      <c r="CJ35" t="inlineStr"/>
+      <c r="CK35" t="inlineStr"/>
+      <c r="CL35" t="inlineStr"/>
+      <c r="CM35" t="inlineStr"/>
+      <c r="CN35" t="inlineStr"/>
+      <c r="CO35" t="inlineStr"/>
+      <c r="CP35" t="inlineStr"/>
+      <c r="CQ35" t="inlineStr"/>
+      <c r="CR35" t="inlineStr"/>
+      <c r="CS35" t="inlineStr"/>
+      <c r="CT35" t="inlineStr"/>
+      <c r="CU35" t="inlineStr"/>
+      <c r="CV35" t="inlineStr"/>
+      <c r="CW35" t="inlineStr"/>
+      <c r="CX35" t="inlineStr"/>
+      <c r="CY35" t="inlineStr"/>
+      <c r="CZ35" t="inlineStr"/>
+      <c r="DA35" t="inlineStr"/>
+      <c r="DB35" t="inlineStr"/>
+      <c r="DC35" t="inlineStr"/>
+      <c r="DD35" t="inlineStr"/>
+      <c r="DE35" t="inlineStr"/>
+      <c r="DF35" t="inlineStr"/>
+      <c r="DG35" t="inlineStr"/>
+      <c r="DH35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -8489,6 +10439,56 @@
       <c r="BJ36" t="n">
         <v>9.712984233463659e-06</v>
       </c>
+      <c r="BK36" t="inlineStr"/>
+      <c r="BL36" t="inlineStr"/>
+      <c r="BM36" t="inlineStr"/>
+      <c r="BN36" t="inlineStr"/>
+      <c r="BO36" t="inlineStr"/>
+      <c r="BP36" t="inlineStr"/>
+      <c r="BQ36" t="inlineStr"/>
+      <c r="BR36" t="inlineStr"/>
+      <c r="BS36" t="inlineStr"/>
+      <c r="BT36" t="inlineStr"/>
+      <c r="BU36" t="inlineStr"/>
+      <c r="BV36" t="inlineStr"/>
+      <c r="BW36" t="inlineStr"/>
+      <c r="BX36" t="inlineStr"/>
+      <c r="BY36" t="inlineStr"/>
+      <c r="BZ36" t="inlineStr"/>
+      <c r="CA36" t="inlineStr"/>
+      <c r="CB36" t="inlineStr"/>
+      <c r="CC36" t="inlineStr"/>
+      <c r="CD36" t="inlineStr"/>
+      <c r="CE36" t="inlineStr"/>
+      <c r="CF36" t="inlineStr"/>
+      <c r="CG36" t="inlineStr"/>
+      <c r="CH36" t="inlineStr"/>
+      <c r="CI36" t="inlineStr"/>
+      <c r="CJ36" t="inlineStr"/>
+      <c r="CK36" t="inlineStr"/>
+      <c r="CL36" t="inlineStr"/>
+      <c r="CM36" t="inlineStr"/>
+      <c r="CN36" t="inlineStr"/>
+      <c r="CO36" t="inlineStr"/>
+      <c r="CP36" t="inlineStr"/>
+      <c r="CQ36" t="inlineStr"/>
+      <c r="CR36" t="inlineStr"/>
+      <c r="CS36" t="inlineStr"/>
+      <c r="CT36" t="inlineStr"/>
+      <c r="CU36" t="inlineStr"/>
+      <c r="CV36" t="inlineStr"/>
+      <c r="CW36" t="inlineStr"/>
+      <c r="CX36" t="inlineStr"/>
+      <c r="CY36" t="inlineStr"/>
+      <c r="CZ36" t="inlineStr"/>
+      <c r="DA36" t="inlineStr"/>
+      <c r="DB36" t="inlineStr"/>
+      <c r="DC36" t="inlineStr"/>
+      <c r="DD36" t="inlineStr"/>
+      <c r="DE36" t="inlineStr"/>
+      <c r="DF36" t="inlineStr"/>
+      <c r="DG36" t="inlineStr"/>
+      <c r="DH36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -8719,6 +10719,56 @@
       <c r="BJ37" t="n">
         <v>0</v>
       </c>
+      <c r="BK37" t="inlineStr"/>
+      <c r="BL37" t="inlineStr"/>
+      <c r="BM37" t="inlineStr"/>
+      <c r="BN37" t="inlineStr"/>
+      <c r="BO37" t="inlineStr"/>
+      <c r="BP37" t="inlineStr"/>
+      <c r="BQ37" t="inlineStr"/>
+      <c r="BR37" t="inlineStr"/>
+      <c r="BS37" t="inlineStr"/>
+      <c r="BT37" t="inlineStr"/>
+      <c r="BU37" t="inlineStr"/>
+      <c r="BV37" t="inlineStr"/>
+      <c r="BW37" t="inlineStr"/>
+      <c r="BX37" t="inlineStr"/>
+      <c r="BY37" t="inlineStr"/>
+      <c r="BZ37" t="inlineStr"/>
+      <c r="CA37" t="inlineStr"/>
+      <c r="CB37" t="inlineStr"/>
+      <c r="CC37" t="inlineStr"/>
+      <c r="CD37" t="inlineStr"/>
+      <c r="CE37" t="inlineStr"/>
+      <c r="CF37" t="inlineStr"/>
+      <c r="CG37" t="inlineStr"/>
+      <c r="CH37" t="inlineStr"/>
+      <c r="CI37" t="inlineStr"/>
+      <c r="CJ37" t="inlineStr"/>
+      <c r="CK37" t="inlineStr"/>
+      <c r="CL37" t="inlineStr"/>
+      <c r="CM37" t="inlineStr"/>
+      <c r="CN37" t="inlineStr"/>
+      <c r="CO37" t="inlineStr"/>
+      <c r="CP37" t="inlineStr"/>
+      <c r="CQ37" t="inlineStr"/>
+      <c r="CR37" t="inlineStr"/>
+      <c r="CS37" t="inlineStr"/>
+      <c r="CT37" t="inlineStr"/>
+      <c r="CU37" t="inlineStr"/>
+      <c r="CV37" t="inlineStr"/>
+      <c r="CW37" t="inlineStr"/>
+      <c r="CX37" t="inlineStr"/>
+      <c r="CY37" t="inlineStr"/>
+      <c r="CZ37" t="inlineStr"/>
+      <c r="DA37" t="inlineStr"/>
+      <c r="DB37" t="inlineStr"/>
+      <c r="DC37" t="inlineStr"/>
+      <c r="DD37" t="inlineStr"/>
+      <c r="DE37" t="inlineStr"/>
+      <c r="DF37" t="inlineStr"/>
+      <c r="DG37" t="inlineStr"/>
+      <c r="DH37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -8939,6 +10989,56 @@
       <c r="BJ38" t="n">
         <v>0.006069971402500744</v>
       </c>
+      <c r="BK38" t="inlineStr"/>
+      <c r="BL38" t="inlineStr"/>
+      <c r="BM38" t="inlineStr"/>
+      <c r="BN38" t="inlineStr"/>
+      <c r="BO38" t="inlineStr"/>
+      <c r="BP38" t="inlineStr"/>
+      <c r="BQ38" t="inlineStr"/>
+      <c r="BR38" t="inlineStr"/>
+      <c r="BS38" t="inlineStr"/>
+      <c r="BT38" t="inlineStr"/>
+      <c r="BU38" t="inlineStr"/>
+      <c r="BV38" t="inlineStr"/>
+      <c r="BW38" t="inlineStr"/>
+      <c r="BX38" t="inlineStr"/>
+      <c r="BY38" t="inlineStr"/>
+      <c r="BZ38" t="inlineStr"/>
+      <c r="CA38" t="inlineStr"/>
+      <c r="CB38" t="inlineStr"/>
+      <c r="CC38" t="inlineStr"/>
+      <c r="CD38" t="inlineStr"/>
+      <c r="CE38" t="inlineStr"/>
+      <c r="CF38" t="inlineStr"/>
+      <c r="CG38" t="inlineStr"/>
+      <c r="CH38" t="inlineStr"/>
+      <c r="CI38" t="inlineStr"/>
+      <c r="CJ38" t="inlineStr"/>
+      <c r="CK38" t="inlineStr"/>
+      <c r="CL38" t="inlineStr"/>
+      <c r="CM38" t="inlineStr"/>
+      <c r="CN38" t="inlineStr"/>
+      <c r="CO38" t="inlineStr"/>
+      <c r="CP38" t="inlineStr"/>
+      <c r="CQ38" t="inlineStr"/>
+      <c r="CR38" t="inlineStr"/>
+      <c r="CS38" t="inlineStr"/>
+      <c r="CT38" t="inlineStr"/>
+      <c r="CU38" t="inlineStr"/>
+      <c r="CV38" t="inlineStr"/>
+      <c r="CW38" t="inlineStr"/>
+      <c r="CX38" t="inlineStr"/>
+      <c r="CY38" t="inlineStr"/>
+      <c r="CZ38" t="inlineStr"/>
+      <c r="DA38" t="inlineStr"/>
+      <c r="DB38" t="inlineStr"/>
+      <c r="DC38" t="inlineStr"/>
+      <c r="DD38" t="inlineStr"/>
+      <c r="DE38" t="inlineStr"/>
+      <c r="DF38" t="inlineStr"/>
+      <c r="DG38" t="inlineStr"/>
+      <c r="DH38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -9159,6 +11259,56 @@
       <c r="BJ39" t="n">
         <v>0.005872685742408556</v>
       </c>
+      <c r="BK39" t="inlineStr"/>
+      <c r="BL39" t="inlineStr"/>
+      <c r="BM39" t="inlineStr"/>
+      <c r="BN39" t="inlineStr"/>
+      <c r="BO39" t="inlineStr"/>
+      <c r="BP39" t="inlineStr"/>
+      <c r="BQ39" t="inlineStr"/>
+      <c r="BR39" t="inlineStr"/>
+      <c r="BS39" t="inlineStr"/>
+      <c r="BT39" t="inlineStr"/>
+      <c r="BU39" t="inlineStr"/>
+      <c r="BV39" t="inlineStr"/>
+      <c r="BW39" t="inlineStr"/>
+      <c r="BX39" t="inlineStr"/>
+      <c r="BY39" t="inlineStr"/>
+      <c r="BZ39" t="inlineStr"/>
+      <c r="CA39" t="inlineStr"/>
+      <c r="CB39" t="inlineStr"/>
+      <c r="CC39" t="inlineStr"/>
+      <c r="CD39" t="inlineStr"/>
+      <c r="CE39" t="inlineStr"/>
+      <c r="CF39" t="inlineStr"/>
+      <c r="CG39" t="inlineStr"/>
+      <c r="CH39" t="inlineStr"/>
+      <c r="CI39" t="inlineStr"/>
+      <c r="CJ39" t="inlineStr"/>
+      <c r="CK39" t="inlineStr"/>
+      <c r="CL39" t="inlineStr"/>
+      <c r="CM39" t="inlineStr"/>
+      <c r="CN39" t="inlineStr"/>
+      <c r="CO39" t="inlineStr"/>
+      <c r="CP39" t="inlineStr"/>
+      <c r="CQ39" t="inlineStr"/>
+      <c r="CR39" t="inlineStr"/>
+      <c r="CS39" t="inlineStr"/>
+      <c r="CT39" t="inlineStr"/>
+      <c r="CU39" t="inlineStr"/>
+      <c r="CV39" t="inlineStr"/>
+      <c r="CW39" t="inlineStr"/>
+      <c r="CX39" t="inlineStr"/>
+      <c r="CY39" t="inlineStr"/>
+      <c r="CZ39" t="inlineStr"/>
+      <c r="DA39" t="inlineStr"/>
+      <c r="DB39" t="inlineStr"/>
+      <c r="DC39" t="inlineStr"/>
+      <c r="DD39" t="inlineStr"/>
+      <c r="DE39" t="inlineStr"/>
+      <c r="DF39" t="inlineStr"/>
+      <c r="DG39" t="inlineStr"/>
+      <c r="DH39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -9379,6 +11529,56 @@
       <c r="BJ40" t="n">
         <v>0.006459060535969795</v>
       </c>
+      <c r="BK40" t="inlineStr"/>
+      <c r="BL40" t="inlineStr"/>
+      <c r="BM40" t="inlineStr"/>
+      <c r="BN40" t="inlineStr"/>
+      <c r="BO40" t="inlineStr"/>
+      <c r="BP40" t="inlineStr"/>
+      <c r="BQ40" t="inlineStr"/>
+      <c r="BR40" t="inlineStr"/>
+      <c r="BS40" t="inlineStr"/>
+      <c r="BT40" t="inlineStr"/>
+      <c r="BU40" t="inlineStr"/>
+      <c r="BV40" t="inlineStr"/>
+      <c r="BW40" t="inlineStr"/>
+      <c r="BX40" t="inlineStr"/>
+      <c r="BY40" t="inlineStr"/>
+      <c r="BZ40" t="inlineStr"/>
+      <c r="CA40" t="inlineStr"/>
+      <c r="CB40" t="inlineStr"/>
+      <c r="CC40" t="inlineStr"/>
+      <c r="CD40" t="inlineStr"/>
+      <c r="CE40" t="inlineStr"/>
+      <c r="CF40" t="inlineStr"/>
+      <c r="CG40" t="inlineStr"/>
+      <c r="CH40" t="inlineStr"/>
+      <c r="CI40" t="inlineStr"/>
+      <c r="CJ40" t="inlineStr"/>
+      <c r="CK40" t="inlineStr"/>
+      <c r="CL40" t="inlineStr"/>
+      <c r="CM40" t="inlineStr"/>
+      <c r="CN40" t="inlineStr"/>
+      <c r="CO40" t="inlineStr"/>
+      <c r="CP40" t="inlineStr"/>
+      <c r="CQ40" t="inlineStr"/>
+      <c r="CR40" t="inlineStr"/>
+      <c r="CS40" t="inlineStr"/>
+      <c r="CT40" t="inlineStr"/>
+      <c r="CU40" t="inlineStr"/>
+      <c r="CV40" t="inlineStr"/>
+      <c r="CW40" t="inlineStr"/>
+      <c r="CX40" t="inlineStr"/>
+      <c r="CY40" t="inlineStr"/>
+      <c r="CZ40" t="inlineStr"/>
+      <c r="DA40" t="inlineStr"/>
+      <c r="DB40" t="inlineStr"/>
+      <c r="DC40" t="inlineStr"/>
+      <c r="DD40" t="inlineStr"/>
+      <c r="DE40" t="inlineStr"/>
+      <c r="DF40" t="inlineStr"/>
+      <c r="DG40" t="inlineStr"/>
+      <c r="DH40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -9599,6 +11799,56 @@
       <c r="BJ41" t="n">
         <v>0.005749128469435981</v>
       </c>
+      <c r="BK41" t="inlineStr"/>
+      <c r="BL41" t="inlineStr"/>
+      <c r="BM41" t="inlineStr"/>
+      <c r="BN41" t="inlineStr"/>
+      <c r="BO41" t="inlineStr"/>
+      <c r="BP41" t="inlineStr"/>
+      <c r="BQ41" t="inlineStr"/>
+      <c r="BR41" t="inlineStr"/>
+      <c r="BS41" t="inlineStr"/>
+      <c r="BT41" t="inlineStr"/>
+      <c r="BU41" t="inlineStr"/>
+      <c r="BV41" t="inlineStr"/>
+      <c r="BW41" t="inlineStr"/>
+      <c r="BX41" t="inlineStr"/>
+      <c r="BY41" t="inlineStr"/>
+      <c r="BZ41" t="inlineStr"/>
+      <c r="CA41" t="inlineStr"/>
+      <c r="CB41" t="inlineStr"/>
+      <c r="CC41" t="inlineStr"/>
+      <c r="CD41" t="inlineStr"/>
+      <c r="CE41" t="inlineStr"/>
+      <c r="CF41" t="inlineStr"/>
+      <c r="CG41" t="inlineStr"/>
+      <c r="CH41" t="inlineStr"/>
+      <c r="CI41" t="inlineStr"/>
+      <c r="CJ41" t="inlineStr"/>
+      <c r="CK41" t="inlineStr"/>
+      <c r="CL41" t="inlineStr"/>
+      <c r="CM41" t="inlineStr"/>
+      <c r="CN41" t="inlineStr"/>
+      <c r="CO41" t="inlineStr"/>
+      <c r="CP41" t="inlineStr"/>
+      <c r="CQ41" t="inlineStr"/>
+      <c r="CR41" t="inlineStr"/>
+      <c r="CS41" t="inlineStr"/>
+      <c r="CT41" t="inlineStr"/>
+      <c r="CU41" t="inlineStr"/>
+      <c r="CV41" t="inlineStr"/>
+      <c r="CW41" t="inlineStr"/>
+      <c r="CX41" t="inlineStr"/>
+      <c r="CY41" t="inlineStr"/>
+      <c r="CZ41" t="inlineStr"/>
+      <c r="DA41" t="inlineStr"/>
+      <c r="DB41" t="inlineStr"/>
+      <c r="DC41" t="inlineStr"/>
+      <c r="DD41" t="inlineStr"/>
+      <c r="DE41" t="inlineStr"/>
+      <c r="DF41" t="inlineStr"/>
+      <c r="DG41" t="inlineStr"/>
+      <c r="DH41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -9819,6 +12069,56 @@
       <c r="BJ42" t="n">
         <v>0.002583684299501075</v>
       </c>
+      <c r="BK42" t="inlineStr"/>
+      <c r="BL42" t="inlineStr"/>
+      <c r="BM42" t="inlineStr"/>
+      <c r="BN42" t="inlineStr"/>
+      <c r="BO42" t="inlineStr"/>
+      <c r="BP42" t="inlineStr"/>
+      <c r="BQ42" t="inlineStr"/>
+      <c r="BR42" t="inlineStr"/>
+      <c r="BS42" t="inlineStr"/>
+      <c r="BT42" t="inlineStr"/>
+      <c r="BU42" t="inlineStr"/>
+      <c r="BV42" t="inlineStr"/>
+      <c r="BW42" t="inlineStr"/>
+      <c r="BX42" t="inlineStr"/>
+      <c r="BY42" t="inlineStr"/>
+      <c r="BZ42" t="inlineStr"/>
+      <c r="CA42" t="inlineStr"/>
+      <c r="CB42" t="inlineStr"/>
+      <c r="CC42" t="inlineStr"/>
+      <c r="CD42" t="inlineStr"/>
+      <c r="CE42" t="inlineStr"/>
+      <c r="CF42" t="inlineStr"/>
+      <c r="CG42" t="inlineStr"/>
+      <c r="CH42" t="inlineStr"/>
+      <c r="CI42" t="inlineStr"/>
+      <c r="CJ42" t="inlineStr"/>
+      <c r="CK42" t="inlineStr"/>
+      <c r="CL42" t="inlineStr"/>
+      <c r="CM42" t="inlineStr"/>
+      <c r="CN42" t="inlineStr"/>
+      <c r="CO42" t="inlineStr"/>
+      <c r="CP42" t="inlineStr"/>
+      <c r="CQ42" t="inlineStr"/>
+      <c r="CR42" t="inlineStr"/>
+      <c r="CS42" t="inlineStr"/>
+      <c r="CT42" t="inlineStr"/>
+      <c r="CU42" t="inlineStr"/>
+      <c r="CV42" t="inlineStr"/>
+      <c r="CW42" t="inlineStr"/>
+      <c r="CX42" t="inlineStr"/>
+      <c r="CY42" t="inlineStr"/>
+      <c r="CZ42" t="inlineStr"/>
+      <c r="DA42" t="inlineStr"/>
+      <c r="DB42" t="inlineStr"/>
+      <c r="DC42" t="inlineStr"/>
+      <c r="DD42" t="inlineStr"/>
+      <c r="DE42" t="inlineStr"/>
+      <c r="DF42" t="inlineStr"/>
+      <c r="DG42" t="inlineStr"/>
+      <c r="DH42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -10039,6 +12339,56 @@
       <c r="BJ43" t="n">
         <v>0.003602719364528168</v>
       </c>
+      <c r="BK43" t="inlineStr"/>
+      <c r="BL43" t="inlineStr"/>
+      <c r="BM43" t="inlineStr"/>
+      <c r="BN43" t="inlineStr"/>
+      <c r="BO43" t="inlineStr"/>
+      <c r="BP43" t="inlineStr"/>
+      <c r="BQ43" t="inlineStr"/>
+      <c r="BR43" t="inlineStr"/>
+      <c r="BS43" t="inlineStr"/>
+      <c r="BT43" t="inlineStr"/>
+      <c r="BU43" t="inlineStr"/>
+      <c r="BV43" t="inlineStr"/>
+      <c r="BW43" t="inlineStr"/>
+      <c r="BX43" t="inlineStr"/>
+      <c r="BY43" t="inlineStr"/>
+      <c r="BZ43" t="inlineStr"/>
+      <c r="CA43" t="inlineStr"/>
+      <c r="CB43" t="inlineStr"/>
+      <c r="CC43" t="inlineStr"/>
+      <c r="CD43" t="inlineStr"/>
+      <c r="CE43" t="inlineStr"/>
+      <c r="CF43" t="inlineStr"/>
+      <c r="CG43" t="inlineStr"/>
+      <c r="CH43" t="inlineStr"/>
+      <c r="CI43" t="inlineStr"/>
+      <c r="CJ43" t="inlineStr"/>
+      <c r="CK43" t="inlineStr"/>
+      <c r="CL43" t="inlineStr"/>
+      <c r="CM43" t="inlineStr"/>
+      <c r="CN43" t="inlineStr"/>
+      <c r="CO43" t="inlineStr"/>
+      <c r="CP43" t="inlineStr"/>
+      <c r="CQ43" t="inlineStr"/>
+      <c r="CR43" t="inlineStr"/>
+      <c r="CS43" t="inlineStr"/>
+      <c r="CT43" t="inlineStr"/>
+      <c r="CU43" t="inlineStr"/>
+      <c r="CV43" t="inlineStr"/>
+      <c r="CW43" t="inlineStr"/>
+      <c r="CX43" t="inlineStr"/>
+      <c r="CY43" t="inlineStr"/>
+      <c r="CZ43" t="inlineStr"/>
+      <c r="DA43" t="inlineStr"/>
+      <c r="DB43" t="inlineStr"/>
+      <c r="DC43" t="inlineStr"/>
+      <c r="DD43" t="inlineStr"/>
+      <c r="DE43" t="inlineStr"/>
+      <c r="DF43" t="inlineStr"/>
+      <c r="DG43" t="inlineStr"/>
+      <c r="DH43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -10259,6 +12609,56 @@
       <c r="BJ44" t="n">
         <v>0.007162357584063435</v>
       </c>
+      <c r="BK44" t="inlineStr"/>
+      <c r="BL44" t="inlineStr"/>
+      <c r="BM44" t="inlineStr"/>
+      <c r="BN44" t="inlineStr"/>
+      <c r="BO44" t="inlineStr"/>
+      <c r="BP44" t="inlineStr"/>
+      <c r="BQ44" t="inlineStr"/>
+      <c r="BR44" t="inlineStr"/>
+      <c r="BS44" t="inlineStr"/>
+      <c r="BT44" t="inlineStr"/>
+      <c r="BU44" t="inlineStr"/>
+      <c r="BV44" t="inlineStr"/>
+      <c r="BW44" t="inlineStr"/>
+      <c r="BX44" t="inlineStr"/>
+      <c r="BY44" t="inlineStr"/>
+      <c r="BZ44" t="inlineStr"/>
+      <c r="CA44" t="inlineStr"/>
+      <c r="CB44" t="inlineStr"/>
+      <c r="CC44" t="inlineStr"/>
+      <c r="CD44" t="inlineStr"/>
+      <c r="CE44" t="inlineStr"/>
+      <c r="CF44" t="inlineStr"/>
+      <c r="CG44" t="inlineStr"/>
+      <c r="CH44" t="inlineStr"/>
+      <c r="CI44" t="inlineStr"/>
+      <c r="CJ44" t="inlineStr"/>
+      <c r="CK44" t="inlineStr"/>
+      <c r="CL44" t="inlineStr"/>
+      <c r="CM44" t="inlineStr"/>
+      <c r="CN44" t="inlineStr"/>
+      <c r="CO44" t="inlineStr"/>
+      <c r="CP44" t="inlineStr"/>
+      <c r="CQ44" t="inlineStr"/>
+      <c r="CR44" t="inlineStr"/>
+      <c r="CS44" t="inlineStr"/>
+      <c r="CT44" t="inlineStr"/>
+      <c r="CU44" t="inlineStr"/>
+      <c r="CV44" t="inlineStr"/>
+      <c r="CW44" t="inlineStr"/>
+      <c r="CX44" t="inlineStr"/>
+      <c r="CY44" t="inlineStr"/>
+      <c r="CZ44" t="inlineStr"/>
+      <c r="DA44" t="inlineStr"/>
+      <c r="DB44" t="inlineStr"/>
+      <c r="DC44" t="inlineStr"/>
+      <c r="DD44" t="inlineStr"/>
+      <c r="DE44" t="inlineStr"/>
+      <c r="DF44" t="inlineStr"/>
+      <c r="DG44" t="inlineStr"/>
+      <c r="DH44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -10479,6 +12879,56 @@
       <c r="BJ45" t="n">
         <v>0.004703518105213435</v>
       </c>
+      <c r="BK45" t="inlineStr"/>
+      <c r="BL45" t="inlineStr"/>
+      <c r="BM45" t="inlineStr"/>
+      <c r="BN45" t="inlineStr"/>
+      <c r="BO45" t="inlineStr"/>
+      <c r="BP45" t="inlineStr"/>
+      <c r="BQ45" t="inlineStr"/>
+      <c r="BR45" t="inlineStr"/>
+      <c r="BS45" t="inlineStr"/>
+      <c r="BT45" t="inlineStr"/>
+      <c r="BU45" t="inlineStr"/>
+      <c r="BV45" t="inlineStr"/>
+      <c r="BW45" t="inlineStr"/>
+      <c r="BX45" t="inlineStr"/>
+      <c r="BY45" t="inlineStr"/>
+      <c r="BZ45" t="inlineStr"/>
+      <c r="CA45" t="inlineStr"/>
+      <c r="CB45" t="inlineStr"/>
+      <c r="CC45" t="inlineStr"/>
+      <c r="CD45" t="inlineStr"/>
+      <c r="CE45" t="inlineStr"/>
+      <c r="CF45" t="inlineStr"/>
+      <c r="CG45" t="inlineStr"/>
+      <c r="CH45" t="inlineStr"/>
+      <c r="CI45" t="inlineStr"/>
+      <c r="CJ45" t="inlineStr"/>
+      <c r="CK45" t="inlineStr"/>
+      <c r="CL45" t="inlineStr"/>
+      <c r="CM45" t="inlineStr"/>
+      <c r="CN45" t="inlineStr"/>
+      <c r="CO45" t="inlineStr"/>
+      <c r="CP45" t="inlineStr"/>
+      <c r="CQ45" t="inlineStr"/>
+      <c r="CR45" t="inlineStr"/>
+      <c r="CS45" t="inlineStr"/>
+      <c r="CT45" t="inlineStr"/>
+      <c r="CU45" t="inlineStr"/>
+      <c r="CV45" t="inlineStr"/>
+      <c r="CW45" t="inlineStr"/>
+      <c r="CX45" t="inlineStr"/>
+      <c r="CY45" t="inlineStr"/>
+      <c r="CZ45" t="inlineStr"/>
+      <c r="DA45" t="inlineStr"/>
+      <c r="DB45" t="inlineStr"/>
+      <c r="DC45" t="inlineStr"/>
+      <c r="DD45" t="inlineStr"/>
+      <c r="DE45" t="inlineStr"/>
+      <c r="DF45" t="inlineStr"/>
+      <c r="DG45" t="inlineStr"/>
+      <c r="DH45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -10699,6 +13149,56 @@
       <c r="BJ46" t="n">
         <v>0.0002690319894887233</v>
       </c>
+      <c r="BK46" t="inlineStr"/>
+      <c r="BL46" t="inlineStr"/>
+      <c r="BM46" t="inlineStr"/>
+      <c r="BN46" t="inlineStr"/>
+      <c r="BO46" t="inlineStr"/>
+      <c r="BP46" t="inlineStr"/>
+      <c r="BQ46" t="inlineStr"/>
+      <c r="BR46" t="inlineStr"/>
+      <c r="BS46" t="inlineStr"/>
+      <c r="BT46" t="inlineStr"/>
+      <c r="BU46" t="inlineStr"/>
+      <c r="BV46" t="inlineStr"/>
+      <c r="BW46" t="inlineStr"/>
+      <c r="BX46" t="inlineStr"/>
+      <c r="BY46" t="inlineStr"/>
+      <c r="BZ46" t="inlineStr"/>
+      <c r="CA46" t="inlineStr"/>
+      <c r="CB46" t="inlineStr"/>
+      <c r="CC46" t="inlineStr"/>
+      <c r="CD46" t="inlineStr"/>
+      <c r="CE46" t="inlineStr"/>
+      <c r="CF46" t="inlineStr"/>
+      <c r="CG46" t="inlineStr"/>
+      <c r="CH46" t="inlineStr"/>
+      <c r="CI46" t="inlineStr"/>
+      <c r="CJ46" t="inlineStr"/>
+      <c r="CK46" t="inlineStr"/>
+      <c r="CL46" t="inlineStr"/>
+      <c r="CM46" t="inlineStr"/>
+      <c r="CN46" t="inlineStr"/>
+      <c r="CO46" t="inlineStr"/>
+      <c r="CP46" t="inlineStr"/>
+      <c r="CQ46" t="inlineStr"/>
+      <c r="CR46" t="inlineStr"/>
+      <c r="CS46" t="inlineStr"/>
+      <c r="CT46" t="inlineStr"/>
+      <c r="CU46" t="inlineStr"/>
+      <c r="CV46" t="inlineStr"/>
+      <c r="CW46" t="inlineStr"/>
+      <c r="CX46" t="inlineStr"/>
+      <c r="CY46" t="inlineStr"/>
+      <c r="CZ46" t="inlineStr"/>
+      <c r="DA46" t="inlineStr"/>
+      <c r="DB46" t="inlineStr"/>
+      <c r="DC46" t="inlineStr"/>
+      <c r="DD46" t="inlineStr"/>
+      <c r="DE46" t="inlineStr"/>
+      <c r="DF46" t="inlineStr"/>
+      <c r="DG46" t="inlineStr"/>
+      <c r="DH46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -10919,6 +13419,56 @@
       <c r="BJ47" t="n">
         <v>4.189518119265814e-05</v>
       </c>
+      <c r="BK47" t="inlineStr"/>
+      <c r="BL47" t="inlineStr"/>
+      <c r="BM47" t="inlineStr"/>
+      <c r="BN47" t="inlineStr"/>
+      <c r="BO47" t="inlineStr"/>
+      <c r="BP47" t="inlineStr"/>
+      <c r="BQ47" t="inlineStr"/>
+      <c r="BR47" t="inlineStr"/>
+      <c r="BS47" t="inlineStr"/>
+      <c r="BT47" t="inlineStr"/>
+      <c r="BU47" t="inlineStr"/>
+      <c r="BV47" t="inlineStr"/>
+      <c r="BW47" t="inlineStr"/>
+      <c r="BX47" t="inlineStr"/>
+      <c r="BY47" t="inlineStr"/>
+      <c r="BZ47" t="inlineStr"/>
+      <c r="CA47" t="inlineStr"/>
+      <c r="CB47" t="inlineStr"/>
+      <c r="CC47" t="inlineStr"/>
+      <c r="CD47" t="inlineStr"/>
+      <c r="CE47" t="inlineStr"/>
+      <c r="CF47" t="inlineStr"/>
+      <c r="CG47" t="inlineStr"/>
+      <c r="CH47" t="inlineStr"/>
+      <c r="CI47" t="inlineStr"/>
+      <c r="CJ47" t="inlineStr"/>
+      <c r="CK47" t="inlineStr"/>
+      <c r="CL47" t="inlineStr"/>
+      <c r="CM47" t="inlineStr"/>
+      <c r="CN47" t="inlineStr"/>
+      <c r="CO47" t="inlineStr"/>
+      <c r="CP47" t="inlineStr"/>
+      <c r="CQ47" t="inlineStr"/>
+      <c r="CR47" t="inlineStr"/>
+      <c r="CS47" t="inlineStr"/>
+      <c r="CT47" t="inlineStr"/>
+      <c r="CU47" t="inlineStr"/>
+      <c r="CV47" t="inlineStr"/>
+      <c r="CW47" t="inlineStr"/>
+      <c r="CX47" t="inlineStr"/>
+      <c r="CY47" t="inlineStr"/>
+      <c r="CZ47" t="inlineStr"/>
+      <c r="DA47" t="inlineStr"/>
+      <c r="DB47" t="inlineStr"/>
+      <c r="DC47" t="inlineStr"/>
+      <c r="DD47" t="inlineStr"/>
+      <c r="DE47" t="inlineStr"/>
+      <c r="DF47" t="inlineStr"/>
+      <c r="DG47" t="inlineStr"/>
+      <c r="DH47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -11149,6 +13699,56 @@
       <c r="BJ48" t="n">
         <v>9.712984233428587e-06</v>
       </c>
+      <c r="BK48" t="inlineStr"/>
+      <c r="BL48" t="inlineStr"/>
+      <c r="BM48" t="inlineStr"/>
+      <c r="BN48" t="inlineStr"/>
+      <c r="BO48" t="inlineStr"/>
+      <c r="BP48" t="inlineStr"/>
+      <c r="BQ48" t="inlineStr"/>
+      <c r="BR48" t="inlineStr"/>
+      <c r="BS48" t="inlineStr"/>
+      <c r="BT48" t="inlineStr"/>
+      <c r="BU48" t="inlineStr"/>
+      <c r="BV48" t="inlineStr"/>
+      <c r="BW48" t="inlineStr"/>
+      <c r="BX48" t="inlineStr"/>
+      <c r="BY48" t="inlineStr"/>
+      <c r="BZ48" t="inlineStr"/>
+      <c r="CA48" t="inlineStr"/>
+      <c r="CB48" t="inlineStr"/>
+      <c r="CC48" t="inlineStr"/>
+      <c r="CD48" t="inlineStr"/>
+      <c r="CE48" t="inlineStr"/>
+      <c r="CF48" t="inlineStr"/>
+      <c r="CG48" t="inlineStr"/>
+      <c r="CH48" t="inlineStr"/>
+      <c r="CI48" t="inlineStr"/>
+      <c r="CJ48" t="inlineStr"/>
+      <c r="CK48" t="inlineStr"/>
+      <c r="CL48" t="inlineStr"/>
+      <c r="CM48" t="inlineStr"/>
+      <c r="CN48" t="inlineStr"/>
+      <c r="CO48" t="inlineStr"/>
+      <c r="CP48" t="inlineStr"/>
+      <c r="CQ48" t="inlineStr"/>
+      <c r="CR48" t="inlineStr"/>
+      <c r="CS48" t="inlineStr"/>
+      <c r="CT48" t="inlineStr"/>
+      <c r="CU48" t="inlineStr"/>
+      <c r="CV48" t="inlineStr"/>
+      <c r="CW48" t="inlineStr"/>
+      <c r="CX48" t="inlineStr"/>
+      <c r="CY48" t="inlineStr"/>
+      <c r="CZ48" t="inlineStr"/>
+      <c r="DA48" t="inlineStr"/>
+      <c r="DB48" t="inlineStr"/>
+      <c r="DC48" t="inlineStr"/>
+      <c r="DD48" t="inlineStr"/>
+      <c r="DE48" t="inlineStr"/>
+      <c r="DF48" t="inlineStr"/>
+      <c r="DG48" t="inlineStr"/>
+      <c r="DH48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -11379,6 +13979,56 @@
       <c r="BJ49" t="n">
         <v>4.196248604251576e-17</v>
       </c>
+      <c r="BK49" t="inlineStr"/>
+      <c r="BL49" t="inlineStr"/>
+      <c r="BM49" t="inlineStr"/>
+      <c r="BN49" t="inlineStr"/>
+      <c r="BO49" t="inlineStr"/>
+      <c r="BP49" t="inlineStr"/>
+      <c r="BQ49" t="inlineStr"/>
+      <c r="BR49" t="inlineStr"/>
+      <c r="BS49" t="inlineStr"/>
+      <c r="BT49" t="inlineStr"/>
+      <c r="BU49" t="inlineStr"/>
+      <c r="BV49" t="inlineStr"/>
+      <c r="BW49" t="inlineStr"/>
+      <c r="BX49" t="inlineStr"/>
+      <c r="BY49" t="inlineStr"/>
+      <c r="BZ49" t="inlineStr"/>
+      <c r="CA49" t="inlineStr"/>
+      <c r="CB49" t="inlineStr"/>
+      <c r="CC49" t="inlineStr"/>
+      <c r="CD49" t="inlineStr"/>
+      <c r="CE49" t="inlineStr"/>
+      <c r="CF49" t="inlineStr"/>
+      <c r="CG49" t="inlineStr"/>
+      <c r="CH49" t="inlineStr"/>
+      <c r="CI49" t="inlineStr"/>
+      <c r="CJ49" t="inlineStr"/>
+      <c r="CK49" t="inlineStr"/>
+      <c r="CL49" t="inlineStr"/>
+      <c r="CM49" t="inlineStr"/>
+      <c r="CN49" t="inlineStr"/>
+      <c r="CO49" t="inlineStr"/>
+      <c r="CP49" t="inlineStr"/>
+      <c r="CQ49" t="inlineStr"/>
+      <c r="CR49" t="inlineStr"/>
+      <c r="CS49" t="inlineStr"/>
+      <c r="CT49" t="inlineStr"/>
+      <c r="CU49" t="inlineStr"/>
+      <c r="CV49" t="inlineStr"/>
+      <c r="CW49" t="inlineStr"/>
+      <c r="CX49" t="inlineStr"/>
+      <c r="CY49" t="inlineStr"/>
+      <c r="CZ49" t="inlineStr"/>
+      <c r="DA49" t="inlineStr"/>
+      <c r="DB49" t="inlineStr"/>
+      <c r="DC49" t="inlineStr"/>
+      <c r="DD49" t="inlineStr"/>
+      <c r="DE49" t="inlineStr"/>
+      <c r="DF49" t="inlineStr"/>
+      <c r="DG49" t="inlineStr"/>
+      <c r="DH49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -11599,6 +14249,56 @@
       <c r="BJ50" t="n">
         <v>0.01108411101526533</v>
       </c>
+      <c r="BK50" t="inlineStr"/>
+      <c r="BL50" t="inlineStr"/>
+      <c r="BM50" t="inlineStr"/>
+      <c r="BN50" t="inlineStr"/>
+      <c r="BO50" t="inlineStr"/>
+      <c r="BP50" t="inlineStr"/>
+      <c r="BQ50" t="inlineStr"/>
+      <c r="BR50" t="inlineStr"/>
+      <c r="BS50" t="inlineStr"/>
+      <c r="BT50" t="inlineStr"/>
+      <c r="BU50" t="inlineStr"/>
+      <c r="BV50" t="inlineStr"/>
+      <c r="BW50" t="inlineStr"/>
+      <c r="BX50" t="inlineStr"/>
+      <c r="BY50" t="inlineStr"/>
+      <c r="BZ50" t="inlineStr"/>
+      <c r="CA50" t="inlineStr"/>
+      <c r="CB50" t="inlineStr"/>
+      <c r="CC50" t="inlineStr"/>
+      <c r="CD50" t="inlineStr"/>
+      <c r="CE50" t="inlineStr"/>
+      <c r="CF50" t="inlineStr"/>
+      <c r="CG50" t="inlineStr"/>
+      <c r="CH50" t="inlineStr"/>
+      <c r="CI50" t="inlineStr"/>
+      <c r="CJ50" t="inlineStr"/>
+      <c r="CK50" t="inlineStr"/>
+      <c r="CL50" t="inlineStr"/>
+      <c r="CM50" t="inlineStr"/>
+      <c r="CN50" t="inlineStr"/>
+      <c r="CO50" t="inlineStr"/>
+      <c r="CP50" t="inlineStr"/>
+      <c r="CQ50" t="inlineStr"/>
+      <c r="CR50" t="inlineStr"/>
+      <c r="CS50" t="inlineStr"/>
+      <c r="CT50" t="inlineStr"/>
+      <c r="CU50" t="inlineStr"/>
+      <c r="CV50" t="inlineStr"/>
+      <c r="CW50" t="inlineStr"/>
+      <c r="CX50" t="inlineStr"/>
+      <c r="CY50" t="inlineStr"/>
+      <c r="CZ50" t="inlineStr"/>
+      <c r="DA50" t="inlineStr"/>
+      <c r="DB50" t="inlineStr"/>
+      <c r="DC50" t="inlineStr"/>
+      <c r="DD50" t="inlineStr"/>
+      <c r="DE50" t="inlineStr"/>
+      <c r="DF50" t="inlineStr"/>
+      <c r="DG50" t="inlineStr"/>
+      <c r="DH50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -11819,6 +14519,56 @@
       <c r="BJ51" t="n">
         <v>0.004629350087943543</v>
       </c>
+      <c r="BK51" t="inlineStr"/>
+      <c r="BL51" t="inlineStr"/>
+      <c r="BM51" t="inlineStr"/>
+      <c r="BN51" t="inlineStr"/>
+      <c r="BO51" t="inlineStr"/>
+      <c r="BP51" t="inlineStr"/>
+      <c r="BQ51" t="inlineStr"/>
+      <c r="BR51" t="inlineStr"/>
+      <c r="BS51" t="inlineStr"/>
+      <c r="BT51" t="inlineStr"/>
+      <c r="BU51" t="inlineStr"/>
+      <c r="BV51" t="inlineStr"/>
+      <c r="BW51" t="inlineStr"/>
+      <c r="BX51" t="inlineStr"/>
+      <c r="BY51" t="inlineStr"/>
+      <c r="BZ51" t="inlineStr"/>
+      <c r="CA51" t="inlineStr"/>
+      <c r="CB51" t="inlineStr"/>
+      <c r="CC51" t="inlineStr"/>
+      <c r="CD51" t="inlineStr"/>
+      <c r="CE51" t="inlineStr"/>
+      <c r="CF51" t="inlineStr"/>
+      <c r="CG51" t="inlineStr"/>
+      <c r="CH51" t="inlineStr"/>
+      <c r="CI51" t="inlineStr"/>
+      <c r="CJ51" t="inlineStr"/>
+      <c r="CK51" t="inlineStr"/>
+      <c r="CL51" t="inlineStr"/>
+      <c r="CM51" t="inlineStr"/>
+      <c r="CN51" t="inlineStr"/>
+      <c r="CO51" t="inlineStr"/>
+      <c r="CP51" t="inlineStr"/>
+      <c r="CQ51" t="inlineStr"/>
+      <c r="CR51" t="inlineStr"/>
+      <c r="CS51" t="inlineStr"/>
+      <c r="CT51" t="inlineStr"/>
+      <c r="CU51" t="inlineStr"/>
+      <c r="CV51" t="inlineStr"/>
+      <c r="CW51" t="inlineStr"/>
+      <c r="CX51" t="inlineStr"/>
+      <c r="CY51" t="inlineStr"/>
+      <c r="CZ51" t="inlineStr"/>
+      <c r="DA51" t="inlineStr"/>
+      <c r="DB51" t="inlineStr"/>
+      <c r="DC51" t="inlineStr"/>
+      <c r="DD51" t="inlineStr"/>
+      <c r="DE51" t="inlineStr"/>
+      <c r="DF51" t="inlineStr"/>
+      <c r="DG51" t="inlineStr"/>
+      <c r="DH51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -12039,6 +14789,56 @@
       <c r="BJ52" t="n">
         <v>0.009056712480178981</v>
       </c>
+      <c r="BK52" t="inlineStr"/>
+      <c r="BL52" t="inlineStr"/>
+      <c r="BM52" t="inlineStr"/>
+      <c r="BN52" t="inlineStr"/>
+      <c r="BO52" t="inlineStr"/>
+      <c r="BP52" t="inlineStr"/>
+      <c r="BQ52" t="inlineStr"/>
+      <c r="BR52" t="inlineStr"/>
+      <c r="BS52" t="inlineStr"/>
+      <c r="BT52" t="inlineStr"/>
+      <c r="BU52" t="inlineStr"/>
+      <c r="BV52" t="inlineStr"/>
+      <c r="BW52" t="inlineStr"/>
+      <c r="BX52" t="inlineStr"/>
+      <c r="BY52" t="inlineStr"/>
+      <c r="BZ52" t="inlineStr"/>
+      <c r="CA52" t="inlineStr"/>
+      <c r="CB52" t="inlineStr"/>
+      <c r="CC52" t="inlineStr"/>
+      <c r="CD52" t="inlineStr"/>
+      <c r="CE52" t="inlineStr"/>
+      <c r="CF52" t="inlineStr"/>
+      <c r="CG52" t="inlineStr"/>
+      <c r="CH52" t="inlineStr"/>
+      <c r="CI52" t="inlineStr"/>
+      <c r="CJ52" t="inlineStr"/>
+      <c r="CK52" t="inlineStr"/>
+      <c r="CL52" t="inlineStr"/>
+      <c r="CM52" t="inlineStr"/>
+      <c r="CN52" t="inlineStr"/>
+      <c r="CO52" t="inlineStr"/>
+      <c r="CP52" t="inlineStr"/>
+      <c r="CQ52" t="inlineStr"/>
+      <c r="CR52" t="inlineStr"/>
+      <c r="CS52" t="inlineStr"/>
+      <c r="CT52" t="inlineStr"/>
+      <c r="CU52" t="inlineStr"/>
+      <c r="CV52" t="inlineStr"/>
+      <c r="CW52" t="inlineStr"/>
+      <c r="CX52" t="inlineStr"/>
+      <c r="CY52" t="inlineStr"/>
+      <c r="CZ52" t="inlineStr"/>
+      <c r="DA52" t="inlineStr"/>
+      <c r="DB52" t="inlineStr"/>
+      <c r="DC52" t="inlineStr"/>
+      <c r="DD52" t="inlineStr"/>
+      <c r="DE52" t="inlineStr"/>
+      <c r="DF52" t="inlineStr"/>
+      <c r="DG52" t="inlineStr"/>
+      <c r="DH52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -12259,6 +15059,56 @@
       <c r="BJ53" t="n">
         <v>0.006631067788558371</v>
       </c>
+      <c r="BK53" t="inlineStr"/>
+      <c r="BL53" t="inlineStr"/>
+      <c r="BM53" t="inlineStr"/>
+      <c r="BN53" t="inlineStr"/>
+      <c r="BO53" t="inlineStr"/>
+      <c r="BP53" t="inlineStr"/>
+      <c r="BQ53" t="inlineStr"/>
+      <c r="BR53" t="inlineStr"/>
+      <c r="BS53" t="inlineStr"/>
+      <c r="BT53" t="inlineStr"/>
+      <c r="BU53" t="inlineStr"/>
+      <c r="BV53" t="inlineStr"/>
+      <c r="BW53" t="inlineStr"/>
+      <c r="BX53" t="inlineStr"/>
+      <c r="BY53" t="inlineStr"/>
+      <c r="BZ53" t="inlineStr"/>
+      <c r="CA53" t="inlineStr"/>
+      <c r="CB53" t="inlineStr"/>
+      <c r="CC53" t="inlineStr"/>
+      <c r="CD53" t="inlineStr"/>
+      <c r="CE53" t="inlineStr"/>
+      <c r="CF53" t="inlineStr"/>
+      <c r="CG53" t="inlineStr"/>
+      <c r="CH53" t="inlineStr"/>
+      <c r="CI53" t="inlineStr"/>
+      <c r="CJ53" t="inlineStr"/>
+      <c r="CK53" t="inlineStr"/>
+      <c r="CL53" t="inlineStr"/>
+      <c r="CM53" t="inlineStr"/>
+      <c r="CN53" t="inlineStr"/>
+      <c r="CO53" t="inlineStr"/>
+      <c r="CP53" t="inlineStr"/>
+      <c r="CQ53" t="inlineStr"/>
+      <c r="CR53" t="inlineStr"/>
+      <c r="CS53" t="inlineStr"/>
+      <c r="CT53" t="inlineStr"/>
+      <c r="CU53" t="inlineStr"/>
+      <c r="CV53" t="inlineStr"/>
+      <c r="CW53" t="inlineStr"/>
+      <c r="CX53" t="inlineStr"/>
+      <c r="CY53" t="inlineStr"/>
+      <c r="CZ53" t="inlineStr"/>
+      <c r="DA53" t="inlineStr"/>
+      <c r="DB53" t="inlineStr"/>
+      <c r="DC53" t="inlineStr"/>
+      <c r="DD53" t="inlineStr"/>
+      <c r="DE53" t="inlineStr"/>
+      <c r="DF53" t="inlineStr"/>
+      <c r="DG53" t="inlineStr"/>
+      <c r="DH53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -12479,6 +15329,56 @@
       <c r="BJ54" t="n">
         <v>0.00339265427510108</v>
       </c>
+      <c r="BK54" t="inlineStr"/>
+      <c r="BL54" t="inlineStr"/>
+      <c r="BM54" t="inlineStr"/>
+      <c r="BN54" t="inlineStr"/>
+      <c r="BO54" t="inlineStr"/>
+      <c r="BP54" t="inlineStr"/>
+      <c r="BQ54" t="inlineStr"/>
+      <c r="BR54" t="inlineStr"/>
+      <c r="BS54" t="inlineStr"/>
+      <c r="BT54" t="inlineStr"/>
+      <c r="BU54" t="inlineStr"/>
+      <c r="BV54" t="inlineStr"/>
+      <c r="BW54" t="inlineStr"/>
+      <c r="BX54" t="inlineStr"/>
+      <c r="BY54" t="inlineStr"/>
+      <c r="BZ54" t="inlineStr"/>
+      <c r="CA54" t="inlineStr"/>
+      <c r="CB54" t="inlineStr"/>
+      <c r="CC54" t="inlineStr"/>
+      <c r="CD54" t="inlineStr"/>
+      <c r="CE54" t="inlineStr"/>
+      <c r="CF54" t="inlineStr"/>
+      <c r="CG54" t="inlineStr"/>
+      <c r="CH54" t="inlineStr"/>
+      <c r="CI54" t="inlineStr"/>
+      <c r="CJ54" t="inlineStr"/>
+      <c r="CK54" t="inlineStr"/>
+      <c r="CL54" t="inlineStr"/>
+      <c r="CM54" t="inlineStr"/>
+      <c r="CN54" t="inlineStr"/>
+      <c r="CO54" t="inlineStr"/>
+      <c r="CP54" t="inlineStr"/>
+      <c r="CQ54" t="inlineStr"/>
+      <c r="CR54" t="inlineStr"/>
+      <c r="CS54" t="inlineStr"/>
+      <c r="CT54" t="inlineStr"/>
+      <c r="CU54" t="inlineStr"/>
+      <c r="CV54" t="inlineStr"/>
+      <c r="CW54" t="inlineStr"/>
+      <c r="CX54" t="inlineStr"/>
+      <c r="CY54" t="inlineStr"/>
+      <c r="CZ54" t="inlineStr"/>
+      <c r="DA54" t="inlineStr"/>
+      <c r="DB54" t="inlineStr"/>
+      <c r="DC54" t="inlineStr"/>
+      <c r="DD54" t="inlineStr"/>
+      <c r="DE54" t="inlineStr"/>
+      <c r="DF54" t="inlineStr"/>
+      <c r="DG54" t="inlineStr"/>
+      <c r="DH54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -12699,6 +15599,56 @@
       <c r="BJ55" t="n">
         <v>0.000936242175825913</v>
       </c>
+      <c r="BK55" t="inlineStr"/>
+      <c r="BL55" t="inlineStr"/>
+      <c r="BM55" t="inlineStr"/>
+      <c r="BN55" t="inlineStr"/>
+      <c r="BO55" t="inlineStr"/>
+      <c r="BP55" t="inlineStr"/>
+      <c r="BQ55" t="inlineStr"/>
+      <c r="BR55" t="inlineStr"/>
+      <c r="BS55" t="inlineStr"/>
+      <c r="BT55" t="inlineStr"/>
+      <c r="BU55" t="inlineStr"/>
+      <c r="BV55" t="inlineStr"/>
+      <c r="BW55" t="inlineStr"/>
+      <c r="BX55" t="inlineStr"/>
+      <c r="BY55" t="inlineStr"/>
+      <c r="BZ55" t="inlineStr"/>
+      <c r="CA55" t="inlineStr"/>
+      <c r="CB55" t="inlineStr"/>
+      <c r="CC55" t="inlineStr"/>
+      <c r="CD55" t="inlineStr"/>
+      <c r="CE55" t="inlineStr"/>
+      <c r="CF55" t="inlineStr"/>
+      <c r="CG55" t="inlineStr"/>
+      <c r="CH55" t="inlineStr"/>
+      <c r="CI55" t="inlineStr"/>
+      <c r="CJ55" t="inlineStr"/>
+      <c r="CK55" t="inlineStr"/>
+      <c r="CL55" t="inlineStr"/>
+      <c r="CM55" t="inlineStr"/>
+      <c r="CN55" t="inlineStr"/>
+      <c r="CO55" t="inlineStr"/>
+      <c r="CP55" t="inlineStr"/>
+      <c r="CQ55" t="inlineStr"/>
+      <c r="CR55" t="inlineStr"/>
+      <c r="CS55" t="inlineStr"/>
+      <c r="CT55" t="inlineStr"/>
+      <c r="CU55" t="inlineStr"/>
+      <c r="CV55" t="inlineStr"/>
+      <c r="CW55" t="inlineStr"/>
+      <c r="CX55" t="inlineStr"/>
+      <c r="CY55" t="inlineStr"/>
+      <c r="CZ55" t="inlineStr"/>
+      <c r="DA55" t="inlineStr"/>
+      <c r="DB55" t="inlineStr"/>
+      <c r="DC55" t="inlineStr"/>
+      <c r="DD55" t="inlineStr"/>
+      <c r="DE55" t="inlineStr"/>
+      <c r="DF55" t="inlineStr"/>
+      <c r="DG55" t="inlineStr"/>
+      <c r="DH55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -12919,6 +15869,56 @@
       <c r="BJ56" t="n">
         <v>9.712984233428587e-06</v>
       </c>
+      <c r="BK56" t="inlineStr"/>
+      <c r="BL56" t="inlineStr"/>
+      <c r="BM56" t="inlineStr"/>
+      <c r="BN56" t="inlineStr"/>
+      <c r="BO56" t="inlineStr"/>
+      <c r="BP56" t="inlineStr"/>
+      <c r="BQ56" t="inlineStr"/>
+      <c r="BR56" t="inlineStr"/>
+      <c r="BS56" t="inlineStr"/>
+      <c r="BT56" t="inlineStr"/>
+      <c r="BU56" t="inlineStr"/>
+      <c r="BV56" t="inlineStr"/>
+      <c r="BW56" t="inlineStr"/>
+      <c r="BX56" t="inlineStr"/>
+      <c r="BY56" t="inlineStr"/>
+      <c r="BZ56" t="inlineStr"/>
+      <c r="CA56" t="inlineStr"/>
+      <c r="CB56" t="inlineStr"/>
+      <c r="CC56" t="inlineStr"/>
+      <c r="CD56" t="inlineStr"/>
+      <c r="CE56" t="inlineStr"/>
+      <c r="CF56" t="inlineStr"/>
+      <c r="CG56" t="inlineStr"/>
+      <c r="CH56" t="inlineStr"/>
+      <c r="CI56" t="inlineStr"/>
+      <c r="CJ56" t="inlineStr"/>
+      <c r="CK56" t="inlineStr"/>
+      <c r="CL56" t="inlineStr"/>
+      <c r="CM56" t="inlineStr"/>
+      <c r="CN56" t="inlineStr"/>
+      <c r="CO56" t="inlineStr"/>
+      <c r="CP56" t="inlineStr"/>
+      <c r="CQ56" t="inlineStr"/>
+      <c r="CR56" t="inlineStr"/>
+      <c r="CS56" t="inlineStr"/>
+      <c r="CT56" t="inlineStr"/>
+      <c r="CU56" t="inlineStr"/>
+      <c r="CV56" t="inlineStr"/>
+      <c r="CW56" t="inlineStr"/>
+      <c r="CX56" t="inlineStr"/>
+      <c r="CY56" t="inlineStr"/>
+      <c r="CZ56" t="inlineStr"/>
+      <c r="DA56" t="inlineStr"/>
+      <c r="DB56" t="inlineStr"/>
+      <c r="DC56" t="inlineStr"/>
+      <c r="DD56" t="inlineStr"/>
+      <c r="DE56" t="inlineStr"/>
+      <c r="DF56" t="inlineStr"/>
+      <c r="DG56" t="inlineStr"/>
+      <c r="DH56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -13139,6 +16139,56 @@
       <c r="BJ57" t="n">
         <v>0</v>
       </c>
+      <c r="BK57" t="inlineStr"/>
+      <c r="BL57" t="inlineStr"/>
+      <c r="BM57" t="inlineStr"/>
+      <c r="BN57" t="inlineStr"/>
+      <c r="BO57" t="inlineStr"/>
+      <c r="BP57" t="inlineStr"/>
+      <c r="BQ57" t="inlineStr"/>
+      <c r="BR57" t="inlineStr"/>
+      <c r="BS57" t="inlineStr"/>
+      <c r="BT57" t="inlineStr"/>
+      <c r="BU57" t="inlineStr"/>
+      <c r="BV57" t="inlineStr"/>
+      <c r="BW57" t="inlineStr"/>
+      <c r="BX57" t="inlineStr"/>
+      <c r="BY57" t="inlineStr"/>
+      <c r="BZ57" t="inlineStr"/>
+      <c r="CA57" t="inlineStr"/>
+      <c r="CB57" t="inlineStr"/>
+      <c r="CC57" t="inlineStr"/>
+      <c r="CD57" t="inlineStr"/>
+      <c r="CE57" t="inlineStr"/>
+      <c r="CF57" t="inlineStr"/>
+      <c r="CG57" t="inlineStr"/>
+      <c r="CH57" t="inlineStr"/>
+      <c r="CI57" t="inlineStr"/>
+      <c r="CJ57" t="inlineStr"/>
+      <c r="CK57" t="inlineStr"/>
+      <c r="CL57" t="inlineStr"/>
+      <c r="CM57" t="inlineStr"/>
+      <c r="CN57" t="inlineStr"/>
+      <c r="CO57" t="inlineStr"/>
+      <c r="CP57" t="inlineStr"/>
+      <c r="CQ57" t="inlineStr"/>
+      <c r="CR57" t="inlineStr"/>
+      <c r="CS57" t="inlineStr"/>
+      <c r="CT57" t="inlineStr"/>
+      <c r="CU57" t="inlineStr"/>
+      <c r="CV57" t="inlineStr"/>
+      <c r="CW57" t="inlineStr"/>
+      <c r="CX57" t="inlineStr"/>
+      <c r="CY57" t="inlineStr"/>
+      <c r="CZ57" t="inlineStr"/>
+      <c r="DA57" t="inlineStr"/>
+      <c r="DB57" t="inlineStr"/>
+      <c r="DC57" t="inlineStr"/>
+      <c r="DD57" t="inlineStr"/>
+      <c r="DE57" t="inlineStr"/>
+      <c r="DF57" t="inlineStr"/>
+      <c r="DG57" t="inlineStr"/>
+      <c r="DH57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -13359,6 +16409,56 @@
       <c r="BJ58" t="n">
         <v>9.712984233463661e-06</v>
       </c>
+      <c r="BK58" t="inlineStr"/>
+      <c r="BL58" t="inlineStr"/>
+      <c r="BM58" t="inlineStr"/>
+      <c r="BN58" t="inlineStr"/>
+      <c r="BO58" t="inlineStr"/>
+      <c r="BP58" t="inlineStr"/>
+      <c r="BQ58" t="inlineStr"/>
+      <c r="BR58" t="inlineStr"/>
+      <c r="BS58" t="inlineStr"/>
+      <c r="BT58" t="inlineStr"/>
+      <c r="BU58" t="inlineStr"/>
+      <c r="BV58" t="inlineStr"/>
+      <c r="BW58" t="inlineStr"/>
+      <c r="BX58" t="inlineStr"/>
+      <c r="BY58" t="inlineStr"/>
+      <c r="BZ58" t="inlineStr"/>
+      <c r="CA58" t="inlineStr"/>
+      <c r="CB58" t="inlineStr"/>
+      <c r="CC58" t="inlineStr"/>
+      <c r="CD58" t="inlineStr"/>
+      <c r="CE58" t="inlineStr"/>
+      <c r="CF58" t="inlineStr"/>
+      <c r="CG58" t="inlineStr"/>
+      <c r="CH58" t="inlineStr"/>
+      <c r="CI58" t="inlineStr"/>
+      <c r="CJ58" t="inlineStr"/>
+      <c r="CK58" t="inlineStr"/>
+      <c r="CL58" t="inlineStr"/>
+      <c r="CM58" t="inlineStr"/>
+      <c r="CN58" t="inlineStr"/>
+      <c r="CO58" t="inlineStr"/>
+      <c r="CP58" t="inlineStr"/>
+      <c r="CQ58" t="inlineStr"/>
+      <c r="CR58" t="inlineStr"/>
+      <c r="CS58" t="inlineStr"/>
+      <c r="CT58" t="inlineStr"/>
+      <c r="CU58" t="inlineStr"/>
+      <c r="CV58" t="inlineStr"/>
+      <c r="CW58" t="inlineStr"/>
+      <c r="CX58" t="inlineStr"/>
+      <c r="CY58" t="inlineStr"/>
+      <c r="CZ58" t="inlineStr"/>
+      <c r="DA58" t="inlineStr"/>
+      <c r="DB58" t="inlineStr"/>
+      <c r="DC58" t="inlineStr"/>
+      <c r="DD58" t="inlineStr"/>
+      <c r="DE58" t="inlineStr"/>
+      <c r="DF58" t="inlineStr"/>
+      <c r="DG58" t="inlineStr"/>
+      <c r="DH58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -13578,6 +16678,446 @@
       </c>
       <c r="BJ59" t="n">
         <v>0</v>
+      </c>
+      <c r="BK59" t="inlineStr"/>
+      <c r="BL59" t="inlineStr"/>
+      <c r="BM59" t="inlineStr"/>
+      <c r="BN59" t="inlineStr"/>
+      <c r="BO59" t="inlineStr"/>
+      <c r="BP59" t="inlineStr"/>
+      <c r="BQ59" t="inlineStr"/>
+      <c r="BR59" t="inlineStr"/>
+      <c r="BS59" t="inlineStr"/>
+      <c r="BT59" t="inlineStr"/>
+      <c r="BU59" t="inlineStr"/>
+      <c r="BV59" t="inlineStr"/>
+      <c r="BW59" t="inlineStr"/>
+      <c r="BX59" t="inlineStr"/>
+      <c r="BY59" t="inlineStr"/>
+      <c r="BZ59" t="inlineStr"/>
+      <c r="CA59" t="inlineStr"/>
+      <c r="CB59" t="inlineStr"/>
+      <c r="CC59" t="inlineStr"/>
+      <c r="CD59" t="inlineStr"/>
+      <c r="CE59" t="inlineStr"/>
+      <c r="CF59" t="inlineStr"/>
+      <c r="CG59" t="inlineStr"/>
+      <c r="CH59" t="inlineStr"/>
+      <c r="CI59" t="inlineStr"/>
+      <c r="CJ59" t="inlineStr"/>
+      <c r="CK59" t="inlineStr"/>
+      <c r="CL59" t="inlineStr"/>
+      <c r="CM59" t="inlineStr"/>
+      <c r="CN59" t="inlineStr"/>
+      <c r="CO59" t="inlineStr"/>
+      <c r="CP59" t="inlineStr"/>
+      <c r="CQ59" t="inlineStr"/>
+      <c r="CR59" t="inlineStr"/>
+      <c r="CS59" t="inlineStr"/>
+      <c r="CT59" t="inlineStr"/>
+      <c r="CU59" t="inlineStr"/>
+      <c r="CV59" t="inlineStr"/>
+      <c r="CW59" t="inlineStr"/>
+      <c r="CX59" t="inlineStr"/>
+      <c r="CY59" t="inlineStr"/>
+      <c r="CZ59" t="inlineStr"/>
+      <c r="DA59" t="inlineStr"/>
+      <c r="DB59" t="inlineStr"/>
+      <c r="DC59" t="inlineStr"/>
+      <c r="DD59" t="inlineStr"/>
+      <c r="DE59" t="inlineStr"/>
+      <c r="DF59" t="inlineStr"/>
+      <c r="DG59" t="inlineStr"/>
+      <c r="DH59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Logit_splashing</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>{'estimator': StatsModelsEstimator(model_class=&lt;class 'statsmodels.discrete.discrete_model.Logit'&gt;), 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Re', 'sedimentation_Stk'), 'log_features': ('relative_roughness',), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sign_sedimentation_Re', 'sign_sedimentation_Stk', 'particle_liquid_density_ratio', 'sign_particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False}</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>0.7866666666666666</v>
+      </c>
+      <c r="F60" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="G60" t="n">
+        <v>0.8541666666666666</v>
+      </c>
+      <c r="H60" t="n">
+        <v>0.836734693877551</v>
+      </c>
+      <c r="I60" t="n">
+        <v>0.8765432098765433</v>
+      </c>
+      <c r="J60" t="n">
+        <v>0.7710437710437711</v>
+      </c>
+      <c r="K60" t="n">
+        <v>0.8604651162790697</v>
+      </c>
+      <c r="L60" t="n">
+        <v>0.7708333333333334</v>
+      </c>
+      <c r="M60" t="n">
+        <v>0.8131868131868132</v>
+      </c>
+      <c r="N60" t="n">
+        <v>0.9022569444444445</v>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>0.0, 0.00415349006652832, 0.00912928581237793, 0.004217624664306641, 0.005815267562866211, 0.007185220718383789, 0.004125356674194336</t>
+        </is>
+      </c>
+      <c r="P60" t="n">
+        <v>0.004946606499808175</v>
+      </c>
+      <c r="Q60" t="n">
+        <v>0.004217624664306641</v>
+      </c>
+      <c r="R60" t="n">
+        <v>0.002660950078103845</v>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>0.026595115661621094, 0.012632131576538086, 0.009029865264892578, 0.013502836227416992, 0.009662866592407227, 0.009221792221069336, 0.012566566467285156</t>
+        </is>
+      </c>
+      <c r="T60" t="n">
+        <v>0.01331588200160435</v>
+      </c>
+      <c r="U60" t="n">
+        <v>0.01256656646728516</v>
+      </c>
+      <c r="V60" t="n">
+        <v>0.005680518324840078</v>
+      </c>
+      <c r="W60" t="inlineStr">
+        <is>
+          <t>0.8888888888888888, 0.6981132075471698, 0.8301886792452831, 0.7547169811320755, 0.7924528301886793, 0.7735849056603774, 0.7358490566037735</t>
+        </is>
+      </c>
+      <c r="X60" t="n">
+        <v>0.7819706498951782</v>
+      </c>
+      <c r="Y60" t="n">
+        <v>0.7735849056603774</v>
+      </c>
+      <c r="Z60" t="n">
+        <v>0.05835693062027481</v>
+      </c>
+      <c r="AA60" t="inlineStr">
+        <is>
+          <t>0.9166666666666667, 0.75, 0.8656716417910447, 0.7936507936507937, 0.819672131147541, 0.8125, 0.7999999999999999</t>
+        </is>
+      </c>
+      <c r="AB60" t="n">
+        <v>0.8225944618937209</v>
+      </c>
+      <c r="AC60" t="n">
+        <v>0.8125</v>
+      </c>
+      <c r="AD60" t="n">
+        <v>0.0499054289258703</v>
+      </c>
+      <c r="AE60" t="inlineStr">
+        <is>
+          <t>0.8918918918918919, 0.8275862068965517, 0.8787878787878788, 0.8620689655172413, 0.9259259259259259, 0.8666666666666667, 0.7777777777777778</t>
+        </is>
+      </c>
+      <c r="AF60" t="n">
+        <v>0.8615293304948477</v>
+      </c>
+      <c r="AG60" t="n">
+        <v>0.8666666666666667</v>
+      </c>
+      <c r="AH60" t="n">
+        <v>0.04401266989323341</v>
+      </c>
+      <c r="AI60" t="inlineStr">
+        <is>
+          <t>0.9428571428571428, 0.6857142857142857, 0.8529411764705882, 0.7352941176470589, 0.7352941176470589, 0.7647058823529411, 0.8235294117647058</t>
+        </is>
+      </c>
+      <c r="AJ60" t="n">
+        <v>0.7914765906362545</v>
+      </c>
+      <c r="AK60" t="n">
+        <v>0.7647058823529411</v>
+      </c>
+      <c r="AL60" t="n">
+        <v>0.08100848875408138</v>
+      </c>
+      <c r="AM60" t="inlineStr">
+        <is>
+          <t>0.9533834586466166, 0.8190476190476191, 0.9040247678018576, 0.8993808049535603, 0.9179566563467492, 0.8080495356037152, 0.8622291021671827</t>
+        </is>
+      </c>
+      <c r="AN60" t="n">
+        <v>0.8805817063667573</v>
+      </c>
+      <c r="AO60" t="n">
+        <v>0.8993808049535603</v>
+      </c>
+      <c r="AP60" t="n">
+        <v>0.04925754914855442</v>
+      </c>
+      <c r="AQ60" t="inlineStr">
+        <is>
+          <t>0.7704402515723271, 0.7931034482758621, 0.7962382445141066, 0.7931034482758621, 0.7931034482758621, 0.7931034482758621, 0.8119122257053292</t>
+        </is>
+      </c>
+      <c r="AR60" t="n">
+        <v>0.7930006449850302</v>
+      </c>
+      <c r="AS60" t="n">
+        <v>0.7931034482758621</v>
+      </c>
+      <c r="AT60" t="n">
+        <v>0.01119402621971342</v>
+      </c>
+      <c r="AU60" t="inlineStr">
+        <is>
+          <t>0.8142493638676844, 0.8333333333333334, 0.8354430379746836, 0.8333333333333333, 0.83248730964467, 0.8341708542713568, 0.8492462311557789</t>
+        </is>
+      </c>
+      <c r="AV60" t="n">
+        <v>0.833180494797263</v>
+      </c>
+      <c r="AW60" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="AX60" t="n">
+        <v>0.009434910412352306</v>
+      </c>
+      <c r="AY60" t="inlineStr">
+        <is>
+          <t>0.851063829787234, 0.8638743455497382, 0.873015873015873, 0.868421052631579, 0.8723404255319149, 0.8645833333333334, 0.8802083333333334</t>
+        </is>
+      </c>
+      <c r="AZ60" t="n">
+        <v>0.8676438847404293</v>
+      </c>
+      <c r="BA60" t="n">
+        <v>0.868421052631579</v>
+      </c>
+      <c r="BB60" t="n">
+        <v>0.008517710412420229</v>
+      </c>
+      <c r="BC60" t="inlineStr">
+        <is>
+          <t>0.7804878048780488, 0.8048780487804879, 0.8009708737864077, 0.8009708737864077, 0.7961165048543689, 0.8058252427184466, 0.8203883495145631</t>
+        </is>
+      </c>
+      <c r="BD60" t="n">
+        <v>0.801376814045533</v>
+      </c>
+      <c r="BE60" t="n">
+        <v>0.8009708737864077</v>
+      </c>
+      <c r="BF60" t="n">
+        <v>0.01107014501770598</v>
+      </c>
+      <c r="BG60" t="inlineStr">
+        <is>
+          <t>0.8888625080941075, 0.9075738125802311, 0.8931824039865969, 0.8986381991580032, 0.8930535269353038, 0.9099149411461466, 0.9015594123206461</t>
+        </is>
+      </c>
+      <c r="BH60" t="n">
+        <v>0.8989692577458621</v>
+      </c>
+      <c r="BI60" t="n">
+        <v>0.8986381991580032</v>
+      </c>
+      <c r="BJ60" t="n">
+        <v>0.007283001593575346</v>
+      </c>
+      <c r="BK60" t="n">
+        <v>0.7645211930926217</v>
+      </c>
+      <c r="BL60" t="n">
+        <v>0.7604166666666666</v>
+      </c>
+      <c r="BM60" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="BN60" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="BO60" t="n">
+        <v>0.6923076923076923</v>
+      </c>
+      <c r="BP60" t="n">
+        <v>0.7587673196368849</v>
+      </c>
+      <c r="BQ60" t="n">
+        <v>0.7711309523809524</v>
+      </c>
+      <c r="BR60" t="n">
+        <v>0.648</v>
+      </c>
+      <c r="BS60" t="n">
+        <v>0.7714285714285715</v>
+      </c>
+      <c r="BT60" t="n">
+        <v>0.7043478260869566</v>
+      </c>
+      <c r="BU60" t="inlineStr">
+        <is>
+          <t>0.8661654135338346, 0.7039682539682539, 0.8212074303405572, 0.7623839009287926, 0.8150154798761611, 0.7770897832817337, 0.7012383900928792</t>
+        </is>
+      </c>
+      <c r="BV60" t="n">
+        <v>0.7781526645746017</v>
+      </c>
+      <c r="BW60" t="n">
+        <v>0.7770897832817337</v>
+      </c>
+      <c r="BX60" t="n">
+        <v>0.05685538045414647</v>
+      </c>
+      <c r="BY60" t="inlineStr">
+        <is>
+          <t>0.8333333333333333, 0.619047619047619, 0.7692307692307692, 0.6976744186046512, 0.7555555555555555, 0.7142857142857143, 0.6111111111111113</t>
+        </is>
+      </c>
+      <c r="BZ60" t="n">
+        <v>0.7143197887383934</v>
+      </c>
+      <c r="CA60" t="n">
+        <v>0.7142857142857143</v>
+      </c>
+      <c r="CB60" t="n">
+        <v>0.07453255760672911</v>
+      </c>
+      <c r="CC60" t="inlineStr">
+        <is>
+          <t>0.875, 0.6845238095238095, 0.8174512055109069, 0.7456626061277225, 0.7876138433515483, 0.7633928571428572, 0.7055555555555556</t>
+        </is>
+      </c>
+      <c r="CD60" t="n">
+        <v>0.7684571253160571</v>
+      </c>
+      <c r="CE60" t="n">
+        <v>0.7633928571428572</v>
+      </c>
+      <c r="CF60" t="n">
+        <v>0.06055154802943036</v>
+      </c>
+      <c r="CG60" t="inlineStr">
+        <is>
+          <t>0.8823529411764706, 0.5416666666666666, 0.75, 0.625, 0.6538461538461539, 0.6521739130434783, 0.6470588235294118</t>
+        </is>
+      </c>
+      <c r="CH60" t="n">
+        <v>0.6788712140374544</v>
+      </c>
+      <c r="CI60" t="n">
+        <v>0.6521739130434783</v>
+      </c>
+      <c r="CJ60" t="n">
+        <v>0.1003866387672127</v>
+      </c>
+      <c r="CK60" t="inlineStr">
+        <is>
+          <t>0.7894736842105263, 0.7222222222222222, 0.7894736842105263, 0.7894736842105263, 0.8947368421052632, 0.7894736842105263, 0.5789473684210527</t>
+        </is>
+      </c>
+      <c r="CL60" t="n">
+        <v>0.764828738512949</v>
+      </c>
+      <c r="CM60" t="n">
+        <v>0.7894736842105263</v>
+      </c>
+      <c r="CN60" t="n">
+        <v>0.08918104198792963</v>
+      </c>
+      <c r="CO60" t="inlineStr">
+        <is>
+          <t>0.7663500971292898, 0.7884039366709457, 0.7942907466277171, 0.7898659678666552, 0.7918635621616977, 0.7878683735716127, 0.8084242632528568</t>
+        </is>
+      </c>
+      <c r="CP60" t="n">
+        <v>0.7895809924686821</v>
+      </c>
+      <c r="CQ60" t="n">
+        <v>0.7898659678666552</v>
+      </c>
+      <c r="CR60" t="n">
+        <v>0.0115048747157305</v>
+      </c>
+      <c r="CS60" t="inlineStr">
+        <is>
+          <t>0.6995884773662552, 0.7272727272727273, 0.7325102880658437, 0.7272727272727273, 0.7295081967213114, 0.725, 0.7499999999999999</t>
+        </is>
+      </c>
+      <c r="CT60" t="n">
+        <v>0.7273074880998377</v>
+      </c>
+      <c r="CU60" t="n">
+        <v>0.7272727272727273</v>
+      </c>
+      <c r="CV60" t="n">
+        <v>0.01373490244529015</v>
+      </c>
+      <c r="CW60" t="inlineStr">
+        <is>
+          <t>0.7569189206169697, 0.7803030303030303, 0.7839766630202636, 0.7803030303030303, 0.7809977531829907, 0.7795854271356784, 0.7996231155778895</t>
+        </is>
+      </c>
+      <c r="CX60" t="n">
+        <v>0.7802439914485504</v>
+      </c>
+      <c r="CY60" t="n">
+        <v>0.7803030303030303</v>
+      </c>
+      <c r="CZ60" t="n">
+        <v>0.01155453561692818</v>
+      </c>
+      <c r="DA60" t="inlineStr">
+        <is>
+          <t>0.6538461538461539, 0.6875, 0.6846153846153846, 0.6821705426356589, 0.6793893129770993, 0.6850393700787402, 0.7086614173228346</t>
+        </is>
+      </c>
+      <c r="DB60" t="n">
+        <v>0.6830317402108387</v>
+      </c>
+      <c r="DC60" t="n">
+        <v>0.6846153846153846</v>
+      </c>
+      <c r="DD60" t="n">
+        <v>0.01487659518727417</v>
+      </c>
+      <c r="DE60" t="inlineStr">
+        <is>
+          <t>0.7522123893805309, 0.7719298245614035, 0.7876106194690266, 0.7787610619469026, 0.7876106194690266, 0.7699115044247787, 0.7964601769911505</t>
+        </is>
+      </c>
+      <c r="DF60" t="n">
+        <v>0.7777851708918313</v>
+      </c>
+      <c r="DG60" t="n">
+        <v>0.7787610619469026</v>
+      </c>
+      <c r="DH60" t="n">
+        <v>0.01359114183238239</v>
       </c>
     </row>
   </sheetData>

</xml_diff>